<commit_message>
Daily jobs update - 2026-02-16 00:00:03
</commit_message>
<xml_diff>
--- a/2026-02-14/DE_jobs_2026-02-14.xlsx
+++ b/2026-02-14/DE_jobs_2026-02-14.xlsx
@@ -433,7 +433,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I35"/>
+  <dimension ref="A1:I47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2587,20 +2587,14 @@
           <t>indeed</t>
         </is>
       </c>
-      <c r="E29">
-        <f>HYPERLINK("https://www.indeed.com/viewjob?jk=a08d96a788848f73", "https://www.indeed.com/viewjob?jk=a08d96a788848f73")</f>
-        <v/>
-      </c>
-      <c r="F29">
-        <f>HYPERLINK("https://careers.intrado.com/jobs/4457/job?utm_source=indeed_integration&amp;iis=Job%20Board&amp;iisn=Indeed&amp;indeed-apply-token=73a2d2b2a8d6d5c0a62696875eaebd669103652d3f0c2cd5445d3e66b1592b0f", "https://careers.intrado.com/jobs/4457/job?utm_source=indeed_integration&amp;iis=Job%20Board&amp;iisn=Indeed&amp;indeed-apply-token=73a2d2b2a8d6d5c0a62696875eaebd669103652d3f0c2cd5445d3e66b1592b0f")</f>
-        <v/>
-      </c>
+      <c r="E29" t="inlineStr"/>
+      <c r="F29" t="inlineStr"/>
       <c r="G29" t="inlineStr">
         <is>
           <t>Remote, US</t>
         </is>
       </c>
-      <c r="H29" s="3" t="n">
+      <c r="H29" s="2" t="n">
         <v>46066</v>
       </c>
       <c r="I29" t="inlineStr">
@@ -2653,20 +2647,14 @@
           <t>indeed</t>
         </is>
       </c>
-      <c r="E30">
-        <f>HYPERLINK("https://www.indeed.com/viewjob?jk=0e21339192c561d7", "https://www.indeed.com/viewjob?jk=0e21339192c561d7")</f>
-        <v/>
-      </c>
-      <c r="F30">
-        <f>HYPERLINK("https://careers.intrado.com/jobs/4455/job?utm_source=indeed_integration&amp;iis=Job%20Board&amp;iisn=Indeed&amp;indeed-apply-token=73a2d2b2a8d6d5c0a62696875eaebd669103652d3f0c2cd5445d3e66b1592b0f", "https://careers.intrado.com/jobs/4455/job?utm_source=indeed_integration&amp;iis=Job%20Board&amp;iisn=Indeed&amp;indeed-apply-token=73a2d2b2a8d6d5c0a62696875eaebd669103652d3f0c2cd5445d3e66b1592b0f")</f>
-        <v/>
-      </c>
+      <c r="E30" t="inlineStr"/>
+      <c r="F30" t="inlineStr"/>
       <c r="G30" t="inlineStr">
         <is>
           <t>Remote, US</t>
         </is>
       </c>
-      <c r="H30" s="3" t="n">
+      <c r="H30" s="2" t="n">
         <v>46066</v>
       </c>
       <c r="I30" t="inlineStr">
@@ -2718,20 +2706,14 @@
           <t>indeed</t>
         </is>
       </c>
-      <c r="E31">
-        <f>HYPERLINK("https://www.indeed.com/viewjob?jk=6b2a5a8c0bc2f157", "https://www.indeed.com/viewjob?jk=6b2a5a8c0bc2f157")</f>
-        <v/>
-      </c>
-      <c r="F31">
-        <f>HYPERLINK("https://careers.intrado.com/jobs/4454/job?utm_source=indeed_integration&amp;iis=Job%20Board&amp;iisn=Indeed&amp;indeed-apply-token=73a2d2b2a8d6d5c0a62696875eaebd669103652d3f0c2cd5445d3e66b1592b0f", "https://careers.intrado.com/jobs/4454/job?utm_source=indeed_integration&amp;iis=Job%20Board&amp;iisn=Indeed&amp;indeed-apply-token=73a2d2b2a8d6d5c0a62696875eaebd669103652d3f0c2cd5445d3e66b1592b0f")</f>
-        <v/>
-      </c>
+      <c r="E31" t="inlineStr"/>
+      <c r="F31" t="inlineStr"/>
       <c r="G31" t="inlineStr">
         <is>
           <t>Remote, US</t>
         </is>
       </c>
-      <c r="H31" s="3" t="n">
+      <c r="H31" s="2" t="n">
         <v>46066</v>
       </c>
       <c r="I31" t="inlineStr">
@@ -2779,20 +2761,14 @@
           <t>indeed</t>
         </is>
       </c>
-      <c r="E32">
-        <f>HYPERLINK("https://www.indeed.com/viewjob?jk=f5499876b043b01c", "https://www.indeed.com/viewjob?jk=f5499876b043b01c")</f>
-        <v/>
-      </c>
-      <c r="F32">
-        <f>HYPERLINK("https://candidateportalnew.ceipal.com/job-details/HAa_aMCBVWcxo8_M6exZhc-cIHXe9nw0u_vNPCOwH2Q#.job_boards.Indeed", "https://candidateportalnew.ceipal.com/job-details/HAa_aMCBVWcxo8_M6exZhc-cIHXe9nw0u_vNPCOwH2Q#.job_boards.Indeed")</f>
-        <v/>
-      </c>
+      <c r="E32" t="inlineStr"/>
+      <c r="F32" t="inlineStr"/>
       <c r="G32" t="inlineStr">
         <is>
           <t>MD, US</t>
         </is>
       </c>
-      <c r="H32" s="3" t="n">
+      <c r="H32" s="2" t="n">
         <v>46066</v>
       </c>
       <c r="I32" t="inlineStr">
@@ -2888,20 +2864,14 @@
           <t>indeed</t>
         </is>
       </c>
-      <c r="E33">
-        <f>HYPERLINK("https://www.indeed.com/viewjob?jk=f13cdaf5afff4db9", "https://www.indeed.com/viewjob?jk=f13cdaf5afff4db9")</f>
-        <v/>
-      </c>
-      <c r="F33">
-        <f>HYPERLINK("https://candidateportalnew.ceipal.com/job-details/S80ObZE5ViGmb0j6cXe5NROl7BdqR8HmR6E8Gxj4ovU#.job_boards.Indeed", "https://candidateportalnew.ceipal.com/job-details/S80ObZE5ViGmb0j6cXe5NROl7BdqR8HmR6E8Gxj4ovU#.job_boards.Indeed")</f>
-        <v/>
-      </c>
+      <c r="E33" t="inlineStr"/>
+      <c r="F33" t="inlineStr"/>
       <c r="G33" t="inlineStr">
         <is>
           <t>GA, US</t>
         </is>
       </c>
-      <c r="H33" s="3" t="n">
+      <c r="H33" s="2" t="n">
         <v>46066</v>
       </c>
       <c r="I33" t="inlineStr">
@@ -2941,20 +2911,14 @@
           <t>indeed</t>
         </is>
       </c>
-      <c r="E34">
-        <f>HYPERLINK("https://www.indeed.com/viewjob?jk=95db0cf13cfff2e0", "https://www.indeed.com/viewjob?jk=95db0cf13cfff2e0")</f>
-        <v/>
-      </c>
-      <c r="F34">
-        <f>HYPERLINK("https://candidateportalnew.ceipal.com/job-details/B5yax7geznzByp65mojvbkBQDsyq7tiglSPkbKP6JTE#.job_boards.Indeed", "https://candidateportalnew.ceipal.com/job-details/B5yax7geznzByp65mojvbkBQDsyq7tiglSPkbKP6JTE#.job_boards.Indeed")</f>
-        <v/>
-      </c>
+      <c r="E34" t="inlineStr"/>
+      <c r="F34" t="inlineStr"/>
       <c r="G34" t="inlineStr">
         <is>
           <t>GA, US</t>
         </is>
       </c>
-      <c r="H34" s="3" t="n">
+      <c r="H34" s="2" t="n">
         <v>46066</v>
       </c>
       <c r="I34" t="inlineStr">
@@ -2999,20 +2963,14 @@
           <t>indeed</t>
         </is>
       </c>
-      <c r="E35">
-        <f>HYPERLINK("https://www.indeed.com/viewjob?jk=78ff06faf283a092", "https://www.indeed.com/viewjob?jk=78ff06faf283a092")</f>
-        <v/>
-      </c>
-      <c r="F35">
-        <f>HYPERLINK("https://careers.hcahealthcare.com/en/jobs/16846850-staff-data-engineer?tm_job=1-INFOR-3819724&amp;tm_event=view&amp;tm_company=2537", "https://careers.hcahealthcare.com/en/jobs/16846850-staff-data-engineer?tm_job=1-INFOR-3819724&amp;tm_event=view&amp;tm_company=2537")</f>
-        <v/>
-      </c>
+      <c r="E35" t="inlineStr"/>
+      <c r="F35" t="inlineStr"/>
       <c r="G35" t="inlineStr">
         <is>
           <t>Nashville, TN, US</t>
         </is>
       </c>
-      <c r="H35" s="3" t="n">
+      <c r="H35" s="2" t="n">
         <v>46066</v>
       </c>
       <c r="I35" t="inlineStr">
@@ -3119,6 +3077,1068 @@
         </is>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>in-631e8e3565da88d6</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Data Engineer - SSIS / SQL Server, Azure</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>Impact Makers</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>indeed</t>
+        </is>
+      </c>
+      <c r="E36">
+        <f>HYPERLINK("https://www.indeed.com/viewjob?jk=631e8e3565da88d6", "https://www.indeed.com/viewjob?jk=631e8e3565da88d6")</f>
+        <v/>
+      </c>
+      <c r="F36">
+        <f>HYPERLINK("https://theapplicantmanager.com/jobs?pos=ik647&amp;src=Indeed", "https://theapplicantmanager.com/jobs?pos=ik647&amp;src=Indeed")</f>
+        <v/>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>US</t>
+        </is>
+      </c>
+      <c r="H36" s="3" t="n">
+        <v>46066</v>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>**Data Engineer \- SSIS / SQL Server, Azure**  
+**Preferred Location: Pune/Hyderabad, India**
+Impact Makers is a mission\-driven management and technology consulting company that delivers exceptional value to make an impact for our clients and the world. Our experienced teams help organizations manage transformation in IT, data, cloud, and security with a focus on their customers and their people. We utilize our innovative business model to transform the business value of our work into social value for the community. We are committed to gifting 100% of our net profits to the community over the life of the company and our annual community contributions rival companies 100x our size.
+**About the Role**
+We are looking for a Data Engineer to join a larger Impact Makers (IM) delivery team supporting a key client engagement. This role focuses on engineering and maintenance of business\-critical data platforms built on the SQL Server ecosystem. It is well suited for someone who enjoys understanding existing systems, building strong context, and taking thoughtful ownership over how data platforms operate and evolve. You will work as part of a collaborative IM team, partnering closely with the client’s stakeholders.
+**Engagement Details**
+* **Start:** March 1
+* **Employment Type:** Full Time
+* **Preferred location**: Pune/Hyderabad, India
+**What You’ll Do**
+**Discovery \&amp; System Understanding**
+* Take time to understand existing data platforms, including architecture, data flows, and dependencies
+* Build a clear picture of how data is modeled, processed, and consumed across the organization
+* Ask thoughtful technical and business questions to establish shared understanding
+* Translate what you learn into clear plans for stabilization and improvement
+**Data Engineering \&amp; Relational Databases**
+* Design, develop, and maintain **SSIS packages** and SQL Server Agent jobs
+* Write and optimize **SQL** including stored procedures, views, triggers, and functions
+* Work confidently with **relational data models**, understanding how tables, keys, and relationships support reporting and analytics
+* Tune performance using indexes, statistics, execution plans, and query design
+* Support large datasets and frequently used tables with a focus on reliability and scalability
+**Reliability \&amp; Ongoing Support**
+* Help ensure data pipelines run predictably and consistently
+* Investigate and resolve data issues in a structured, calm manner
+* Reduce repeat issues through thoughtful, durable improvements
+* Balance short\-term fixes with longer\-term enhancements
+**Agile Delivery \&amp; Engineering Practices**
+* Work within an **Agile delivery model**, participating in planning and retrospectives
+* Use **Git** for version control and collaborate through structured release processes
+Support smooth promotion of changes across environments (Dev QA UAT* Prod)
+* Take ownership of work from start to finish, with a focus on quality and follow\-through
+**Collaboration \&amp; Communication**
+* Work with client stakeholders in collaboration with IM team.
+* Explain data structures, dependencies, and impacts in clear, accessible language
+* Collaborate with analytics, application, infrastructure, and platform teams
+**What We’re Looking For**
+**Must\-Have**
+* Strong experience with **SQL Server (on\-premise)**
+* Advanced SQL skills, including performance tuning
+* Hands\-on experience with **SSIS**
+* Solid understanding of **relational database concepts and data modeling**
+* Experience supporting production data systems
+* Comfortable learning existing systems and building context before making changes
+* Exposure to **Azure, AWS, or GCP**
+* Strong communication skills
+**Nice to Have**
+* Experience with **SSAS**
+* Working knowledge of **Oracle / PL\-SQL**
+* Shell scripting for automation
+* Experience with **Azure Data Factory (ADF)**
+* Familiarity with **Microsoft Fabric**
+* Experience with **Power BI**
+* Exposure to **Snowflake**
+* Familiarity with open orchestration tools such as **Airflow**
+* Experience with **Azure DevOps, Jira, or similar tools**
+**Growth \&amp; Future Opportunities**
+While the initial focus is understanding and strengthening an existing SQL Server–based platform, there is a clear opportunity to participate in **future modernization efforts**.  
+As the platform stabilizes, you may:
+* Contribute to evolution toward **Microsoft Fabric**
+* Expand orchestration beyond SSIS using **ADF or open orchestration tools**
+* Participate in cloud discussions across **Azure, AWS, or GCP**
+* Work with modern analytics platforms such as **Power BI**
+We value thoughtful evolution built on a strong understanding of what exists today.
+**Why This Role**
+* Part of a **larger IM delivery team**, not staff augmentation
+* Opportunity to stabilize today’s platform and help shape what comes next
+* A balanced mix of ownership, collaboration, and forward\-looking work
+**Experience**
+* 2\-5 years of experience in data engineering on SQL Server/SSIS, Cloud
+* Experience with established data platforms and relational databases preferred
+**Benefits of working at Impact Makers****:**
+As a values\-based company, taking care of our employees is of the utmost importance and our employee benefits package reflects that. We offer healthcare plans with generous contributions to premiums, 401(k) with matching, and generous PTO. Impact Makers embraces the pursuit of balance between work, family, and personal interests, with a flexible, dog\-friendly work environment in Scott’s Addition. We like to have fun at work, collaborating through company sponsored events and pro bono opportunities. Our team members work with Impact Makers, not for Impact Makers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>in-7ebf98b873a11aa5</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Data Engineer</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Liberty Mutual Insurance</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>indeed</t>
+        </is>
+      </c>
+      <c r="E37">
+        <f>HYPERLINK("https://www.indeed.com/viewjob?jk=7ebf98b873a11aa5", "https://www.indeed.com/viewjob?jk=7ebf98b873a11aa5")</f>
+        <v/>
+      </c>
+      <c r="F37">
+        <f>HYPERLINK("https://searchjobs.libertymutualgroup.com/careers/job/618515551654?utm_source=indeed&amp;domain=libertymutual.com", "https://searchjobs.libertymutualgroup.com/careers/job/618515551654?utm_source=indeed&amp;domain=libertymutual.com")</f>
+        <v/>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Plano, TX, US</t>
+        </is>
+      </c>
+      <c r="H37" s="3" t="n">
+        <v>46065</v>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>**Description**We deliver our customers peace of mind every day by helping them protect what they value most. Our passion for placing the customer at the center of everything we do is drive a transformational shift at Liberty Mutual. Operating as a tech startup within a Fortune 100 company, we are leading a digital disruption that will redefine how people experience insurance.
+The US Retail Markets (USRM) Data and Analytics Engineering team is actively searching for a highly productive Data Engineer for a distributed, dynamic agile team to serve as a technical expert designing, developing, analyzing \&amp; testing innovative data warehouse reporting solutions. This candidate will join an energetic and engaged Claims Data Solutions Engineering team focused on delivering exceptional value to our Claims business partners. You will work collaboratively in an agile squad to design and build data pipelines \&amp; workflows, ingest, curate \&amp; provision data workflows in a Cloud\-based environment as well as own responsibility of thorough end\-to\-end testing.
+ This is a fast\-paced environment providing rapid delivery for our business partners. You will be working in a highly collaborative environment that values speed and quality, with a strong desire to drive change and foster a positive work environment. You will have the opportunity to help lead this change as we grow this culture, mindset, and capability.
+**\*\*This is a hybrid role requiring two days in the office a week in one of the following locations: Plano, TX, Boston, MA, Portsmouth, NH, Indianapolis, IN and Columbus, OH\*\***
+ **\*\******You must be authorized to work in the United States without employer sponsorship now or in the future. We will not sponsor employment visas. Candidates who will require future sponsorship, including candidates on CPT/OPT/STEMOPT who will require future sponsorship, are not eligible to apply.*** **\*\***
+We encourage you to apply if this interests you:
+Work as ONE team committed to excellence.
+Model and promote a Data First attitude.
+ Help advance Data Engineering operations into the future.
+Work with a modern data tech stack.
+About the job:
+Work in a dynamic and exciting agile environment with Scrum Masters, Product Owners, and team members.
+Analyze, develop, and execute data integration solutions, to manage the information lifecycle needs of an organization.
+Actively participates in code reviews within each Agile sprint, with focus on test driven development and Continuous Integration and Continuous Development (CICD).
+Designs and builds data provisioning workflows/pipelines, physical data schemas, extracts, data transformations, and data integrations and/or designs using ETL and API microservices.
+Build data architecture and data applications (marts/warehouses) that enable reporting, analytics, data science, and data management and improve accessibility, efficiency, governance, processing, and quality of data.
+Improve speed to market by focusing on current data needs as well as building out the long\-term strategic data solutions using AWS, Snowflake, SQL, Data Vault methodology, as well as other modern data technologies.
+Design and develop programs and tools to support ingestion, curation, and provisioning of complex enterprise data to achieve analytics, reporting, and data science.
+Demonstrate an open\-minded and collaborative approach to creating innovative technical solutions.
+Continuously learn to maintain strong knowledge of technology enablers
+Mentor new and junior developers.
+Provide successful deployment and provisioning of data solutions to production or other required environments.
+Analyze complex technical problems and is expected to recommend process improvements that address complex technology gaps within a single business process and improve data reliability, quality, and efficiency.
+**Qualifications**
+Bachelor\`s degree in technical or business discipline or equivalent experience. Generally, 3\+ years of professional experience.
+Experience integrating Guidewire systems with Snowflake for reporting, analytics, or data warehousing purposes, often using APIs and ETL tools.
+Knowledge of a variety of data platforms including Snowflake, Teradata, SQL, DB2 (Cloud based DB a plus).
+Experience with AWS (such as S3, Snowflake, Athena), Unix, Informatica (IDMC) and strong SQL skillset.
+Strong oral and written communication skills; presentation skills. Proficient in negotiation, facilitation and consensus building skills.
+Knowledge of layered systems architectures and layered solutions and designs, understanding of shared data engineering concepts of agile data engineering concepts and processes
+Must be proactive and demonstrate initiative and be a logical thinker. Consultative skills, including the ability to understand and apply customer requirements, including drawing out unforeseen implications and making recommendations for design, the ability to define design reasoning, understanding potential impacts of design requirements. Collaboration, prioritization, and adaptability skills required.
+Additional Qualifications:
+Snowflake, NoSQL, Python development experience.
+Understanding Cloud / Hybrid data architecture concepts.
+Understanding of insurance industry and products.
+Excited by trying new technology and learning new tools.
+ **About Us****Pay Philosophy:** The typical starting salary range for this role is determined by a number of factors including skills, experience, education, certifications and location. The full salary range for this role reflects the competitive labor market value for all employees in these positions across the national market and provides an opportunity to progress as employees grow and develop within the role. Some roles at Liberty Mutual have a corresponding compensation plan which may include commission and/or bonus earnings at rates that vary based on multiple factors set forth in the compensation plan for the role.
+At Liberty Mutual, our goal is to create a workplace where everyone feels valued, supported, and can thrive. We build an environment that welcomes a wide range of perspectives and experiences, with inclusion embedded in every aspect of our culture and reflected in everyday interactions. This comes to life through comprehensive benefits, workplace flexibility, professional development opportunities, and a host of opportunities provided through our Employee Resource Groups. Each employee plays a role in creating our inclusive culture, which supports every individual to do their best work. Together, we cultivate a community where everyone can make a meaningful impact for our business, our customers, and the communities we serve.
+We value your hard work, integrity and commitment to make things better, and we put people first by offering you benefits that support your life and well\-being. To learn more about our benefit offerings please visit: https://LMI.co/Benefits  
+Liberty Mutual is an equal opportunity employer. We will not tolerate discrimination on the basis of race, color, national origin, sex, sexual orientation, gender identity, religion, age, disability, veteran's status, pregnancy, genetic information or on any basis prohibited by federal, state or local law.  
+**Fair Chance Notices**
+* California
+* Los Angeles Incorporated
+* Los Angeles Unincorporated
+* Philadelphia
+* San Francisco</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>in-d01a65dd80ef9c1e</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Data Engineer</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Liberty Mutual Insurance</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>indeed</t>
+        </is>
+      </c>
+      <c r="E38">
+        <f>HYPERLINK("https://www.indeed.com/viewjob?jk=d01a65dd80ef9c1e", "https://www.indeed.com/viewjob?jk=d01a65dd80ef9c1e")</f>
+        <v/>
+      </c>
+      <c r="F38">
+        <f>HYPERLINK("https://searchjobs.libertymutualgroup.com/careers/job/618515551654?utm_source=indeed&amp;domain=libertymutual.com", "https://searchjobs.libertymutualgroup.com/careers/job/618515551654?utm_source=indeed&amp;domain=libertymutual.com")</f>
+        <v/>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Columbus, OH, US</t>
+        </is>
+      </c>
+      <c r="H38" s="3" t="n">
+        <v>46065</v>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>**Description**We deliver our customers peace of mind every day by helping them protect what they value most. Our passion for placing the customer at the center of everything we do is drive a transformational shift at Liberty Mutual. Operating as a tech startup within a Fortune 100 company, we are leading a digital disruption that will redefine how people experience insurance.
+The US Retail Markets (USRM) Data and Analytics Engineering team is actively searching for a highly productive Data Engineer for a distributed, dynamic agile team to serve as a technical expert designing, developing, analyzing \&amp; testing innovative data warehouse reporting solutions. This candidate will join an energetic and engaged Claims Data Solutions Engineering team focused on delivering exceptional value to our Claims business partners. You will work collaboratively in an agile squad to design and build data pipelines \&amp; workflows, ingest, curate \&amp; provision data workflows in a Cloud\-based environment as well as own responsibility of thorough end\-to\-end testing.
+ This is a fast\-paced environment providing rapid delivery for our business partners. You will be working in a highly collaborative environment that values speed and quality, with a strong desire to drive change and foster a positive work environment. You will have the opportunity to help lead this change as we grow this culture, mindset, and capability.
+**\*\*This is a hybrid role requiring two days in the office a week in one of the following locations: Plano, TX, Boston, MA, Portsmouth, NH, Indianapolis, IN and Columbus, OH\*\***
+ **\*\******You must be authorized to work in the United States without employer sponsorship now or in the future. We will not sponsor employment visas. Candidates who will require future sponsorship, including candidates on CPT/OPT/STEMOPT who will require future sponsorship, are not eligible to apply.*** **\*\***
+We encourage you to apply if this interests you:
+Work as ONE team committed to excellence.
+Model and promote a Data First attitude.
+ Help advance Data Engineering operations into the future.
+Work with a modern data tech stack.
+About the job:
+Work in a dynamic and exciting agile environment with Scrum Masters, Product Owners, and team members.
+Analyze, develop, and execute data integration solutions, to manage the information lifecycle needs of an organization.
+Actively participates in code reviews within each Agile sprint, with focus on test driven development and Continuous Integration and Continuous Development (CICD).
+Designs and builds data provisioning workflows/pipelines, physical data schemas, extracts, data transformations, and data integrations and/or designs using ETL and API microservices.
+Build data architecture and data applications (marts/warehouses) that enable reporting, analytics, data science, and data management and improve accessibility, efficiency, governance, processing, and quality of data.
+Improve speed to market by focusing on current data needs as well as building out the long\-term strategic data solutions using AWS, Snowflake, SQL, Data Vault methodology, as well as other modern data technologies.
+Design and develop programs and tools to support ingestion, curation, and provisioning of complex enterprise data to achieve analytics, reporting, and data science.
+Demonstrate an open\-minded and collaborative approach to creating innovative technical solutions.
+Continuously learn to maintain strong knowledge of technology enablers
+Mentor new and junior developers.
+Provide successful deployment and provisioning of data solutions to production or other required environments.
+Analyze complex technical problems and is expected to recommend process improvements that address complex technology gaps within a single business process and improve data reliability, quality, and efficiency.
+**Qualifications**
+Bachelor\`s degree in technical or business discipline or equivalent experience. Generally, 3\+ years of professional experience.
+Experience integrating Guidewire systems with Snowflake for reporting, analytics, or data warehousing purposes, often using APIs and ETL tools.
+Knowledge of a variety of data platforms including Snowflake, Teradata, SQL, DB2 (Cloud based DB a plus).
+Experience with AWS (such as S3, Snowflake, Athena), Unix, Informatica (IDMC) and strong SQL skillset.
+Strong oral and written communication skills; presentation skills. Proficient in negotiation, facilitation and consensus building skills.
+Knowledge of layered systems architectures and layered solutions and designs, understanding of shared data engineering concepts of agile data engineering concepts and processes
+Must be proactive and demonstrate initiative and be a logical thinker. Consultative skills, including the ability to understand and apply customer requirements, including drawing out unforeseen implications and making recommendations for design, the ability to define design reasoning, understanding potential impacts of design requirements. Collaboration, prioritization, and adaptability skills required.
+Additional Qualifications:
+Snowflake, NoSQL, Python development experience.
+Understanding Cloud / Hybrid data architecture concepts.
+Understanding of insurance industry and products.
+Excited by trying new technology and learning new tools.
+ **About Us****Pay Philosophy:** The typical starting salary range for this role is determined by a number of factors including skills, experience, education, certifications and location. The full salary range for this role reflects the competitive labor market value for all employees in these positions across the national market and provides an opportunity to progress as employees grow and develop within the role. Some roles at Liberty Mutual have a corresponding compensation plan which may include commission and/or bonus earnings at rates that vary based on multiple factors set forth in the compensation plan for the role.
+At Liberty Mutual, our goal is to create a workplace where everyone feels valued, supported, and can thrive. We build an environment that welcomes a wide range of perspectives and experiences, with inclusion embedded in every aspect of our culture and reflected in everyday interactions. This comes to life through comprehensive benefits, workplace flexibility, professional development opportunities, and a host of opportunities provided through our Employee Resource Groups. Each employee plays a role in creating our inclusive culture, which supports every individual to do their best work. Together, we cultivate a community where everyone can make a meaningful impact for our business, our customers, and the communities we serve.
+We value your hard work, integrity and commitment to make things better, and we put people first by offering you benefits that support your life and well\-being. To learn more about our benefit offerings please visit: https://LMI.co/Benefits  
+Liberty Mutual is an equal opportunity employer. We will not tolerate discrimination on the basis of race, color, national origin, sex, sexual orientation, gender identity, religion, age, disability, veteran's status, pregnancy, genetic information or on any basis prohibited by federal, state or local law.  
+**Fair Chance Notices**
+* California
+* Los Angeles Incorporated
+* Los Angeles Unincorporated
+* Philadelphia
+* San Francisco</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>in-981059363e287ee1</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Data Engineer</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Liberty Mutual Insurance</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>indeed</t>
+        </is>
+      </c>
+      <c r="E39">
+        <f>HYPERLINK("https://www.indeed.com/viewjob?jk=981059363e287ee1", "https://www.indeed.com/viewjob?jk=981059363e287ee1")</f>
+        <v/>
+      </c>
+      <c r="F39">
+        <f>HYPERLINK("https://searchjobs.libertymutualgroup.com/careers/job/618515551654?utm_source=indeed&amp;domain=libertymutual.com", "https://searchjobs.libertymutualgroup.com/careers/job/618515551654?utm_source=indeed&amp;domain=libertymutual.com")</f>
+        <v/>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Indianapolis, IN, US</t>
+        </is>
+      </c>
+      <c r="H39" s="3" t="n">
+        <v>46065</v>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>**Description**We deliver our customers peace of mind every day by helping them protect what they value most. Our passion for placing the customer at the center of everything we do is drive a transformational shift at Liberty Mutual. Operating as a tech startup within a Fortune 100 company, we are leading a digital disruption that will redefine how people experience insurance.
+The US Retail Markets (USRM) Data and Analytics Engineering team is actively searching for a highly productive Data Engineer for a distributed, dynamic agile team to serve as a technical expert designing, developing, analyzing \&amp; testing innovative data warehouse reporting solutions. This candidate will join an energetic and engaged Claims Data Solutions Engineering team focused on delivering exceptional value to our Claims business partners. You will work collaboratively in an agile squad to design and build data pipelines \&amp; workflows, ingest, curate \&amp; provision data workflows in a Cloud\-based environment as well as own responsibility of thorough end\-to\-end testing.
+ This is a fast\-paced environment providing rapid delivery for our business partners. You will be working in a highly collaborative environment that values speed and quality, with a strong desire to drive change and foster a positive work environment. You will have the opportunity to help lead this change as we grow this culture, mindset, and capability.
+**\*\*This is a hybrid role requiring two days in the office a week in one of the following locations: Plano, TX, Boston, MA, Portsmouth, NH, Indianapolis, IN and Columbus, OH\*\***
+ **\*\******You must be authorized to work in the United States without employer sponsorship now or in the future. We will not sponsor employment visas. Candidates who will require future sponsorship, including candidates on CPT/OPT/STEMOPT who will require future sponsorship, are not eligible to apply.*** **\*\***
+We encourage you to apply if this interests you:
+Work as ONE team committed to excellence.
+Model and promote a Data First attitude.
+ Help advance Data Engineering operations into the future.
+Work with a modern data tech stack.
+About the job:
+Work in a dynamic and exciting agile environment with Scrum Masters, Product Owners, and team members.
+Analyze, develop, and execute data integration solutions, to manage the information lifecycle needs of an organization.
+Actively participates in code reviews within each Agile sprint, with focus on test driven development and Continuous Integration and Continuous Development (CICD).
+Designs and builds data provisioning workflows/pipelines, physical data schemas, extracts, data transformations, and data integrations and/or designs using ETL and API microservices.
+Build data architecture and data applications (marts/warehouses) that enable reporting, analytics, data science, and data management and improve accessibility, efficiency, governance, processing, and quality of data.
+Improve speed to market by focusing on current data needs as well as building out the long\-term strategic data solutions using AWS, Snowflake, SQL, Data Vault methodology, as well as other modern data technologies.
+Design and develop programs and tools to support ingestion, curation, and provisioning of complex enterprise data to achieve analytics, reporting, and data science.
+Demonstrate an open\-minded and collaborative approach to creating innovative technical solutions.
+Continuously learn to maintain strong knowledge of technology enablers
+Mentor new and junior developers.
+Provide successful deployment and provisioning of data solutions to production or other required environments.
+Analyze complex technical problems and is expected to recommend process improvements that address complex technology gaps within a single business process and improve data reliability, quality, and efficiency.
+**Qualifications**
+Bachelor\`s degree in technical or business discipline or equivalent experience. Generally, 3\+ years of professional experience.
+Experience integrating Guidewire systems with Snowflake for reporting, analytics, or data warehousing purposes, often using APIs and ETL tools.
+Knowledge of a variety of data platforms including Snowflake, Teradata, SQL, DB2 (Cloud based DB a plus).
+Experience with AWS (such as S3, Snowflake, Athena), Unix, Informatica (IDMC) and strong SQL skillset.
+Strong oral and written communication skills; presentation skills. Proficient in negotiation, facilitation and consensus building skills.
+Knowledge of layered systems architectures and layered solutions and designs, understanding of shared data engineering concepts of agile data engineering concepts and processes
+Must be proactive and demonstrate initiative and be a logical thinker. Consultative skills, including the ability to understand and apply customer requirements, including drawing out unforeseen implications and making recommendations for design, the ability to define design reasoning, understanding potential impacts of design requirements. Collaboration, prioritization, and adaptability skills required.
+Additional Qualifications:
+Snowflake, NoSQL, Python development experience.
+Understanding Cloud / Hybrid data architecture concepts.
+Understanding of insurance industry and products.
+Excited by trying new technology and learning new tools.
+ **About Us****Pay Philosophy:** The typical starting salary range for this role is determined by a number of factors including skills, experience, education, certifications and location. The full salary range for this role reflects the competitive labor market value for all employees in these positions across the national market and provides an opportunity to progress as employees grow and develop within the role. Some roles at Liberty Mutual have a corresponding compensation plan which may include commission and/or bonus earnings at rates that vary based on multiple factors set forth in the compensation plan for the role.
+At Liberty Mutual, our goal is to create a workplace where everyone feels valued, supported, and can thrive. We build an environment that welcomes a wide range of perspectives and experiences, with inclusion embedded in every aspect of our culture and reflected in everyday interactions. This comes to life through comprehensive benefits, workplace flexibility, professional development opportunities, and a host of opportunities provided through our Employee Resource Groups. Each employee plays a role in creating our inclusive culture, which supports every individual to do their best work. Together, we cultivate a community where everyone can make a meaningful impact for our business, our customers, and the communities we serve.
+We value your hard work, integrity and commitment to make things better, and we put people first by offering you benefits that support your life and well\-being. To learn more about our benefit offerings please visit: https://LMI.co/Benefits  
+Liberty Mutual is an equal opportunity employer. We will not tolerate discrimination on the basis of race, color, national origin, sex, sexual orientation, gender identity, religion, age, disability, veteran's status, pregnancy, genetic information or on any basis prohibited by federal, state or local law.  
+**Fair Chance Notices**
+* California
+* Los Angeles Incorporated
+* Los Angeles Unincorporated
+* Philadelphia
+* San Francisco</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>in-e399ba3723db74de</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Data Engineer</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Liberty Mutual Insurance</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>indeed</t>
+        </is>
+      </c>
+      <c r="E40">
+        <f>HYPERLINK("https://www.indeed.com/viewjob?jk=e399ba3723db74de", "https://www.indeed.com/viewjob?jk=e399ba3723db74de")</f>
+        <v/>
+      </c>
+      <c r="F40">
+        <f>HYPERLINK("https://searchjobs.libertymutualgroup.com/careers/job/618515551654?utm_source=indeed&amp;domain=libertymutual.com", "https://searchjobs.libertymutualgroup.com/careers/job/618515551654?utm_source=indeed&amp;domain=libertymutual.com")</f>
+        <v/>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Boston, MA, US</t>
+        </is>
+      </c>
+      <c r="H40" s="3" t="n">
+        <v>46065</v>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>**Description**We deliver our customers peace of mind every day by helping them protect what they value most. Our passion for placing the customer at the center of everything we do is drive a transformational shift at Liberty Mutual. Operating as a tech startup within a Fortune 100 company, we are leading a digital disruption that will redefine how people experience insurance.
+The US Retail Markets (USRM) Data and Analytics Engineering team is actively searching for a highly productive Data Engineer for a distributed, dynamic agile team to serve as a technical expert designing, developing, analyzing \&amp; testing innovative data warehouse reporting solutions. This candidate will join an energetic and engaged Claims Data Solutions Engineering team focused on delivering exceptional value to our Claims business partners. You will work collaboratively in an agile squad to design and build data pipelines \&amp; workflows, ingest, curate \&amp; provision data workflows in a Cloud\-based environment as well as own responsibility of thorough end\-to\-end testing.
+ This is a fast\-paced environment providing rapid delivery for our business partners. You will be working in a highly collaborative environment that values speed and quality, with a strong desire to drive change and foster a positive work environment. You will have the opportunity to help lead this change as we grow this culture, mindset, and capability.
+**\*\*This is a hybrid role requiring two days in the office a week in one of the following locations: Plano, TX, Boston, MA, Portsmouth, NH, Indianapolis, IN and Columbus, OH\*\***
+ **\*\******You must be authorized to work in the United States without employer sponsorship now or in the future. We will not sponsor employment visas. Candidates who will require future sponsorship, including candidates on CPT/OPT/STEMOPT who will require future sponsorship, are not eligible to apply.*** **\*\***
+We encourage you to apply if this interests you:
+Work as ONE team committed to excellence.
+Model and promote a Data First attitude.
+ Help advance Data Engineering operations into the future.
+Work with a modern data tech stack.
+About the job:
+Work in a dynamic and exciting agile environment with Scrum Masters, Product Owners, and team members.
+Analyze, develop, and execute data integration solutions, to manage the information lifecycle needs of an organization.
+Actively participates in code reviews within each Agile sprint, with focus on test driven development and Continuous Integration and Continuous Development (CICD).
+Designs and builds data provisioning workflows/pipelines, physical data schemas, extracts, data transformations, and data integrations and/or designs using ETL and API microservices.
+Build data architecture and data applications (marts/warehouses) that enable reporting, analytics, data science, and data management and improve accessibility, efficiency, governance, processing, and quality of data.
+Improve speed to market by focusing on current data needs as well as building out the long\-term strategic data solutions using AWS, Snowflake, SQL, Data Vault methodology, as well as other modern data technologies.
+Design and develop programs and tools to support ingestion, curation, and provisioning of complex enterprise data to achieve analytics, reporting, and data science.
+Demonstrate an open\-minded and collaborative approach to creating innovative technical solutions.
+Continuously learn to maintain strong knowledge of technology enablers
+Mentor new and junior developers.
+Provide successful deployment and provisioning of data solutions to production or other required environments.
+Analyze complex technical problems and is expected to recommend process improvements that address complex technology gaps within a single business process and improve data reliability, quality, and efficiency.
+**Qualifications**
+Bachelor\`s degree in technical or business discipline or equivalent experience. Generally, 3\+ years of professional experience.
+Experience integrating Guidewire systems with Snowflake for reporting, analytics, or data warehousing purposes, often using APIs and ETL tools.
+Knowledge of a variety of data platforms including Snowflake, Teradata, SQL, DB2 (Cloud based DB a plus).
+Experience with AWS (such as S3, Snowflake, Athena), Unix, Informatica (IDMC) and strong SQL skillset.
+Strong oral and written communication skills; presentation skills. Proficient in negotiation, facilitation and consensus building skills.
+Knowledge of layered systems architectures and layered solutions and designs, understanding of shared data engineering concepts of agile data engineering concepts and processes
+Must be proactive and demonstrate initiative and be a logical thinker. Consultative skills, including the ability to understand and apply customer requirements, including drawing out unforeseen implications and making recommendations for design, the ability to define design reasoning, understanding potential impacts of design requirements. Collaboration, prioritization, and adaptability skills required.
+Additional Qualifications:
+Snowflake, NoSQL, Python development experience.
+Understanding Cloud / Hybrid data architecture concepts.
+Understanding of insurance industry and products.
+Excited by trying new technology and learning new tools.
+ **About Us****Pay Philosophy:** The typical starting salary range for this role is determined by a number of factors including skills, experience, education, certifications and location. The full salary range for this role reflects the competitive labor market value for all employees in these positions across the national market and provides an opportunity to progress as employees grow and develop within the role. Some roles at Liberty Mutual have a corresponding compensation plan which may include commission and/or bonus earnings at rates that vary based on multiple factors set forth in the compensation plan for the role.
+At Liberty Mutual, our goal is to create a workplace where everyone feels valued, supported, and can thrive. We build an environment that welcomes a wide range of perspectives and experiences, with inclusion embedded in every aspect of our culture and reflected in everyday interactions. This comes to life through comprehensive benefits, workplace flexibility, professional development opportunities, and a host of opportunities provided through our Employee Resource Groups. Each employee plays a role in creating our inclusive culture, which supports every individual to do their best work. Together, we cultivate a community where everyone can make a meaningful impact for our business, our customers, and the communities we serve.
+We value your hard work, integrity and commitment to make things better, and we put people first by offering you benefits that support your life and well\-being. To learn more about our benefit offerings please visit: https://LMI.co/Benefits  
+Liberty Mutual is an equal opportunity employer. We will not tolerate discrimination on the basis of race, color, national origin, sex, sexual orientation, gender identity, religion, age, disability, veteran's status, pregnancy, genetic information or on any basis prohibited by federal, state or local law.  
+**Fair Chance Notices**
+* California
+* Los Angeles Incorporated
+* Los Angeles Unincorporated
+* Philadelphia
+* San Francisco</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>in-795130d358ca7647</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Data Engineer</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Liberty Mutual Insurance</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>indeed</t>
+        </is>
+      </c>
+      <c r="E41">
+        <f>HYPERLINK("https://www.indeed.com/viewjob?jk=795130d358ca7647", "https://www.indeed.com/viewjob?jk=795130d358ca7647")</f>
+        <v/>
+      </c>
+      <c r="F41">
+        <f>HYPERLINK("https://searchjobs.libertymutualgroup.com/careers/job/618515551654?utm_source=indeed&amp;domain=libertymutual.com", "https://searchjobs.libertymutualgroup.com/careers/job/618515551654?utm_source=indeed&amp;domain=libertymutual.com")</f>
+        <v/>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Portsmouth, NH, US</t>
+        </is>
+      </c>
+      <c r="H41" s="3" t="n">
+        <v>46065</v>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>**Description**We deliver our customers peace of mind every day by helping them protect what they value most. Our passion for placing the customer at the center of everything we do is drive a transformational shift at Liberty Mutual. Operating as a tech startup within a Fortune 100 company, we are leading a digital disruption that will redefine how people experience insurance.
+The US Retail Markets (USRM) Data and Analytics Engineering team is actively searching for a highly productive Data Engineer for a distributed, dynamic agile team to serve as a technical expert designing, developing, analyzing \&amp; testing innovative data warehouse reporting solutions. This candidate will join an energetic and engaged Claims Data Solutions Engineering team focused on delivering exceptional value to our Claims business partners. You will work collaboratively in an agile squad to design and build data pipelines \&amp; workflows, ingest, curate \&amp; provision data workflows in a Cloud\-based environment as well as own responsibility of thorough end\-to\-end testing.
+ This is a fast\-paced environment providing rapid delivery for our business partners. You will be working in a highly collaborative environment that values speed and quality, with a strong desire to drive change and foster a positive work environment. You will have the opportunity to help lead this change as we grow this culture, mindset, and capability.
+**\*\*This is a hybrid role requiring two days in the office a week in one of the following locations: Plano, TX, Boston, MA, Portsmouth, NH, Indianapolis, IN and Columbus, OH\*\***
+ **\*\******You must be authorized to work in the United States without employer sponsorship now or in the future. We will not sponsor employment visas. Candidates who will require future sponsorship, including candidates on CPT/OPT/STEMOPT who will require future sponsorship, are not eligible to apply.*** **\*\***
+We encourage you to apply if this interests you:
+Work as ONE team committed to excellence.
+Model and promote a Data First attitude.
+ Help advance Data Engineering operations into the future.
+Work with a modern data tech stack.
+About the job:
+Work in a dynamic and exciting agile environment with Scrum Masters, Product Owners, and team members.
+Analyze, develop, and execute data integration solutions, to manage the information lifecycle needs of an organization.
+Actively participates in code reviews within each Agile sprint, with focus on test driven development and Continuous Integration and Continuous Development (CICD).
+Designs and builds data provisioning workflows/pipelines, physical data schemas, extracts, data transformations, and data integrations and/or designs using ETL and API microservices.
+Build data architecture and data applications (marts/warehouses) that enable reporting, analytics, data science, and data management and improve accessibility, efficiency, governance, processing, and quality of data.
+Improve speed to market by focusing on current data needs as well as building out the long\-term strategic data solutions using AWS, Snowflake, SQL, Data Vault methodology, as well as other modern data technologies.
+Design and develop programs and tools to support ingestion, curation, and provisioning of complex enterprise data to achieve analytics, reporting, and data science.
+Demonstrate an open\-minded and collaborative approach to creating innovative technical solutions.
+Continuously learn to maintain strong knowledge of technology enablers
+Mentor new and junior developers.
+Provide successful deployment and provisioning of data solutions to production or other required environments.
+Analyze complex technical problems and is expected to recommend process improvements that address complex technology gaps within a single business process and improve data reliability, quality, and efficiency.
+**Qualifications**
+Bachelor\`s degree in technical or business discipline or equivalent experience. Generally, 3\+ years of professional experience.
+Experience integrating Guidewire systems with Snowflake for reporting, analytics, or data warehousing purposes, often using APIs and ETL tools.
+Knowledge of a variety of data platforms including Snowflake, Teradata, SQL, DB2 (Cloud based DB a plus).
+Experience with AWS (such as S3, Snowflake, Athena), Unix, Informatica (IDMC) and strong SQL skillset.
+Strong oral and written communication skills; presentation skills. Proficient in negotiation, facilitation and consensus building skills.
+Knowledge of layered systems architectures and layered solutions and designs, understanding of shared data engineering concepts of agile data engineering concepts and processes
+Must be proactive and demonstrate initiative and be a logical thinker. Consultative skills, including the ability to understand and apply customer requirements, including drawing out unforeseen implications and making recommendations for design, the ability to define design reasoning, understanding potential impacts of design requirements. Collaboration, prioritization, and adaptability skills required.
+Additional Qualifications:
+Snowflake, NoSQL, Python development experience.
+Understanding Cloud / Hybrid data architecture concepts.
+Understanding of insurance industry and products.
+Excited by trying new technology and learning new tools.
+ **About Us****Pay Philosophy:** The typical starting salary range for this role is determined by a number of factors including skills, experience, education, certifications and location. The full salary range for this role reflects the competitive labor market value for all employees in these positions across the national market and provides an opportunity to progress as employees grow and develop within the role. Some roles at Liberty Mutual have a corresponding compensation plan which may include commission and/or bonus earnings at rates that vary based on multiple factors set forth in the compensation plan for the role.
+At Liberty Mutual, our goal is to create a workplace where everyone feels valued, supported, and can thrive. We build an environment that welcomes a wide range of perspectives and experiences, with inclusion embedded in every aspect of our culture and reflected in everyday interactions. This comes to life through comprehensive benefits, workplace flexibility, professional development opportunities, and a host of opportunities provided through our Employee Resource Groups. Each employee plays a role in creating our inclusive culture, which supports every individual to do their best work. Together, we cultivate a community where everyone can make a meaningful impact for our business, our customers, and the communities we serve.
+We value your hard work, integrity and commitment to make things better, and we put people first by offering you benefits that support your life and well\-being. To learn more about our benefit offerings please visit: https://LMI.co/Benefits  
+Liberty Mutual is an equal opportunity employer. We will not tolerate discrimination on the basis of race, color, national origin, sex, sexual orientation, gender identity, religion, age, disability, veteran's status, pregnancy, genetic information or on any basis prohibited by federal, state or local law.  
+**Fair Chance Notices**
+* California
+* Los Angeles Incorporated
+* Los Angeles Unincorporated
+* Philadelphia
+* San Francisco</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>in-80cd866c899d8f8c</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Data Engineer, Denied Party Screening, AWS Compliance &amp; Security Assurance</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Amazon.com</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>indeed</t>
+        </is>
+      </c>
+      <c r="E42">
+        <f>HYPERLINK("https://www.indeed.com/viewjob?jk=80cd866c899d8f8c", "https://www.indeed.com/viewjob?jk=80cd866c899d8f8c")</f>
+        <v/>
+      </c>
+      <c r="F42">
+        <f>HYPERLINK("https://www.amazon.jobs/jobs/3160403/data-engineer-denied-party-screening-aws-compliance--security-assurance?cmpid=DA_INAD200785B", "https://www.amazon.jobs/jobs/3160403/data-engineer-denied-party-screening-aws-compliance--security-assurance?cmpid=DA_INAD200785B")</f>
+        <v/>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Seattle, WA, US</t>
+        </is>
+      </c>
+      <c r="H42" s="3" t="n">
+        <v>46029</v>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>**DESCRIPTION**
+---------------
+Amazon seeks an experienced Data Engineer to join the DPS (Deny Party Screening) team. Our mission is to prevent denied parties from transacting with Amazon businesses, including AWS, customers, vendors, sellers, subsidiaries, etc. We screen billions of events every day. We integrate with Tier 1 systems, build DPS systems, and deal with unique scaling challenges.  
+As a Data Engineer, you will design, implement and support scalable data infrastructure solutions to integrate with multi heterogeneous data sources, aggregate and retrieve data in a fast and safe mode, curate data that can be used in reporting, analysis, machine learning models and ad\-hoc data requests. You will be exposed to cutting edge AWS big data technologies. You should have excellent business and communication skills to be able to work with business owners and Tech leaders to gather infrastructure requirements, design data infrastructure, build up data pipelines and datasets to meet business needs. You stay abreast of emerging technologies, investigating and implementing where appropriate.  
+Key job responsibilities  
+* Design, implement, and support data warehouse/ data lake infrastructure using AWS bigdata stack, Python, Redshift, QuickSight, Glue/lake formation, EMR/Spark, Athena etc.
+* Develop and manage ETLs to source data from various financial, AWS networking and operational systems and create unified data model for analytics and reporting.
+* Creation and support of real\-time data pipelines built on AWS technologies including EMR, Glue, Redshift/Spectrum and Athena.
+* Collaborate with other Engineering teams, Product/Finance Managers/Analysts to implement advanced analytics algorithms that exploit our rich datasets for financial model development, statistical analysis, prediction, etc.
+* Continual research of the latest big data and visualization technologies to provide new capabilities and increase efficiency.
+* Use business intelligence and visualization software (e.g., QuickSight) to develop dashboards those are used by senior leadership.
+* Empower technical and non\-technical, internal customers to drive their own analytics and reporting (self\-serve reporting) and support ad\-hoc reporting when needed.
+* Working closely with team members to drive real\-time model implementations for monitoring and alerting of risk systems.
+* Manage numerous requests concurrently and strategically, prioritizing when necessary
+* Partner/collaborate across teams/roles to deliver results.
+* Mentor other engineers, influence positively team culture, and help grow the team
+About the team  
+Denied Party Screening (DPS) is a part of Amazon Security, an organization designed to drive bar\-raising security engagements. The vision of the Amazon DPS program is to ensure that 1\+ billion Amazon accounts spanning across consumers, sellers, developers, employees, and all other Amazon party, are not a denied party, located or incorporated in a sanctioned region or country, or owned or controlled by or subject to the jurisdiction of the government of a sanctioned country.
+Why Amazon Security  
+At Amazon, security is central to maintaining customer trust and delivering delightful customer experiences. Our organization is responsible for creating and maintaining a high bar for security across all of Amazon’s products and services.  
+Work/Life Balance  
+We value work\-life harmony. Achieving success at work should never come at the expense of sacrifices at home, which is why flexible work hours and arrangements are part of our culture. When we feel supported in the workplace and at home, there’s nothing we can’t achieve.  
+Inclusive Team Culture  
+In Amazon Security, it’s in our nature to learn and be curious. Ongoing DEI events and learning experiences inspire us to continue learning and to embrace our uniqueness. Addressing the toughest security challenges requires that we seek out and celebrate a diversity of ideas, perspectives, and voices.  
+Training and Career growth  
+We’re continuously raising our performance bar as we strive to become Earth’s Best Employer. That’s why you’ll find endless knowledge\-sharing, training, and other career\-advancing resources here to help you develop into a better\-rounded professional.**BASIC QUALIFICATIONS**
+------------------------
+* 5\+ years of data engineering experience
+* Experience programming with at least one modern language such as C\+\+, C\#, Java, Python, Golang, PowerShell, Ruby
+* Experience working on and delivering end to end projects independently
+* Experience with big data technologies such as: Hadoop, Hive, Spark, EMR
+**PREFERRED QUALIFICATIONS**
+----------------------------
+* Experience with AWS technologies like Redshift, S3, AWS Glue, EMR, Kinesis, FireHose, Lambda, and IAM roles and permissions
+* Experience with non\-relational databases / data stores (object storage, document or key\-value stores, graph databases, column\-family databases)
+* Experience in at least one modern scripting or programming language, such as Python, Java, Scala, or NodeJS
+* Experience with distributed systems as it pertains to data storage and computing
+* Experience as a data engineer or related specialty (e.g., software engineer, business intelligence engineer, data scientist) with a track record of manipulating, processing, and extracting value from large datasets
+* Experience providing technical leadership and mentoring other engineers for best practices on data engineering
+Amazon is an equal opportunity employer and does not discriminate on the basis of protected veteran status, disability, or other legally protected status.  
+Our inclusive culture empowers Amazonians to deliver the best results for our customers. If you have a disability and need a workplace accommodation or adjustment during the application and hiring process, including support for the interview or onboarding process, please visit https://amazon.jobs/content/en/how\-we\-hire/accommodations for more information. If the country/region you’re applying in isn’t listed, please contact your Recruiting Partner.  
+The base salary range for this position is listed below. Your Amazon package will include sign\-on payments and restricted stock units (RSUs). Final compensation will be determined based on factors including experience, qualifications, and location. Amazon also offers comprehensive benefits including health insurance (medical, dental, vision, prescription, Basic Life \&amp; AD\&amp;D insurance and option for Supplemental life plans, EAP, Mental Health Support, Medical Advice Line, Flexible Spending Accounts, Adoption and Surrogacy Reimbursement coverage), 401(k) matching, paid time off, and parental leave. Learn more about our benefits at https://amazon.jobs/en/benefits.
+USA, TX, Dallas \- 132,100\.00 \- 178,800\.00 USD annually  
+USA, WA, Seattle \- 132,100\.00 \- 178,800\.00 USD annually</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>in-71f0595ea6b2ae6e</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Data Engineer, Denied Party Screening, AWS Compliance &amp; Security Assurance</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Amazon.com</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>indeed</t>
+        </is>
+      </c>
+      <c r="E43">
+        <f>HYPERLINK("https://www.indeed.com/viewjob?jk=71f0595ea6b2ae6e", "https://www.indeed.com/viewjob?jk=71f0595ea6b2ae6e")</f>
+        <v/>
+      </c>
+      <c r="F43">
+        <f>HYPERLINK("https://www.amazon.jobs/jobs/3160403/data-engineer-denied-party-screening-aws-compliance--security-assurance?cmpid=DA_INAD200785B", "https://www.amazon.jobs/jobs/3160403/data-engineer-denied-party-screening-aws-compliance--security-assurance?cmpid=DA_INAD200785B")</f>
+        <v/>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Dallas, TX, US</t>
+        </is>
+      </c>
+      <c r="H43" s="3" t="n">
+        <v>46029</v>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>**DESCRIPTION**
+---------------
+Amazon seeks an experienced Data Engineer to join the DPS (Deny Party Screening) team. Our mission is to prevent denied parties from transacting with Amazon businesses, including AWS, customers, vendors, sellers, subsidiaries, etc. We screen billions of events every day. We integrate with Tier 1 systems, build DPS systems, and deal with unique scaling challenges.  
+As a Data Engineer, you will design, implement and support scalable data infrastructure solutions to integrate with multi heterogeneous data sources, aggregate and retrieve data in a fast and safe mode, curate data that can be used in reporting, analysis, machine learning models and ad\-hoc data requests. You will be exposed to cutting edge AWS big data technologies. You should have excellent business and communication skills to be able to work with business owners and Tech leaders to gather infrastructure requirements, design data infrastructure, build up data pipelines and datasets to meet business needs. You stay abreast of emerging technologies, investigating and implementing where appropriate.  
+Key job responsibilities  
+* Design, implement, and support data warehouse/ data lake infrastructure using AWS bigdata stack, Python, Redshift, QuickSight, Glue/lake formation, EMR/Spark, Athena etc.
+* Develop and manage ETLs to source data from various financial, AWS networking and operational systems and create unified data model for analytics and reporting.
+* Creation and support of real\-time data pipelines built on AWS technologies including EMR, Glue, Redshift/Spectrum and Athena.
+* Collaborate with other Engineering teams, Product/Finance Managers/Analysts to implement advanced analytics algorithms that exploit our rich datasets for financial model development, statistical analysis, prediction, etc.
+* Continual research of the latest big data and visualization technologies to provide new capabilities and increase efficiency.
+* Use business intelligence and visualization software (e.g., QuickSight) to develop dashboards those are used by senior leadership.
+* Empower technical and non\-technical, internal customers to drive their own analytics and reporting (self\-serve reporting) and support ad\-hoc reporting when needed.
+* Working closely with team members to drive real\-time model implementations for monitoring and alerting of risk systems.
+* Manage numerous requests concurrently and strategically, prioritizing when necessary
+* Partner/collaborate across teams/roles to deliver results.
+* Mentor other engineers, influence positively team culture, and help grow the team
+About the team  
+Denied Party Screening (DPS) is a part of Amazon Security, an organization designed to drive bar\-raising security engagements. The vision of the Amazon DPS program is to ensure that 1\+ billion Amazon accounts spanning across consumers, sellers, developers, employees, and all other Amazon party, are not a denied party, located or incorporated in a sanctioned region or country, or owned or controlled by or subject to the jurisdiction of the government of a sanctioned country.
+Why Amazon Security  
+At Amazon, security is central to maintaining customer trust and delivering delightful customer experiences. Our organization is responsible for creating and maintaining a high bar for security across all of Amazon’s products and services.  
+Work/Life Balance  
+We value work\-life harmony. Achieving success at work should never come at the expense of sacrifices at home, which is why flexible work hours and arrangements are part of our culture. When we feel supported in the workplace and at home, there’s nothing we can’t achieve.  
+Inclusive Team Culture  
+In Amazon Security, it’s in our nature to learn and be curious. Ongoing DEI events and learning experiences inspire us to continue learning and to embrace our uniqueness. Addressing the toughest security challenges requires that we seek out and celebrate a diversity of ideas, perspectives, and voices.  
+Training and Career growth  
+We’re continuously raising our performance bar as we strive to become Earth’s Best Employer. That’s why you’ll find endless knowledge\-sharing, training, and other career\-advancing resources here to help you develop into a better\-rounded professional.**BASIC QUALIFICATIONS**
+------------------------
+* 5\+ years of data engineering experience
+* Experience programming with at least one modern language such as C\+\+, C\#, Java, Python, Golang, PowerShell, Ruby
+* Experience working on and delivering end to end projects independently
+* Experience with big data technologies such as: Hadoop, Hive, Spark, EMR
+**PREFERRED QUALIFICATIONS**
+----------------------------
+* Experience with AWS technologies like Redshift, S3, AWS Glue, EMR, Kinesis, FireHose, Lambda, and IAM roles and permissions
+* Experience with non\-relational databases / data stores (object storage, document or key\-value stores, graph databases, column\-family databases)
+* Experience in at least one modern scripting or programming language, such as Python, Java, Scala, or NodeJS
+* Experience with distributed systems as it pertains to data storage and computing
+* Experience as a data engineer or related specialty (e.g., software engineer, business intelligence engineer, data scientist) with a track record of manipulating, processing, and extracting value from large datasets
+* Experience providing technical leadership and mentoring other engineers for best practices on data engineering
+Amazon is an equal opportunity employer and does not discriminate on the basis of protected veteran status, disability, or other legally protected status.  
+Our inclusive culture empowers Amazonians to deliver the best results for our customers. If you have a disability and need a workplace accommodation or adjustment during the application and hiring process, including support for the interview or onboarding process, please visit https://amazon.jobs/content/en/how\-we\-hire/accommodations for more information. If the country/region you’re applying in isn’t listed, please contact your Recruiting Partner.  
+The base salary range for this position is listed below. Your Amazon package will include sign\-on payments and restricted stock units (RSUs). Final compensation will be determined based on factors including experience, qualifications, and location. Amazon also offers comprehensive benefits including health insurance (medical, dental, vision, prescription, Basic Life \&amp; AD\&amp;D insurance and option for Supplemental life plans, EAP, Mental Health Support, Medical Advice Line, Flexible Spending Accounts, Adoption and Surrogacy Reimbursement coverage), 401(k) matching, paid time off, and parental leave. Learn more about our benefits at https://amazon.jobs/en/benefits.
+USA, TX, Dallas \- 132,100\.00 \- 178,800\.00 USD annually  
+USA, WA, Seattle \- 132,100\.00 \- 178,800\.00 USD annually</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>in-7de6cbf75b9bc482</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Data Engineer</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Amazon.com</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>indeed</t>
+        </is>
+      </c>
+      <c r="E44">
+        <f>HYPERLINK("https://www.indeed.com/viewjob?jk=7de6cbf75b9bc482", "https://www.indeed.com/viewjob?jk=7de6cbf75b9bc482")</f>
+        <v/>
+      </c>
+      <c r="F44">
+        <f>HYPERLINK("https://www.amazon.jobs/jobs/3141339/data-engineer?cmpid=DA_INAD200785B", "https://www.amazon.jobs/jobs/3141339/data-engineer?cmpid=DA_INAD200785B")</f>
+        <v/>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>San Francisco, CA, US</t>
+        </is>
+      </c>
+      <c r="H44" s="3" t="n">
+        <v>46001</v>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>**DESCRIPTION**
+---------------
+If you are interested in this position, please apply on Twitch's Career site https://www.twitch.tv/jobs/en/  
+About Us:  
+Twitch is the world’s biggest live streaming service, with global communities built around gaming, entertainment, music, sports, cooking, and more. It is where thousands of communities come together for whatever, every day.  
+We’re about community, inside and out. You’ll find coworkers who are eager to team up, collaborate, and smash (or elegantly solve) problems together. We’re on a quest to empower live communities, so if this sounds good to you, see what we’re up to on LinkedIn and X, and discover the projects we’re solving on our Blog. Be sure to explore our Interviewing Guide to learn how to ace our interview process.  
+About the Role  
+As a data engineer in the Data Platform organization, you will be transforming Twitch’s largest data sets into offerings that are usable by the entire company. You’ll be working with other senior team members, as well as other data engineers, scientists, and stakeholders from all across the business. You will help define how our core business metrics are managed, as well as how other parts of the company define their individual metrics.  
+You Will  
+* Work closely with data scientists and engineers from across the company to define and create robust data architectures and pipelines
+* Develop and manage scalable data pipelines to extract, transform, and load data from various sources
+* Partner with a range of stakeholders to translate the company’s needs into data offerings
+* Automate data processing and reporting workflows to improve efficiency and data integrity
+* Implement data quality checks and monitor processes to maintain high data accuracy
+* Simplify and enhance the accessibility, clarity, and usability of large and complex datasets through the development of data cubes and data sharing solutions
+Perks  
+* Medical, Dental, Vision \&amp; Disability Insurance
+* 401(k)
+* Maternity \&amp; Parental Leave
+* Flexible PTO
+* Amazon Employee Discount
+**BASIC QUALIFICATIONS**
+------------------------
+* 3\+ years of data engineering experience
+* 3\+ year of experience working in a data engineering, data science, or software engineering capacity
+* Expertise in writing and maintaining robust data pipelines in SQL and Python
+* A track record of turning data requirements from stakeholders into actionable plans
+* Experience with cloud\-native solutions
+* A history of implementing and upholding best practices in data pipelines, ensuring accuracy, consistency, and reliability
+**PREFERRED QUALIFICATIONS**
+----------------------------
+* Bachelor's degree, or Master's degree in computer science, statistics, information systems, or a related, technical field
+* Experience with a scripting language (e.g., Python, Java, or R)
+* Familiarity and interest in Twitch!
+Twitch is an equal opportunity employer and does not discriminate on the basis of protected veteran status, disability, or other legally protected status.  
+Los Angeles County applicants: Job duties for this position include: work safely and cooperatively with other employees, supervisors, and staff; adhere to standards of excellence despite stressful conditions; communicate effectively and respectfully with employees, supervisors, and staff to ensure exceptional customer service; and follow all federal, state, and local laws and Company policies. Criminal history may have a direct, adverse, and negative relationship with some of the material job duties of this position. These include the duties and responsibilities listed above, as well as the abilities to adhere to company policies, exercise sound judgment, effectively manage stress and work safely and respectfully with others, exhibit trustworthiness and professionalism, and safeguard business operations and the Company’s reputation. Pursuant to the Los Angeles County Fair Chance Ordinance, we will consider for employment qualified applicants with arrest and conviction records.  
+Pursuant to the San Francisco Fair Chance Ordinance, we will consider for employment qualified applicants with arrest and conviction records.  
+Our inclusive culture empowers Amazonians to deliver the best results for our customers. If you have a disability and need a workplace accommodation or adjustment during the application and hiring process, including support for the interview or onboarding process, please visit https://amazon.jobs/content/en/how\-we\-hire/accommodations for more information. If the country/region you’re applying in isn’t listed, please contact your Recruiting Partner.  
+The base salary range for this position is listed below. Your Amazon package will include sign\-on payments and restricted stock units (RSUs). Final compensation will be determined based on factors including experience, qualifications, and location. Amazon also offers comprehensive benefits including health insurance (medical, dental, vision, prescription, Basic Life \&amp; AD\&amp;D insurance and option for Supplemental life plans, EAP, Mental Health Support, Medical Advice Line, Flexible Spending Accounts, Adoption and Surrogacy Reimbursement coverage), 401(k) matching, paid time off, and parental leave. Learn more about our benefits at https://amazon.jobs/en/benefits.
+USA, CA, San Francisco \- 152,000\.00 \- 205,600\.00 USD annually  
+USA, WA, SEATTLE \- 132,100\.00 \- 178,800\.00 USD annually  
+USA, WA, Seattle \- 132,100\.00 \- 178,800\.00 USD annually</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>in-f90f2ec36f80df06</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Data Engineer</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Amazon.com</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>indeed</t>
+        </is>
+      </c>
+      <c r="E45">
+        <f>HYPERLINK("https://www.indeed.com/viewjob?jk=f90f2ec36f80df06", "https://www.indeed.com/viewjob?jk=f90f2ec36f80df06")</f>
+        <v/>
+      </c>
+      <c r="F45">
+        <f>HYPERLINK("https://www.amazon.jobs/jobs/3141339/data-engineer?cmpid=DA_INAD200785B", "https://www.amazon.jobs/jobs/3141339/data-engineer?cmpid=DA_INAD200785B")</f>
+        <v/>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Seattle, WA, US</t>
+        </is>
+      </c>
+      <c r="H45" s="3" t="n">
+        <v>46001</v>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>**DESCRIPTION**
+---------------
+If you are interested in this position, please apply on Twitch's Career site https://www.twitch.tv/jobs/en/  
+About Us:  
+Twitch is the world’s biggest live streaming service, with global communities built around gaming, entertainment, music, sports, cooking, and more. It is where thousands of communities come together for whatever, every day.  
+We’re about community, inside and out. You’ll find coworkers who are eager to team up, collaborate, and smash (or elegantly solve) problems together. We’re on a quest to empower live communities, so if this sounds good to you, see what we’re up to on LinkedIn and X, and discover the projects we’re solving on our Blog. Be sure to explore our Interviewing Guide to learn how to ace our interview process.  
+About the Role  
+As a data engineer in the Data Platform organization, you will be transforming Twitch’s largest data sets into offerings that are usable by the entire company. You’ll be working with other senior team members, as well as other data engineers, scientists, and stakeholders from all across the business. You will help define how our core business metrics are managed, as well as how other parts of the company define their individual metrics.  
+You Will  
+* Work closely with data scientists and engineers from across the company to define and create robust data architectures and pipelines
+* Develop and manage scalable data pipelines to extract, transform, and load data from various sources
+* Partner with a range of stakeholders to translate the company’s needs into data offerings
+* Automate data processing and reporting workflows to improve efficiency and data integrity
+* Implement data quality checks and monitor processes to maintain high data accuracy
+* Simplify and enhance the accessibility, clarity, and usability of large and complex datasets through the development of data cubes and data sharing solutions
+Perks  
+* Medical, Dental, Vision \&amp; Disability Insurance
+* 401(k)
+* Maternity \&amp; Parental Leave
+* Flexible PTO
+* Amazon Employee Discount
+**BASIC QUALIFICATIONS**
+------------------------
+* 3\+ years of data engineering experience
+* 3\+ year of experience working in a data engineering, data science, or software engineering capacity
+* Expertise in writing and maintaining robust data pipelines in SQL and Python
+* A track record of turning data requirements from stakeholders into actionable plans
+* Experience with cloud\-native solutions
+* A history of implementing and upholding best practices in data pipelines, ensuring accuracy, consistency, and reliability
+**PREFERRED QUALIFICATIONS**
+----------------------------
+* Bachelor's degree, or Master's degree in computer science, statistics, information systems, or a related, technical field
+* Experience with a scripting language (e.g., Python, Java, or R)
+* Familiarity and interest in Twitch!
+Twitch is an equal opportunity employer and does not discriminate on the basis of protected veteran status, disability, or other legally protected status.  
+Los Angeles County applicants: Job duties for this position include: work safely and cooperatively with other employees, supervisors, and staff; adhere to standards of excellence despite stressful conditions; communicate effectively and respectfully with employees, supervisors, and staff to ensure exceptional customer service; and follow all federal, state, and local laws and Company policies. Criminal history may have a direct, adverse, and negative relationship with some of the material job duties of this position. These include the duties and responsibilities listed above, as well as the abilities to adhere to company policies, exercise sound judgment, effectively manage stress and work safely and respectfully with others, exhibit trustworthiness and professionalism, and safeguard business operations and the Company’s reputation. Pursuant to the Los Angeles County Fair Chance Ordinance, we will consider for employment qualified applicants with arrest and conviction records.  
+Pursuant to the San Francisco Fair Chance Ordinance, we will consider for employment qualified applicants with arrest and conviction records.  
+Our inclusive culture empowers Amazonians to deliver the best results for our customers. If you have a disability and need a workplace accommodation or adjustment during the application and hiring process, including support for the interview or onboarding process, please visit https://amazon.jobs/content/en/how\-we\-hire/accommodations for more information. If the country/region you’re applying in isn’t listed, please contact your Recruiting Partner.  
+The base salary range for this position is listed below. Your Amazon package will include sign\-on payments and restricted stock units (RSUs). Final compensation will be determined based on factors including experience, qualifications, and location. Amazon also offers comprehensive benefits including health insurance (medical, dental, vision, prescription, Basic Life \&amp; AD\&amp;D insurance and option for Supplemental life plans, EAP, Mental Health Support, Medical Advice Line, Flexible Spending Accounts, Adoption and Surrogacy Reimbursement coverage), 401(k) matching, paid time off, and parental leave. Learn more about our benefits at https://amazon.jobs/en/benefits.
+USA, CA, San Francisco \- 152,000\.00 \- 205,600\.00 USD annually  
+USA, WA, SEATTLE \- 132,100\.00 \- 178,800\.00 USD annually  
+USA, WA, Seattle \- 132,100\.00 \- 178,800\.00 USD annually</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t>in-d8ade13275994228</t>
+        </is>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>Delivery Consultant - Data Engineer, Data and Machine Learning, WWPS US Federal</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>Amazon Web Services</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>indeed</t>
+        </is>
+      </c>
+      <c r="E46">
+        <f>HYPERLINK("https://www.indeed.com/viewjob?jk=d8ade13275994228", "https://www.indeed.com/viewjob?jk=d8ade13275994228")</f>
+        <v/>
+      </c>
+      <c r="F46">
+        <f>HYPERLINK("https://www.amazon.jobs/jobs/3134583/delivery-consultant--data-engineer-data-and-machine-learning-wwps-us-federal?cmpid=DA_INAD200785B", "https://www.amazon.jobs/jobs/3134583/delivery-consultant--data-engineer-data-and-machine-learning-wwps-us-federal?cmpid=DA_INAD200785B")</f>
+        <v/>
+      </c>
+      <c r="G46" t="inlineStr">
+        <is>
+          <t>Herndon, VA, US</t>
+        </is>
+      </c>
+      <c r="H46" s="3" t="n">
+        <v>45991</v>
+      </c>
+      <c r="I46" t="inlineStr">
+        <is>
+          <t>**DESCRIPTION**
+---------------
+The Amazon Web Services Professional Services (ProServe) team is seeking a skilled Delivery Consultant to join our team at Amazon Web Services (AWS). In this role, you'll work closely with customers to design, implement, and manage AWS solutions that meet their technical requirements and business objectives. You'll be a key player in driving customer success through their cloud journey, providing technical expertise and best practices throughout the project lifecycle.  
+Possessing a deep understanding of AWS products and services, as a Delivery Consultant you will be proficient in architecting complex, scalable, and secure solutions tailored to meet the specific needs of each customer. You’ll work closely with stakeholders to gather requirements, assess current infrastructure, and propose effective migration strategies to AWS. As trusted advisors to our customers, providing guidance on industry trends, emerging technologies, and innovative solutions, you will be responsible for leading the implementation process, ensuring adherence to best practices, optimizing performance, and managing risks throughout the project.
+The AWS Professional Services organization is a global team of experts that help customers realize their desired business outcomes when using the AWS Cloud. We work together with customer teams and the AWS Partner Network (APN) to execute enterprise cloud computing initiatives. Our team provides assistance through a collection of offerings which help customers achieve specific outcomes related to enterprise cloud adoption. We also deliver focused guidance through our global specialty practices, which cover a variety of solutions, technologies, and industries.  
+It is expected to work from one of the above locations (or customer sites) Monday through Friday each week. This is not a remote position. You are expected to be in the office or with customers as needed.
+This position requires that the candidate selected be a US Citizen and must currently possess and maintain an active TS/SCI security clearance with polygraph. The position further requires the candidate to opt into a commensurate clearance for each government agency for which they perform AWS work.
+10040  
+Key job responsibilities  
+As an experienced technology professional, you will be responsible for:
+* Designing and implementing complex, scalable, and secure AWS solutions tailored to customer needs
+* Providing technical guidance and troubleshooting support throughout project delivery
+* Collaborating with stakeholders to gather requirements and propose effective migration strategies
+* Acting as a trusted advisor to customers on industry trends and emerging technologies
+* Sharing knowledge within the organization through mentoring, training, and creating reusable artifacts
+About the team  
+Why AWS?  
+Amazon Web Services (AWS) is the world’s most comprehensive and broadly adopted cloud platform. We pioneered cloud computing and never stopped innovating — that’s why customers from the most successful startups to Global 500 companies trust our robust suite of products and services to power their businesses.  
+Diverse Experiences  
+AWS values diverse experiences. Even if you do not meet all of the qualifications and skills listed in the job description, we encourage candidates to apply. If your career is just starting, hasn’t followed a traditional path, or includes alternative experiences, don’t let it stop you from applying.  
+Inclusive Team Culture  
+Here at AWS, it’s in our nature to learn and be curious. Our employee\-led affinity groups foster a culture of inclusion that empower us to be proud of our differences. Ongoing events and learning experiences, including our Conversations on Race and Ethnicity (CORE) and AmazeCon (diversity) conferences, inspire us to never stop embracing our uniqueness.  
+Work/Life Balance  
+We value work\-life harmony. Achieving success at work should never come at the expense of sacrifices at home, which is why flexible work hours and arrangements are part of our culture. When we feel supported in the workplace and at home, there’s nothing we can’t achieve in the cloud.  
+Mentorship \&amp; Career Growth  
+We’re continuously raising our performance bar as we strive to become Earth’s Best Employer. That’s why you’ll find endless knowledge\-sharing, mentorship and other career\-advancing resources here to help you develop into a better\-rounded professional.**BASIC QUALIFICATIONS**
+------------------------
+* Bachelor's degree in Computer Science, Engineering, a related technical field or equivalent
+* 3\+ years of cloud architecture and solution implementation experience
+* 3\+ years of experience with data warehouse architecture, ETL/ELT tools, data engineering, and large\-scale data manipulation using technologies like Spark, EMR, Hive, Kafka, and Redshift.
+* Experience with relational databases, SQL, and performance tuning, as well as software engineering best practices for the development lifecycle, including coding standards, reviews, source control, and testing.
+* Current, active US Government Security Clearance of TS/SCI with Polygraph.
+**PREFERRED QUALIFICATIONS**
+----------------------------
+* AWS Professional level certifications (e.g., Solutions Architect Professional, DevOps Engineer Professional) preferred.
+* Experience with automation and scripting (e.g., Terraform, Python).
+* Knowledge of security and compliance standards (e.g., HIPAA, GDPR).
+* Experience leading large\-scale data engineering and analytics projects using AWS technologies like Redshift, S3, Glue, EMR, Kinesis, Firehose, and Lambda.
+* Experience with non\-relational databases and implementing data governance solutions.
+Amazon is an equal opportunity employer and does not discriminate on the basis of protected veteran status, disability, or other legally protected status.  
+Our inclusive culture empowers Amazonians to deliver the best results for our customers. If you have a disability and need a workplace accommodation or adjustment during the application and hiring process, including support for the interview or onboarding process, please visit https://amazon.jobs/content/en/how\-we\-hire/accommodations for more information. If the country/region you’re applying in isn’t listed, please contact your Recruiting Partner.  
+Our compensation reflects the cost of labor across several US geographic markets. The base pay for this position ranges from $118,200/year in our lowest geographic market up to $204,300/year in our highest geographic market. Pay is based on a number of factors including market location and may vary depending on job\-related knowledge, skills, and experience. Amazon is a total compensation company. Dependent on the position offered, equity, sign\-on payments, and other forms of compensation may be provided as part of a total compensation package, in addition to a full range of medical, financial, and/or other benefits. For more information, please visit https://www.aboutamazon.com/workplace/employee\-benefits. This position will remain posted until filled. Applicants should apply via our internal or external career site.</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="inlineStr">
+        <is>
+          <t>in-206d142ce940177a</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>Delivery Consultant - Data Engineer, Data and Machine Learning, WWPS US Federal</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Amazon Web Services</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>indeed</t>
+        </is>
+      </c>
+      <c r="E47">
+        <f>HYPERLINK("https://www.indeed.com/viewjob?jk=206d142ce940177a", "https://www.indeed.com/viewjob?jk=206d142ce940177a")</f>
+        <v/>
+      </c>
+      <c r="F47">
+        <f>HYPERLINK("https://www.amazon.jobs/jobs/3134583/delivery-consultant--data-engineer-data-and-machine-learning-wwps-us-federal?cmpid=DA_INAD200785B", "https://www.amazon.jobs/jobs/3134583/delivery-consultant--data-engineer-data-and-machine-learning-wwps-us-federal?cmpid=DA_INAD200785B")</f>
+        <v/>
+      </c>
+      <c r="G47" t="inlineStr">
+        <is>
+          <t>Arlington, VA, US</t>
+        </is>
+      </c>
+      <c r="H47" s="3" t="n">
+        <v>45991</v>
+      </c>
+      <c r="I47" t="inlineStr">
+        <is>
+          <t>**DESCRIPTION**
+---------------
+The Amazon Web Services Professional Services (ProServe) team is seeking a skilled Delivery Consultant to join our team at Amazon Web Services (AWS). In this role, you'll work closely with customers to design, implement, and manage AWS solutions that meet their technical requirements and business objectives. You'll be a key player in driving customer success through their cloud journey, providing technical expertise and best practices throughout the project lifecycle.  
+Possessing a deep understanding of AWS products and services, as a Delivery Consultant you will be proficient in architecting complex, scalable, and secure solutions tailored to meet the specific needs of each customer. You’ll work closely with stakeholders to gather requirements, assess current infrastructure, and propose effective migration strategies to AWS. As trusted advisors to our customers, providing guidance on industry trends, emerging technologies, and innovative solutions, you will be responsible for leading the implementation process, ensuring adherence to best practices, optimizing performance, and managing risks throughout the project.
+The AWS Professional Services organization is a global team of experts that help customers realize their desired business outcomes when using the AWS Cloud. We work together with customer teams and the AWS Partner Network (APN) to execute enterprise cloud computing initiatives. Our team provides assistance through a collection of offerings which help customers achieve specific outcomes related to enterprise cloud adoption. We also deliver focused guidance through our global specialty practices, which cover a variety of solutions, technologies, and industries.  
+It is expected to work from one of the above locations (or customer sites) Monday through Friday each week. This is not a remote position. You are expected to be in the office or with customers as needed.
+This position requires that the candidate selected be a US Citizen and must currently possess and maintain an active TS/SCI security clearance with polygraph. The position further requires the candidate to opt into a commensurate clearance for each government agency for which they perform AWS work.
+10040  
+Key job responsibilities  
+As an experienced technology professional, you will be responsible for:
+* Designing and implementing complex, scalable, and secure AWS solutions tailored to customer needs
+* Providing technical guidance and troubleshooting support throughout project delivery
+* Collaborating with stakeholders to gather requirements and propose effective migration strategies
+* Acting as a trusted advisor to customers on industry trends and emerging technologies
+* Sharing knowledge within the organization through mentoring, training, and creating reusable artifacts
+About the team  
+Why AWS?  
+Amazon Web Services (AWS) is the world’s most comprehensive and broadly adopted cloud platform. We pioneered cloud computing and never stopped innovating — that’s why customers from the most successful startups to Global 500 companies trust our robust suite of products and services to power their businesses.  
+Diverse Experiences  
+AWS values diverse experiences. Even if you do not meet all of the qualifications and skills listed in the job description, we encourage candidates to apply. If your career is just starting, hasn’t followed a traditional path, or includes alternative experiences, don’t let it stop you from applying.  
+Inclusive Team Culture  
+Here at AWS, it’s in our nature to learn and be curious. Our employee\-led affinity groups foster a culture of inclusion that empower us to be proud of our differences. Ongoing events and learning experiences, including our Conversations on Race and Ethnicity (CORE) and AmazeCon (diversity) conferences, inspire us to never stop embracing our uniqueness.  
+Work/Life Balance  
+We value work\-life harmony. Achieving success at work should never come at the expense of sacrifices at home, which is why flexible work hours and arrangements are part of our culture. When we feel supported in the workplace and at home, there’s nothing we can’t achieve in the cloud.  
+Mentorship \&amp; Career Growth  
+We’re continuously raising our performance bar as we strive to become Earth’s Best Employer. That’s why you’ll find endless knowledge\-sharing, mentorship and other career\-advancing resources here to help you develop into a better\-rounded professional.**BASIC QUALIFICATIONS**
+------------------------
+* Bachelor's degree in Computer Science, Engineering, a related technical field or equivalent
+* 3\+ years of cloud architecture and solution implementation experience
+* 3\+ years of experience with data warehouse architecture, ETL/ELT tools, data engineering, and large\-scale data manipulation using technologies like Spark, EMR, Hive, Kafka, and Redshift.
+* Experience with relational databases, SQL, and performance tuning, as well as software engineering best practices for the development lifecycle, including coding standards, reviews, source control, and testing.
+* Current, active US Government Security Clearance of TS/SCI with Polygraph.
+**PREFERRED QUALIFICATIONS**
+----------------------------
+* AWS Professional level certifications (e.g., Solutions Architect Professional, DevOps Engineer Professional) preferred.
+* Experience with automation and scripting (e.g., Terraform, Python).
+* Knowledge of security and compliance standards (e.g., HIPAA, GDPR).
+* Experience leading large\-scale data engineering and analytics projects using AWS technologies like Redshift, S3, Glue, EMR, Kinesis, Firehose, and Lambda.
+* Experience with non\-relational databases and implementing data governance solutions.
+Amazon is an equal opportunity employer and does not discriminate on the basis of protected veteran status, disability, or other legally protected status.  
+Our inclusive culture empowers Amazonians to deliver the best results for our customers. If you have a disability and need a workplace accommodation or adjustment during the application and hiring process, including support for the interview or onboarding process, please visit https://amazon.jobs/content/en/how\-we\-hire/accommodations for more information. If the country/region you’re applying in isn’t listed, please contact your Recruiting Partner.  
+Our compensation reflects the cost of labor across several US geographic markets. The base pay for this position ranges from $118,200/year in our lowest geographic market up to $204,300/year in our highest geographic market. Pay is based on a number of factors including market location and may vary depending on job\-related knowledge, skills, and experience. Amazon is a total compensation company. Dependent on the position offered, equity, sign\-on payments, and other forms of compensation may be provided as part of a total compensation package, in addition to a full range of medical, financial, and/or other benefits. For more information, please visit https://www.aboutamazon.com/workplace/employee\-benefits. This position will remain posted until filled. Applicants should apply via our internal or external career site.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -3130,7 +4150,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I118"/>
+  <dimension ref="A1:I132"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -8523,10 +9543,7 @@
           <t>linkedin</t>
         </is>
       </c>
-      <c r="E74">
-        <f>HYPERLINK("https://www.linkedin.com/jobs/view/4363465235", "https://www.linkedin.com/jobs/view/4363465235")</f>
-        <v/>
-      </c>
+      <c r="E74" t="inlineStr"/>
       <c r="F74" t="inlineStr"/>
       <c r="G74" t="inlineStr">
         <is>
@@ -8617,10 +9634,7 @@
           <t>linkedin</t>
         </is>
       </c>
-      <c r="E75">
-        <f>HYPERLINK("https://www.linkedin.com/jobs/view/4364565344", "https://www.linkedin.com/jobs/view/4364565344")</f>
-        <v/>
-      </c>
+      <c r="E75" t="inlineStr"/>
       <c r="F75" t="inlineStr"/>
       <c r="G75" t="inlineStr">
         <is>
@@ -8686,10 +9700,7 @@
           <t>linkedin</t>
         </is>
       </c>
-      <c r="E76">
-        <f>HYPERLINK("https://www.linkedin.com/jobs/view/4373227617", "https://www.linkedin.com/jobs/view/4373227617")</f>
-        <v/>
-      </c>
+      <c r="E76" t="inlineStr"/>
       <c r="F76" t="inlineStr"/>
       <c r="G76" t="inlineStr">
         <is>
@@ -8750,10 +9761,7 @@
           <t>linkedin</t>
         </is>
       </c>
-      <c r="E77">
-        <f>HYPERLINK("https://www.linkedin.com/jobs/view/4373221938", "https://www.linkedin.com/jobs/view/4373221938")</f>
-        <v/>
-      </c>
+      <c r="E77" t="inlineStr"/>
       <c r="F77" t="inlineStr"/>
       <c r="G77" t="inlineStr">
         <is>
@@ -8814,10 +9822,7 @@
           <t>linkedin</t>
         </is>
       </c>
-      <c r="E78">
-        <f>HYPERLINK("https://www.linkedin.com/jobs/view/4373224818", "https://www.linkedin.com/jobs/view/4373224818")</f>
-        <v/>
-      </c>
+      <c r="E78" t="inlineStr"/>
       <c r="F78" t="inlineStr"/>
       <c r="G78" t="inlineStr">
         <is>
@@ -8878,10 +9883,7 @@
           <t>linkedin</t>
         </is>
       </c>
-      <c r="E79">
-        <f>HYPERLINK("https://www.linkedin.com/jobs/view/4373227614", "https://www.linkedin.com/jobs/view/4373227614")</f>
-        <v/>
-      </c>
+      <c r="E79" t="inlineStr"/>
       <c r="F79" t="inlineStr"/>
       <c r="G79" t="inlineStr">
         <is>
@@ -8942,10 +9944,7 @@
           <t>linkedin</t>
         </is>
       </c>
-      <c r="E80">
-        <f>HYPERLINK("https://www.linkedin.com/jobs/view/4373222990", "https://www.linkedin.com/jobs/view/4373222990")</f>
-        <v/>
-      </c>
+      <c r="E80" t="inlineStr"/>
       <c r="F80" t="inlineStr"/>
       <c r="G80" t="inlineStr">
         <is>
@@ -9006,10 +10005,7 @@
           <t>linkedin</t>
         </is>
       </c>
-      <c r="E81">
-        <f>HYPERLINK("https://www.linkedin.com/jobs/view/4373222998", "https://www.linkedin.com/jobs/view/4373222998")</f>
-        <v/>
-      </c>
+      <c r="E81" t="inlineStr"/>
       <c r="F81" t="inlineStr"/>
       <c r="G81" t="inlineStr">
         <is>
@@ -9070,10 +10066,7 @@
           <t>linkedin</t>
         </is>
       </c>
-      <c r="E82">
-        <f>HYPERLINK("https://www.linkedin.com/jobs/view/4373236058", "https://www.linkedin.com/jobs/view/4373236058")</f>
-        <v/>
-      </c>
+      <c r="E82" t="inlineStr"/>
       <c r="F82" t="inlineStr"/>
       <c r="G82" t="inlineStr">
         <is>
@@ -9131,17 +10124,17 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>li-4327208014</t>
+          <t>li-4373211737</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Analytics Engineer</t>
+          <t>Data Engineer</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Ibotta</t>
+          <t>Wiraa</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
@@ -9149,100 +10142,11 @@
           <t>linkedin</t>
         </is>
       </c>
-      <c r="E83">
-        <f>HYPERLINK("https://www.linkedin.com/jobs/view/4327208014", "https://www.linkedin.com/jobs/view/4327208014")</f>
-        <v/>
-      </c>
+      <c r="E83" t="inlineStr"/>
       <c r="F83" t="inlineStr"/>
-      <c r="G83" t="inlineStr">
-        <is>
-          <t>Denver, CO</t>
-        </is>
-      </c>
+      <c r="G83" t="inlineStr"/>
       <c r="H83" t="inlineStr"/>
       <c r="I83" t="inlineStr">
-        <is>
-          <t>Ibotta is seeking an
- **Analytics Engineer** 
- to join our innovative Core Data \&amp; Analytics team and contribute to our mission to Make Every Purchase Rewarding. Our growing Core Data \&amp; Analytics team provides high\-quality, on\-time analytics products and services across all business areas and teams within Ibotta. We achieve this by offering expert guidance, sharing specialized knowledge, promoting data\-driven solutions, and overseeing mission\-critical data science projects that impact the entire organization.
- This position is located in Denver, Colorado, as a hybrid position requiring 3 days in office (Tuesday, Wednesday, and Thursday). Candidates must live in the United States.
-**What you will be doing:**
-* Helping us organize and optimize our data for analysis
-* Collaborate with other Analytics Engineers and Platform Engineers to understand our data models and translate them into scalable data solutions
-* Implement and utilize engineering best practices and methods to deploy and maintain quality, curated data sets using Airflow, including automated alerting and anomaly detection into data flows to ensure data quality and integrity
-* Work across our full technology stack (Databricks, Spark, Command Line, Airflow, GitHub, Python, Monte Carlo, etc) to develop and maintain these datasets
-* Building UI and automation tools to enable data democratization throughout the company
-* Lead large, complex task force projects that require cross\-functional input across various teams
-* Managing new data requirements and developing solutions that minimize technical debt creation
-* Embrace and uphold Ibotta’s Core Values: Integrity, Boldness, Ownership, Teamwork, Transparency, \&amp; A good idea can come from anywhere
-**What we are looking for:**
-* 2\+ years of practical work experience in a data engineering role supporting an analytics team or equivalent experience as an analytics engineer
-* Bachelor’s degree in Computer Science, Engineering, Analytics, or a related field required
-* Working knowledge and some practical experience with some or all of the following:
-+ End\-to\-end analytics automation, data pipelines, ETL/ELT processes, and tools (AWS Glue, DBT, etc.)
-+ AWS EcoSystem and cloud\-based data warehouse and architecture
-+ Airflow, DataBricks, Git, Monte Carlo
-+ Multiple languages and frameworks (Python, Scala, strong SQL, Spark, Command Line) highly preferred
-+ Development in a modern BI/data visualization platform (Looker, Tableau, etc.)
-+ Event\-driven architectures and platforms are a strong plus
-* An ability to develop solutions by applying data quality principles
-* Ability to think creatively, provide thoughtful insights, and solve problems to answer business questions using data
-* Collaboration with SMEs to understand the business context of the data
-* Experience identifying and troubleshooting data anomalies and pipeline issues
-* Exposure to managing and updating cluster configurations to ensure workflow operation
-* Ownership of data throughout its lifecycle
-* Excellent oral and written communication skills
-**What we are looking for:**
- You…
-* are proactive, collaborative, and driven to solve hard problems while respecting diverse perspectives in a dynamic, fast\-paced environment
-* are an intellectually curious, conceptual thinker who uses creative problem\-solving skills to work with other engineers and analytics stakeholders to challenge yourself and develop as an engineer
-* are a detailed\-oriented team player with an ownership mindset who develops technical solutions that apply data quality principles
-* work collaboratively throughout the organization to drive towards common goals and understand the business context of data
-* understand that delivering products incrementally helps provide more value to the business, and testing your code is one of the most important aspects of engineering
-* trust your teammates, and embrace healthy conflict and debate \- not afraid to voice your opinions but okay with not always being right
-**About Ibotta ("I bought a...")**
- Ibotta (NYSE: IBTA) is a leading performance marketing platform allowing brands to deliver digital promotions to over 200 million consumers through a network of publishers called the Ibotta Performance Network (IPN). The IPN allows marketers to influence what people buy, and where and how often they shop – all while paying only when their campaigns directly result in a sale. American shoppers have earned over $1\.8 billion through the IPN since 2012\. The largest tech IPO in history to come out of Colorado, Ibotta is headquartered in Denver, and is continually listed as a top place to work by The Denver Post and Inc. Magazine.
- To learn more about what our Tech teams are doing day to day, visit Building Ibotta on Medium.com.
-**Additional Details:**
-* This position is located in Denver, CO and includes competitive pay, flexible time off, benefits package (including medical, dental, vision) Employee Stock Purchase Program, and 401k match. Denver office perks include paid parking, snacks, and occasional meals.
-* Base compensation range: $111,000 \- $127,000\. Equity is included in overall compensation package. This compensation range is specific to the United States labor market and may be adjusted based on actual experience.
-* Ibotta is an Equal Opportunity Employer. Ibotta’s employment decisions are made without regard of race, color, religion, national origin, age, sex, marital status, ancestry, physical or mental disability, veteran status, gender identity, sexual orientation, or any other legally protected status.
-* Applicants must be currently authorized to work in the United States on a full\-time basis.
-* Applicants are accepted until the position is filled.
-* For the security of our employees and the business, all employees are responsible for the secure handling of data in accordance with our security policies, identifying and reporting phishing attempts, as well as reporting security incidents to the proper channels.
- \#BI\-Hybrid</t>
-        </is>
-      </c>
-    </row>
-    <row r="84">
-      <c r="A84" t="inlineStr">
-        <is>
-          <t>li-4373211737</t>
-        </is>
-      </c>
-      <c r="B84" t="inlineStr">
-        <is>
-          <t>Data Engineer</t>
-        </is>
-      </c>
-      <c r="C84" t="inlineStr">
-        <is>
-          <t>Wiraa</t>
-        </is>
-      </c>
-      <c r="D84" t="inlineStr">
-        <is>
-          <t>linkedin</t>
-        </is>
-      </c>
-      <c r="E84">
-        <f>HYPERLINK("https://www.linkedin.com/jobs/view/4373211737", "https://www.linkedin.com/jobs/view/4373211737")</f>
-        <v/>
-      </c>
-      <c r="F84" t="inlineStr"/>
-      <c r="G84" t="inlineStr"/>
-      <c r="H84" t="inlineStr"/>
-      <c r="I84" t="inlineStr">
         <is>
           <t>**About The Company**
  Join the Future of Commerce with Whatnot! Whatnot is the largest live shopping platform operating across North America and Europe, revolutionizing the way people buy, sell, and discover their passions. By seamlessly blending community engagement, entertainment, and e\-commerce, Whatnot offers a unique marketplace experience that caters to a diverse range of interests, including fashion, beauty, electronics, collectibles such as trading cards and comic books, and even live plants. The platform is designed to foster a vibrant community where users can participate in live auctions and connect over shared interests. With a strong emphasis on innovation and a values\-driven culture, Whatnot operates as a remote co\-located team with hubs in the US, UK, Germany, Ireland, and Poland, dedicated to building the future of online marketplaces. As one of the fastest\-growing marketplaces, Whatnot is committed to enabling individuals to turn their passions into thriving businesses and bringing people together through commerce.
@@ -9277,38 +10181,32 @@
         </is>
       </c>
     </row>
-    <row r="85">
-      <c r="A85" t="inlineStr">
+    <row r="84">
+      <c r="A84" t="inlineStr">
         <is>
           <t>li-4373230126</t>
         </is>
       </c>
-      <c r="B85" t="inlineStr">
+      <c r="B84" t="inlineStr">
         <is>
           <t>Data Engineer I/II</t>
         </is>
       </c>
-      <c r="C85" t="inlineStr">
+      <c r="C84" t="inlineStr">
         <is>
           <t>Wiraa</t>
         </is>
       </c>
-      <c r="D85" t="inlineStr">
+      <c r="D84" t="inlineStr">
         <is>
           <t>linkedin</t>
         </is>
       </c>
-      <c r="E85">
-        <f>HYPERLINK("https://www.linkedin.com/jobs/view/4373230126", "https://www.linkedin.com/jobs/view/4373230126")</f>
-        <v/>
-      </c>
-      <c r="F85">
-        <f>HYPERLINK("https://www.wiraa.com/job-description/usF7EA4A54A7A1763AEC83F9DE8CF9C92D?source=Linkedin&amp;urlHash=3_1Y", "https://www.wiraa.com/job-description/usF7EA4A54A7A1763AEC83F9DE8CF9C92D?source=Linkedin&amp;urlHash=3_1Y")</f>
-        <v/>
-      </c>
-      <c r="G85" t="inlineStr"/>
-      <c r="H85" t="inlineStr"/>
-      <c r="I85" t="inlineStr">
+      <c r="E84" t="inlineStr"/>
+      <c r="F84" t="inlineStr"/>
+      <c r="G84" t="inlineStr"/>
+      <c r="H84" t="inlineStr"/>
+      <c r="I84" t="inlineStr">
         <is>
           <t>**About The Company**
  BNSF Railway is one of the largest freight railroads in the United States, operating across 28 western states and extending into three Canadian provinces. The company is committed to safety, inclusion, and excellence, playing a vital role in transporting essential products and materials that support communities nationwide and globally. As a member of our team, you will contribute to the movement of goods that feed, clothe, supply, and power communities, ensuring the seamless flow of commerce and daily life. BNSF is dedicated to fostering a culture of diversity, innovation, and continuous improvement, making it an ideal environment for professionals seeking impactful careers in the transportation sector.
@@ -9351,39 +10249,36 @@
         </is>
       </c>
     </row>
-    <row r="86">
-      <c r="A86" t="inlineStr">
+    <row r="85">
+      <c r="A85" t="inlineStr">
         <is>
           <t>li-4323555261</t>
         </is>
       </c>
-      <c r="B86" t="inlineStr">
+      <c r="B85" t="inlineStr">
         <is>
           <t>Data Engineer</t>
         </is>
       </c>
-      <c r="C86" t="inlineStr">
+      <c r="C85" t="inlineStr">
         <is>
           <t>Orveon Global</t>
         </is>
       </c>
-      <c r="D86" t="inlineStr">
+      <c r="D85" t="inlineStr">
         <is>
           <t>linkedin</t>
         </is>
       </c>
-      <c r="E86">
-        <f>HYPERLINK("https://www.linkedin.com/jobs/view/4323555261", "https://www.linkedin.com/jobs/view/4323555261")</f>
-        <v/>
-      </c>
-      <c r="F86" t="inlineStr"/>
-      <c r="G86" t="inlineStr">
+      <c r="E85" t="inlineStr"/>
+      <c r="F85" t="inlineStr"/>
+      <c r="G85" t="inlineStr">
         <is>
           <t>Columbus, OH</t>
         </is>
       </c>
-      <c r="H86" t="inlineStr"/>
-      <c r="I86" t="inlineStr">
+      <c r="H85" t="inlineStr"/>
+      <c r="I85" t="inlineStr">
         <is>
           <t>**About Us**
  Orveon is a new kind of beauty company launched in December 2021 when we acquired our three iconic brands \- bareMinerals, BUXOM, and Laura Mercier. Operating in 40\+ countries, we're a truly global business. Our headquarters are in New York, with additional locations in major cities worldwide.
@@ -9435,35 +10330,32 @@
         </is>
       </c>
     </row>
-    <row r="87">
-      <c r="A87" t="inlineStr">
+    <row r="86">
+      <c r="A86" t="inlineStr">
         <is>
           <t>li-4373226545</t>
         </is>
       </c>
-      <c r="B87" t="inlineStr">
+      <c r="B86" t="inlineStr">
         <is>
           <t>Data Engineer</t>
         </is>
       </c>
-      <c r="C87" t="inlineStr">
+      <c r="C86" t="inlineStr">
         <is>
           <t>Hirenza</t>
         </is>
       </c>
-      <c r="D87" t="inlineStr">
+      <c r="D86" t="inlineStr">
         <is>
           <t>linkedin</t>
         </is>
       </c>
-      <c r="E87">
-        <f>HYPERLINK("https://www.linkedin.com/jobs/view/4373226545", "https://www.linkedin.com/jobs/view/4373226545")</f>
-        <v/>
-      </c>
-      <c r="F87" t="inlineStr"/>
-      <c r="G87" t="inlineStr"/>
-      <c r="H87" t="inlineStr"/>
-      <c r="I87" t="inlineStr">
+      <c r="E86" t="inlineStr"/>
+      <c r="F86" t="inlineStr"/>
+      <c r="G86" t="inlineStr"/>
+      <c r="H86" t="inlineStr"/>
+      <c r="I86" t="inlineStr">
         <is>
           <t>**About The Company**
  PSA Ventures is a dynamic and innovative organization dedicated to leveraging cutting\-edge technology solutions to drive business growth and operational excellence. Our company specializes in data\-driven strategies, providing clients with actionable insights and tailored analytics solutions across various industries. With a focus on fostering a collaborative and inclusive work environment, PSA Ventures is committed to empowering its employees to excel and stay ahead in the rapidly evolving technology landscape. We prioritize integrity, innovation, and excellence in everything we do, ensuring our clients receive the highest quality services and solutions.
@@ -9496,42 +10388,36 @@
         </is>
       </c>
     </row>
-    <row r="88">
-      <c r="A88" t="inlineStr">
+    <row r="87">
+      <c r="A87" t="inlineStr">
         <is>
           <t>li-4373221899</t>
         </is>
       </c>
-      <c r="B88" t="inlineStr">
+      <c r="B87" t="inlineStr">
         <is>
           <t>Data Engineer</t>
         </is>
       </c>
-      <c r="C88" t="inlineStr">
+      <c r="C87" t="inlineStr">
         <is>
           <t>ThinkTek</t>
         </is>
       </c>
-      <c r="D88" t="inlineStr">
+      <c r="D87" t="inlineStr">
         <is>
           <t>linkedin</t>
         </is>
       </c>
-      <c r="E88">
-        <f>HYPERLINK("https://www.linkedin.com/jobs/view/4373221899", "https://www.linkedin.com/jobs/view/4373221899")</f>
-        <v/>
-      </c>
-      <c r="F88">
-        <f>HYPERLINK("https://www.adzuna.com/details/5594358526?v=A9949281D23E3FFFCD7815B9FAD8345BBDF8CF4F&amp;ccd=8c398121578b7184035be02d11eccdee&amp;frd=a66b8538f4c016a663b2fa45a5d8eb5d&amp;r=21262857&amp;utm_source=linkedin7&amp;utm_medium=organic&amp;chnlid=1931&amp;title=Data%20Engineer&amp;a=e&amp;urlHash=rO4_", "https://www.adzuna.com/details/5594358526?v=A9949281D23E3FFFCD7815B9FAD8345BBDF8CF4F&amp;ccd=8c398121578b7184035be02d11eccdee&amp;frd=a66b8538f4c016a663b2fa45a5d8eb5d&amp;r=21262857&amp;utm_source=linkedin7&amp;utm_medium=organic&amp;chnlid=1931&amp;title=Data%20Engineer&amp;a=e&amp;urlHash=rO4_")</f>
-        <v/>
-      </c>
-      <c r="G88" t="inlineStr">
+      <c r="E87" t="inlineStr"/>
+      <c r="F87" t="inlineStr"/>
+      <c r="G87" t="inlineStr">
         <is>
           <t>Fairfax, VA</t>
         </is>
       </c>
-      <c r="H88" t="inlineStr"/>
-      <c r="I88" t="inlineStr">
+      <c r="H87" t="inlineStr"/>
+      <c r="I87" t="inlineStr">
         <is>
           <t>**Who We Are**
  ThinkTek LLC is a fast\-growing Certified SBA 8(a) and Service\-Disabled Veteran\-Owned Small Business (SDVOSB). We specialize in providing management and technology consulting services to support the business and technology modernization efforts of the Federal Government. ThinkTek was formed with the specific purpose of providing clients tailored solutions in Program \&amp; Project Management, Strategic Planning, and IT Services.
@@ -9568,38 +10454,32 @@
         </is>
       </c>
     </row>
-    <row r="89">
-      <c r="A89" t="inlineStr">
+    <row r="88">
+      <c r="A88" t="inlineStr">
         <is>
           <t>li-4373219843</t>
         </is>
       </c>
-      <c r="B89" t="inlineStr">
+      <c r="B88" t="inlineStr">
         <is>
           <t>Data Engineer</t>
         </is>
       </c>
-      <c r="C89" t="inlineStr">
+      <c r="C88" t="inlineStr">
         <is>
           <t>Best Job Tool</t>
         </is>
       </c>
-      <c r="D89" t="inlineStr">
+      <c r="D88" t="inlineStr">
         <is>
           <t>linkedin</t>
         </is>
       </c>
-      <c r="E89">
-        <f>HYPERLINK("https://www.linkedin.com/jobs/view/4373219843", "https://www.linkedin.com/jobs/view/4373219843")</f>
-        <v/>
-      </c>
-      <c r="F89">
-        <f>HYPERLINK("https://www.hirecrap.com/job-description-usj/7533732185383542420?src=LinkedIn&amp;urlHash=mi4m", "https://www.hirecrap.com/job-description-usj/7533732185383542420?src=LinkedIn&amp;urlHash=mi4m")</f>
-        <v/>
-      </c>
-      <c r="G89" t="inlineStr"/>
-      <c r="H89" t="inlineStr"/>
-      <c r="I89" t="inlineStr">
+      <c r="E88" t="inlineStr"/>
+      <c r="F88" t="inlineStr"/>
+      <c r="G88" t="inlineStr"/>
+      <c r="H88" t="inlineStr"/>
+      <c r="I88" t="inlineStr">
         <is>
           <t>**About The Company**
  Fynetra is a forward\-thinking technology company dedicated to delivering innovative solutions that drive digital transformation across various industries. With a strong focus on customer\-centric approaches, Fynetra leverages cutting\-edge technologies such as artificial intelligence, cloud computing, and data analytics to help businesses optimize their operations and achieve sustainable growth. Our commitment to excellence, integrity, and continuous improvement has established us as a trusted partner for organizations seeking to stay ahead in an ever\-evolving digital landscape.
@@ -9628,35 +10508,32 @@
         </is>
       </c>
     </row>
-    <row r="90">
-      <c r="A90" t="inlineStr">
+    <row r="89">
+      <c r="A89" t="inlineStr">
         <is>
           <t>li-4373217644</t>
         </is>
       </c>
-      <c r="B90" t="inlineStr">
+      <c r="B89" t="inlineStr">
         <is>
           <t>Senior Data Engineer</t>
         </is>
       </c>
-      <c r="C90" t="inlineStr">
+      <c r="C89" t="inlineStr">
         <is>
           <t>James Search Group</t>
         </is>
       </c>
-      <c r="D90" t="inlineStr">
+      <c r="D89" t="inlineStr">
         <is>
           <t>linkedin</t>
         </is>
       </c>
-      <c r="E90">
-        <f>HYPERLINK("https://www.linkedin.com/jobs/view/4373217644", "https://www.linkedin.com/jobs/view/4373217644")</f>
-        <v/>
-      </c>
-      <c r="F90" t="inlineStr"/>
-      <c r="G90" t="inlineStr"/>
-      <c r="H90" t="inlineStr"/>
-      <c r="I90" t="inlineStr">
+      <c r="E89" t="inlineStr"/>
+      <c r="F89" t="inlineStr"/>
+      <c r="G89" t="inlineStr"/>
+      <c r="H89" t="inlineStr"/>
+      <c r="I89" t="inlineStr">
         <is>
           <t>**Senior Data Engineer (P\&amp;C Insurance)** 
  Fully Remote \| Full\-Time
@@ -9717,39 +10594,36 @@
         </is>
       </c>
     </row>
-    <row r="91">
-      <c r="A91" t="inlineStr">
+    <row r="90">
+      <c r="A90" t="inlineStr">
         <is>
           <t>li-4355481816</t>
         </is>
       </c>
-      <c r="B91" t="inlineStr">
+      <c r="B90" t="inlineStr">
         <is>
           <t>(Senior) Data Engineer</t>
         </is>
       </c>
-      <c r="C91" t="inlineStr">
+      <c r="C90" t="inlineStr">
         <is>
           <t>Flagship Pioneering</t>
         </is>
       </c>
-      <c r="D91" t="inlineStr">
+      <c r="D90" t="inlineStr">
         <is>
           <t>linkedin</t>
         </is>
       </c>
-      <c r="E91">
-        <f>HYPERLINK("https://www.linkedin.com/jobs/view/4355481816", "https://www.linkedin.com/jobs/view/4355481816")</f>
-        <v/>
-      </c>
-      <c r="F91" t="inlineStr"/>
-      <c r="G91" t="inlineStr">
+      <c r="E90" t="inlineStr"/>
+      <c r="F90" t="inlineStr"/>
+      <c r="G90" t="inlineStr">
         <is>
           <t>Boston, MA</t>
         </is>
       </c>
-      <c r="H91" t="inlineStr"/>
-      <c r="I91" t="inlineStr">
+      <c r="H90" t="inlineStr"/>
+      <c r="I90" t="inlineStr">
         <is>
           <t>**About ProFound Therapeutics**
  ProFound Therapeutics is pioneering the discovery of the expanded human proteome to unlock a new universe of potential therapeutics. By integrating multi\-omics, advanced computation, and translational biology, we aim to reveal and characterize thousands of previously uncharted proteins and systematically explore their role in health and disease.
@@ -9797,39 +10671,36 @@
         </is>
       </c>
     </row>
-    <row r="92">
-      <c r="A92" t="inlineStr">
+    <row r="91">
+      <c r="A91" t="inlineStr">
         <is>
           <t>li-4373213998</t>
         </is>
       </c>
-      <c r="B92" t="inlineStr">
+      <c r="B91" t="inlineStr">
         <is>
           <t>Cloud Data Engineer@ Nebraska</t>
         </is>
       </c>
-      <c r="C92" t="inlineStr">
+      <c r="C91" t="inlineStr">
         <is>
           <t>SohanIT Inc</t>
         </is>
       </c>
-      <c r="D92" t="inlineStr">
+      <c r="D91" t="inlineStr">
         <is>
           <t>linkedin</t>
         </is>
       </c>
-      <c r="E92">
-        <f>HYPERLINK("https://www.linkedin.com/jobs/view/4373213998", "https://www.linkedin.com/jobs/view/4373213998")</f>
-        <v/>
-      </c>
-      <c r="F92" t="inlineStr"/>
-      <c r="G92" t="inlineStr">
+      <c r="E91" t="inlineStr"/>
+      <c r="F91" t="inlineStr"/>
+      <c r="G91" t="inlineStr">
         <is>
           <t>Nebraska, United States</t>
         </is>
       </c>
-      <c r="H92" t="inlineStr"/>
-      <c r="I92" t="inlineStr">
+      <c r="H91" t="inlineStr"/>
+      <c r="I91" t="inlineStr">
         <is>
           <t>\*\*\*\*\*Direct Client Requirement\*\*\*\*\*
  All Openings
@@ -9874,39 +10745,36 @@
         </is>
       </c>
     </row>
-    <row r="93">
-      <c r="A93" t="inlineStr">
+    <row r="92">
+      <c r="A92" t="inlineStr">
         <is>
           <t>li-4363455869</t>
         </is>
       </c>
-      <c r="B93" t="inlineStr">
+      <c r="B92" t="inlineStr">
         <is>
           <t>Senior Analytics Engineer</t>
         </is>
       </c>
-      <c r="C93" t="inlineStr">
+      <c r="C92" t="inlineStr">
         <is>
           <t>Khan Academy</t>
         </is>
       </c>
-      <c r="D93" t="inlineStr">
+      <c r="D92" t="inlineStr">
         <is>
           <t>linkedin</t>
         </is>
       </c>
-      <c r="E93">
-        <f>HYPERLINK("https://www.linkedin.com/jobs/view/4363455869", "https://www.linkedin.com/jobs/view/4363455869")</f>
-        <v/>
-      </c>
-      <c r="F93" t="inlineStr"/>
-      <c r="G93" t="inlineStr">
+      <c r="E92" t="inlineStr"/>
+      <c r="F92" t="inlineStr"/>
+      <c r="G92" t="inlineStr">
         <is>
           <t>Mountain View, CA</t>
         </is>
       </c>
-      <c r="H93" t="inlineStr"/>
-      <c r="I93" t="inlineStr">
+      <c r="H92" t="inlineStr"/>
+      <c r="I92" t="inlineStr">
         <is>
           <t>**About Khan Academy**
  Khan Academy is a nonprofit with the mission to deliver a free, world\-class education to anyone, anywhere. Our proven learning platform offers free, high\-quality supplemental learning content and practice that cover Pre\-K \- 12th grade and early college core academic subjects, focusing on math and science. We have over 181 million registered learners globally and are committed to improving learning outcomes for students worldwide, focusing on learners in historically under\-resourced communities.
@@ -9992,35 +10860,32 @@
         </is>
       </c>
     </row>
-    <row r="94">
-      <c r="A94" t="inlineStr">
+    <row r="93">
+      <c r="A93" t="inlineStr">
         <is>
           <t>li-4372093669</t>
         </is>
       </c>
-      <c r="B94" t="inlineStr">
+      <c r="B93" t="inlineStr">
         <is>
           <t>Data Engineer III</t>
         </is>
       </c>
-      <c r="C94" t="inlineStr">
+      <c r="C93" t="inlineStr">
         <is>
           <t>RemoteHunter</t>
         </is>
       </c>
-      <c r="D94" t="inlineStr">
+      <c r="D93" t="inlineStr">
         <is>
           <t>linkedin</t>
         </is>
       </c>
-      <c r="E94">
-        <f>HYPERLINK("https://www.linkedin.com/jobs/view/4372093669", "https://www.linkedin.com/jobs/view/4372093669")</f>
-        <v/>
-      </c>
-      <c r="F94" t="inlineStr"/>
-      <c r="G94" t="inlineStr"/>
-      <c r="H94" t="inlineStr"/>
-      <c r="I94" t="inlineStr">
+      <c r="E93" t="inlineStr"/>
+      <c r="F93" t="inlineStr"/>
+      <c r="G93" t="inlineStr"/>
+      <c r="H93" t="inlineStr"/>
+      <c r="I93" t="inlineStr">
         <is>
           <t>About the Opportunity:
  The Data Engineer III is responsible for building and maintaining robust data pipelines and models, overseeing a broad scope of ETL infrastructure and databases. This role enables accurate and timely access to data across the organization by simplifying and centralizing a complex ecosystem, providing trustworthy, analytic\-ready resources for various business units. It involves deep collaboration with stakeholders in Engineering, Analytics, Operations, Finance, Marketing, and Customer Service to create a dependable data environment and drive measurable business impact through data.
@@ -10064,42 +10929,36 @@
         </is>
       </c>
     </row>
-    <row r="95">
-      <c r="A95" t="inlineStr">
+    <row r="94">
+      <c r="A94" t="inlineStr">
         <is>
           <t>li-4373235173</t>
         </is>
       </c>
-      <c r="B95" t="inlineStr">
+      <c r="B94" t="inlineStr">
         <is>
           <t>Senior Data Engineer (Remote)</t>
         </is>
       </c>
-      <c r="C95" t="inlineStr">
+      <c r="C94" t="inlineStr">
         <is>
           <t>Jobgether</t>
         </is>
       </c>
-      <c r="D95" t="inlineStr">
+      <c r="D94" t="inlineStr">
         <is>
           <t>linkedin</t>
         </is>
       </c>
-      <c r="E95">
-        <f>HYPERLINK("https://www.linkedin.com/jobs/view/4373235173", "https://www.linkedin.com/jobs/view/4373235173")</f>
-        <v/>
-      </c>
-      <c r="F95">
-        <f>HYPERLINK("https://jobs.lever.co/jobgether/6015297e-8e68-498e-a2c7-efc73fc53153/apply?source=LinkedIn&amp;urlHash=dSWz", "https://jobs.lever.co/jobgether/6015297e-8e68-498e-a2c7-efc73fc53153/apply?source=LinkedIn&amp;urlHash=dSWz")</f>
-        <v/>
-      </c>
-      <c r="G95" t="inlineStr">
+      <c r="E94" t="inlineStr"/>
+      <c r="F94" t="inlineStr"/>
+      <c r="G94" t="inlineStr">
         <is>
           <t>Massachusetts, United States</t>
         </is>
       </c>
-      <c r="H95" t="inlineStr"/>
-      <c r="I95" t="inlineStr">
+      <c r="H94" t="inlineStr"/>
+      <c r="I94" t="inlineStr">
         <is>
           <t>This position is posted by Jobgether on behalf of a partner company. We are currently looking for a Data Engineer. In this role, you will play a crucial part in constructing robust data pipelines that serve as the backbone for internal business analytics. Collaborating closely with senior engineers, you will ensure the seamless ingestion and preparation of data from various sources, elevating data quality for analysis. Your contributions will directly influence critical decision\-making processes, providing leaders with necessary insights efficiently. This role demands a commitment to excellence, allowing you to make a real impact in a fast\-paced, results\-oriented environment.
 **Accountabilities**
@@ -10131,39 +10990,36 @@
         </is>
       </c>
     </row>
-    <row r="96">
-      <c r="A96" t="inlineStr">
+    <row r="95">
+      <c r="A95" t="inlineStr">
         <is>
           <t>li-4371449107</t>
         </is>
       </c>
-      <c r="B96" t="inlineStr">
+      <c r="B95" t="inlineStr">
         <is>
           <t>Data Engineer/Snowflake Architect</t>
         </is>
       </c>
-      <c r="C96" t="inlineStr">
+      <c r="C95" t="inlineStr">
         <is>
           <t>Aezion, Inc</t>
         </is>
       </c>
-      <c r="D96" t="inlineStr">
+      <c r="D95" t="inlineStr">
         <is>
           <t>linkedin</t>
         </is>
       </c>
-      <c r="E96">
-        <f>HYPERLINK("https://www.linkedin.com/jobs/view/4371449107", "https://www.linkedin.com/jobs/view/4371449107")</f>
-        <v/>
-      </c>
-      <c r="F96" t="inlineStr"/>
-      <c r="G96" t="inlineStr">
+      <c r="E95" t="inlineStr"/>
+      <c r="F95" t="inlineStr"/>
+      <c r="G95" t="inlineStr">
         <is>
           <t>Frisco, TX</t>
         </is>
       </c>
-      <c r="H96" t="inlineStr"/>
-      <c r="I96" t="inlineStr">
+      <c r="H95" t="inlineStr"/>
+      <c r="I95" t="inlineStr">
         <is>
           <t>**Title:** 
 **Data Engineer/Snowflake Architect** 
@@ -10205,35 +11061,32 @@
         </is>
       </c>
     </row>
-    <row r="97">
-      <c r="A97" t="inlineStr">
+    <row r="96">
+      <c r="A96" t="inlineStr">
         <is>
           <t>li-4372076748</t>
         </is>
       </c>
-      <c r="B97" t="inlineStr">
+      <c r="B96" t="inlineStr">
         <is>
           <t>Analytics Engineer</t>
         </is>
       </c>
-      <c r="C97" t="inlineStr">
+      <c r="C96" t="inlineStr">
         <is>
           <t>RemoteHunter</t>
         </is>
       </c>
-      <c r="D97" t="inlineStr">
+      <c r="D96" t="inlineStr">
         <is>
           <t>linkedin</t>
         </is>
       </c>
-      <c r="E97">
-        <f>HYPERLINK("https://www.linkedin.com/jobs/view/4372076748", "https://www.linkedin.com/jobs/view/4372076748")</f>
-        <v/>
-      </c>
-      <c r="F97" t="inlineStr"/>
-      <c r="G97" t="inlineStr"/>
-      <c r="H97" t="inlineStr"/>
-      <c r="I97" t="inlineStr">
+      <c r="E96" t="inlineStr"/>
+      <c r="F96" t="inlineStr"/>
+      <c r="G96" t="inlineStr"/>
+      <c r="H96" t="inlineStr"/>
+      <c r="I96" t="inlineStr">
         <is>
           <t>About the Opportunity:
  A United States based Analytics Engineer is needed to support reporting, ad\-hoc analysis, and analytics development across the organization while helping evolve the data platform over time. This role bridges data engineering and business functions, managing day\-to\-day analytics needs such as Power BI dashboards, ad\-hoc reporting, and SQL development, with growth into data modeling and advanced analytics including machine learning. The role collaborates closely with a Senior Solutions Engineer focused on data ingestion and integrations.
@@ -10277,39 +11130,36 @@
         </is>
       </c>
     </row>
-    <row r="98">
-      <c r="A98" t="inlineStr">
+    <row r="97">
+      <c r="A97" t="inlineStr">
         <is>
           <t>li-4373239085</t>
         </is>
       </c>
-      <c r="B98" t="inlineStr">
+      <c r="B97" t="inlineStr">
         <is>
           <t>Sr. Data Engineer - REMOTE</t>
         </is>
       </c>
-      <c r="C98" t="inlineStr">
+      <c r="C97" t="inlineStr">
         <is>
           <t>Jobgether</t>
         </is>
       </c>
-      <c r="D98" t="inlineStr">
+      <c r="D97" t="inlineStr">
         <is>
           <t>linkedin</t>
         </is>
       </c>
-      <c r="E98">
-        <f>HYPERLINK("https://www.linkedin.com/jobs/view/4373239085", "https://www.linkedin.com/jobs/view/4373239085")</f>
-        <v/>
-      </c>
-      <c r="F98" t="inlineStr"/>
-      <c r="G98" t="inlineStr">
+      <c r="E97" t="inlineStr"/>
+      <c r="F97" t="inlineStr"/>
+      <c r="G97" t="inlineStr">
         <is>
           <t>Indiana, United States</t>
         </is>
       </c>
-      <c r="H98" t="inlineStr"/>
-      <c r="I98" t="inlineStr">
+      <c r="H97" t="inlineStr"/>
+      <c r="I97" t="inlineStr">
         <is>
           <t>This position is posted by Jobgether on behalf of a partner company. We are currently looking for a Data Engineer. In this role, you will play a crucial part in constructing robust data pipelines that serve as the backbone for internal business analytics. Collaborating closely with senior engineers, you will ensure the seamless ingestion and preparation of data from various sources, elevating data quality for analysis. Your contributions will directly influence critical decision\-making processes, providing leaders with necessary insights efficiently. This role demands a commitment to excellence, allowing you to make a real impact in a fast\-paced, results\-oriented environment.
 **Accountabilities**
@@ -10341,39 +11191,36 @@
         </is>
       </c>
     </row>
-    <row r="99">
-      <c r="A99" t="inlineStr">
+    <row r="98">
+      <c r="A98" t="inlineStr">
         <is>
           <t>li-4373242003</t>
         </is>
       </c>
-      <c r="B99" t="inlineStr">
+      <c r="B98" t="inlineStr">
         <is>
           <t>Remote Sr Data Engineer</t>
         </is>
       </c>
-      <c r="C99" t="inlineStr">
+      <c r="C98" t="inlineStr">
         <is>
           <t>Jobgether</t>
         </is>
       </c>
-      <c r="D99" t="inlineStr">
+      <c r="D98" t="inlineStr">
         <is>
           <t>linkedin</t>
         </is>
       </c>
-      <c r="E99">
-        <f>HYPERLINK("https://www.linkedin.com/jobs/view/4373242003", "https://www.linkedin.com/jobs/view/4373242003")</f>
-        <v/>
-      </c>
-      <c r="F99" t="inlineStr"/>
-      <c r="G99" t="inlineStr">
+      <c r="E98" t="inlineStr"/>
+      <c r="F98" t="inlineStr"/>
+      <c r="G98" t="inlineStr">
         <is>
           <t>Michigan, United States</t>
         </is>
       </c>
-      <c r="H99" t="inlineStr"/>
-      <c r="I99" t="inlineStr">
+      <c r="H98" t="inlineStr"/>
+      <c r="I98" t="inlineStr">
         <is>
           <t>This position is posted by Jobgether on behalf of a partner company. We are currently looking for a Data Engineer. In this role, you will play a crucial part in constructing robust data pipelines that serve as the backbone for internal business analytics. Collaborating closely with senior engineers, you will ensure the seamless ingestion and preparation of data from various sources, elevating data quality for analysis. Your contributions will directly influence critical decision\-making processes, providing leaders with necessary insights efficiently. This role demands a commitment to excellence, allowing you to make a real impact in a fast\-paced, results\-oriented environment.
 **Accountabilities**
@@ -10405,39 +11252,36 @@
         </is>
       </c>
     </row>
-    <row r="100">
-      <c r="A100" t="inlineStr">
+    <row r="99">
+      <c r="A99" t="inlineStr">
         <is>
           <t>li-4373227600</t>
         </is>
       </c>
-      <c r="B100" t="inlineStr">
+      <c r="B99" t="inlineStr">
         <is>
           <t>Data Engineer III</t>
         </is>
       </c>
-      <c r="C100" t="inlineStr">
+      <c r="C99" t="inlineStr">
         <is>
           <t>Orrstown Bank</t>
         </is>
       </c>
-      <c r="D100" t="inlineStr">
+      <c r="D99" t="inlineStr">
         <is>
           <t>linkedin</t>
         </is>
       </c>
-      <c r="E100">
-        <f>HYPERLINK("https://www.linkedin.com/jobs/view/4373227600", "https://www.linkedin.com/jobs/view/4373227600")</f>
-        <v/>
-      </c>
-      <c r="F100" t="inlineStr"/>
-      <c r="G100" t="inlineStr">
+      <c r="E99" t="inlineStr"/>
+      <c r="F99" t="inlineStr"/>
+      <c r="G99" t="inlineStr">
         <is>
           <t>Harrisburg, PA</t>
         </is>
       </c>
-      <c r="H100" t="inlineStr"/>
-      <c r="I100" t="inlineStr">
+      <c r="H99" t="inlineStr"/>
+      <c r="I99" t="inlineStr">
         <is>
           <t>**Position Summary**
  The Data Engineer III is responsible for designing, developing, and maintaining the bank's data infrastructure and systems. This position involves leading the implementation of scalable and robust data solutions, ensuring data quality, security, and compliance. The Data Engineer III will provide technical leadership, collaborate with cross\-functional teams, and drive innovation in data engineering practices to support the bank's strategic objectives.
@@ -10489,35 +11333,32 @@
         </is>
       </c>
     </row>
-    <row r="101">
-      <c r="A101" t="inlineStr">
+    <row r="100">
+      <c r="A100" t="inlineStr">
         <is>
           <t>li-4372085738</t>
         </is>
       </c>
-      <c r="B101" t="inlineStr">
+      <c r="B100" t="inlineStr">
         <is>
           <t>Data Engineer, Support</t>
         </is>
       </c>
-      <c r="C101" t="inlineStr">
+      <c r="C100" t="inlineStr">
         <is>
           <t>RemoteHunter</t>
         </is>
       </c>
-      <c r="D101" t="inlineStr">
+      <c r="D100" t="inlineStr">
         <is>
           <t>linkedin</t>
         </is>
       </c>
-      <c r="E101">
-        <f>HYPERLINK("https://www.linkedin.com/jobs/view/4372085738", "https://www.linkedin.com/jobs/view/4372085738")</f>
-        <v/>
-      </c>
-      <c r="F101" t="inlineStr"/>
-      <c r="G101" t="inlineStr"/>
-      <c r="H101" t="inlineStr"/>
-      <c r="I101" t="inlineStr">
+      <c r="E100" t="inlineStr"/>
+      <c r="F100" t="inlineStr"/>
+      <c r="G100" t="inlineStr"/>
+      <c r="H100" t="inlineStr"/>
+      <c r="I100" t="inlineStr">
         <is>
           <t>About the Opportunity:
  The organization provides an end\-to\-end ecosystem designed to support Programs of All\-Inclusive Care for the Elderly (PACE) in delivering care, improving financial performance, and ensuring compliance. It replaces outdated technology with solutions for care coordination, risk adjustment, population health, and utilization management. The role focuses on supporting operations and improving outcomes for dual\-eligible seniors with complex healthcare needs.
@@ -10557,42 +11398,36 @@
         </is>
       </c>
     </row>
-    <row r="102">
-      <c r="A102" t="inlineStr">
+    <row r="101">
+      <c r="A101" t="inlineStr">
         <is>
           <t>li-4373220984</t>
         </is>
       </c>
-      <c r="B102" t="inlineStr">
+      <c r="B101" t="inlineStr">
         <is>
           <t>Remote Senior Data Engineer</t>
         </is>
       </c>
-      <c r="C102" t="inlineStr">
+      <c r="C101" t="inlineStr">
         <is>
           <t>Jobgether</t>
         </is>
       </c>
-      <c r="D102" t="inlineStr">
+      <c r="D101" t="inlineStr">
         <is>
           <t>linkedin</t>
         </is>
       </c>
-      <c r="E102">
-        <f>HYPERLINK("https://www.linkedin.com/jobs/view/4373220984", "https://www.linkedin.com/jobs/view/4373220984")</f>
-        <v/>
-      </c>
-      <c r="F102">
-        <f>HYPERLINK("https://jobs.lever.co/jobgether/0ad4ed25-3ec4-4ea2-8743-c02799458a36/apply?source=LinkedIn&amp;urlHash=QGAo", "https://jobs.lever.co/jobgether/0ad4ed25-3ec4-4ea2-8743-c02799458a36/apply?source=LinkedIn&amp;urlHash=QGAo")</f>
-        <v/>
-      </c>
-      <c r="G102" t="inlineStr">
+      <c r="E101" t="inlineStr"/>
+      <c r="F101" t="inlineStr"/>
+      <c r="G101" t="inlineStr">
         <is>
           <t>Florida, United States</t>
         </is>
       </c>
-      <c r="H102" t="inlineStr"/>
-      <c r="I102" t="inlineStr">
+      <c r="H101" t="inlineStr"/>
+      <c r="I101" t="inlineStr">
         <is>
           <t>This position is posted by Jobgether on behalf of a partner company. We are currently looking for a Data Engineer. In this role, you will play a crucial part in constructing robust data pipelines that serve as the backbone for internal business analytics. Collaborating closely with senior engineers, you will ensure the seamless ingestion and preparation of data from various sources, elevating data quality for analysis. Your contributions will directly influence critical decision\-making processes, providing leaders with necessary insights efficiently. This role demands a commitment to excellence, allowing you to make a real impact in a fast\-paced, results\-oriented environment.
 **Accountabilities**
@@ -10624,35 +11459,32 @@
         </is>
       </c>
     </row>
-    <row r="103">
-      <c r="A103" t="inlineStr">
+    <row r="102">
+      <c r="A102" t="inlineStr">
         <is>
           <t>li-4373236123</t>
         </is>
       </c>
-      <c r="B103" t="inlineStr">
+      <c r="B102" t="inlineStr">
         <is>
           <t>Data Engineer</t>
         </is>
       </c>
-      <c r="C103" t="inlineStr">
+      <c r="C102" t="inlineStr">
         <is>
           <t>Haystack</t>
         </is>
       </c>
-      <c r="D103" t="inlineStr">
+      <c r="D102" t="inlineStr">
         <is>
           <t>linkedin</t>
         </is>
       </c>
-      <c r="E103">
-        <f>HYPERLINK("https://www.linkedin.com/jobs/view/4373236123", "https://www.linkedin.com/jobs/view/4373236123")</f>
-        <v/>
-      </c>
-      <c r="F103" t="inlineStr"/>
-      <c r="G103" t="inlineStr"/>
-      <c r="H103" t="inlineStr"/>
-      <c r="I103" t="inlineStr">
+      <c r="E102" t="inlineStr"/>
+      <c r="F102" t="inlineStr"/>
+      <c r="G102" t="inlineStr"/>
+      <c r="H102" t="inlineStr"/>
+      <c r="I102" t="inlineStr">
         <is>
           <t>**Splunk Data Engineer \| Reston, VA \| Remote\-Friendly \| $99,000 \- $225,000**
  We're working with Booz Allen Hamilton on this exciting opportunity.
@@ -10678,35 +11510,32 @@
         </is>
       </c>
     </row>
-    <row r="104">
-      <c r="A104" t="inlineStr">
+    <row r="103">
+      <c r="A103" t="inlineStr">
         <is>
           <t>li-4372088708</t>
         </is>
       </c>
-      <c r="B104" t="inlineStr">
+      <c r="B103" t="inlineStr">
         <is>
           <t>Staff Data Engineer</t>
         </is>
       </c>
-      <c r="C104" t="inlineStr">
+      <c r="C103" t="inlineStr">
         <is>
           <t>RemoteHunter</t>
         </is>
       </c>
-      <c r="D104" t="inlineStr">
+      <c r="D103" t="inlineStr">
         <is>
           <t>linkedin</t>
         </is>
       </c>
-      <c r="E104">
-        <f>HYPERLINK("https://www.linkedin.com/jobs/view/4372088708", "https://www.linkedin.com/jobs/view/4372088708")</f>
-        <v/>
-      </c>
-      <c r="F104" t="inlineStr"/>
-      <c r="G104" t="inlineStr"/>
-      <c r="H104" t="inlineStr"/>
-      <c r="I104" t="inlineStr">
+      <c r="E103" t="inlineStr"/>
+      <c r="F103" t="inlineStr"/>
+      <c r="G103" t="inlineStr"/>
+      <c r="H103" t="inlineStr"/>
+      <c r="I103" t="inlineStr">
         <is>
           <t>About the Opportunity:
  This role is for a Staff Data Platform Engineer responsible for designing, building, and owning core systems within a streaming data platform. The position involves hands\-on implementation of key platform capabilities and setting the technical direction for system evolution. The engineer will collaborate with product and engineering teams to translate needs into platform features and develop shared libraries, frameworks, and tooling for reliable data streaming.
@@ -10739,42 +11568,36 @@
         </is>
       </c>
     </row>
-    <row r="105">
-      <c r="A105" t="inlineStr">
+    <row r="104">
+      <c r="A104" t="inlineStr">
         <is>
           <t>li-4312504256</t>
         </is>
       </c>
-      <c r="B105" t="inlineStr">
+      <c r="B104" t="inlineStr">
         <is>
           <t>Data Engineer, Ground Network Engineering (Gateway)</t>
         </is>
       </c>
-      <c r="C105" t="inlineStr">
+      <c r="C104" t="inlineStr">
         <is>
           <t>SpaceX</t>
         </is>
       </c>
-      <c r="D105" t="inlineStr">
+      <c r="D104" t="inlineStr">
         <is>
           <t>linkedin</t>
         </is>
       </c>
-      <c r="E105">
-        <f>HYPERLINK("https://www.linkedin.com/jobs/view/4312504256", "https://www.linkedin.com/jobs/view/4312504256")</f>
-        <v/>
-      </c>
-      <c r="F105">
-        <f>HYPERLINK("https://boards.greenhouse.io/spacex/jobs/8192168002?gh_jid=8192168002&amp;gh_src=3c0864192&amp;urlHash=48pp", "https://boards.greenhouse.io/spacex/jobs/8192168002?gh_jid=8192168002&amp;gh_src=3c0864192&amp;urlHash=48pp")</f>
-        <v/>
-      </c>
-      <c r="G105" t="inlineStr">
+      <c r="E104" t="inlineStr"/>
+      <c r="F104" t="inlineStr"/>
+      <c r="G104" t="inlineStr">
         <is>
           <t>Redmond, WA</t>
         </is>
       </c>
-      <c r="H105" t="inlineStr"/>
-      <c r="I105" t="inlineStr">
+      <c r="H104" t="inlineStr"/>
+      <c r="I104" t="inlineStr">
         <is>
           <t>SpaceX was founded under the belief that a future where humanity is out exploring the stars is fundamentally more exciting than one where we are not. Today SpaceX is actively developing the technologies to make this possible, with the ultimate goal of enabling human life on Mars.
 **DATA ENGINEER, GROUND NETWORK ENGINEERING (GATEWAY)**
@@ -10823,39 +11646,36 @@
         </is>
       </c>
     </row>
-    <row r="106">
-      <c r="A106" t="inlineStr">
+    <row r="105">
+      <c r="A105" t="inlineStr">
         <is>
           <t>li-4373222493</t>
         </is>
       </c>
-      <c r="B106" t="inlineStr">
+      <c r="B105" t="inlineStr">
         <is>
           <t>Data Engineer</t>
         </is>
       </c>
-      <c r="C106" t="inlineStr">
+      <c r="C105" t="inlineStr">
         <is>
           <t>Liberty Mutual Insurance</t>
         </is>
       </c>
-      <c r="D106" t="inlineStr">
+      <c r="D105" t="inlineStr">
         <is>
           <t>linkedin</t>
         </is>
       </c>
-      <c r="E106">
-        <f>HYPERLINK("https://www.linkedin.com/jobs/view/4373222493", "https://www.linkedin.com/jobs/view/4373222493")</f>
-        <v/>
-      </c>
-      <c r="F106" t="inlineStr"/>
-      <c r="G106" t="inlineStr">
+      <c r="E105" t="inlineStr"/>
+      <c r="F105" t="inlineStr"/>
+      <c r="G105" t="inlineStr">
         <is>
           <t>Portsmouth, NH</t>
         </is>
       </c>
-      <c r="H106" t="inlineStr"/>
-      <c r="I106" t="inlineStr">
+      <c r="H105" t="inlineStr"/>
+      <c r="I105" t="inlineStr">
         <is>
           <t>**Description**
  We deliver our customers peace of mind every day by helping them protect what they value most. Our passion for placing the customer at the center of everything we do is drive a transformational shift at Liberty Mutual. Operating as a tech startup within a Fortune 100 company, we are leading a digital disruption that will redefine how people experience insurance.
@@ -10909,39 +11729,36 @@
         </is>
       </c>
     </row>
-    <row r="107">
-      <c r="A107" t="inlineStr">
+    <row r="106">
+      <c r="A106" t="inlineStr">
         <is>
           <t>li-4349735326</t>
         </is>
       </c>
-      <c r="B107" t="inlineStr">
+      <c r="B106" t="inlineStr">
         <is>
           <t>Senior Data Platform Engineer- Weights &amp; Biases</t>
         </is>
       </c>
-      <c r="C107" t="inlineStr">
+      <c r="C106" t="inlineStr">
         <is>
           <t>Weights &amp; Biases</t>
         </is>
       </c>
-      <c r="D107" t="inlineStr">
+      <c r="D106" t="inlineStr">
         <is>
           <t>linkedin</t>
         </is>
       </c>
-      <c r="E107">
-        <f>HYPERLINK("https://www.linkedin.com/jobs/view/4349735326", "https://www.linkedin.com/jobs/view/4349735326")</f>
-        <v/>
-      </c>
-      <c r="F107" t="inlineStr"/>
-      <c r="G107" t="inlineStr">
+      <c r="E106" t="inlineStr"/>
+      <c r="F106" t="inlineStr"/>
+      <c r="G106" t="inlineStr">
         <is>
           <t>New York, NY</t>
         </is>
       </c>
-      <c r="H107" t="inlineStr"/>
-      <c r="I107" t="inlineStr">
+      <c r="H106" t="inlineStr"/>
+      <c r="I106" t="inlineStr">
         <is>
           <t>CoreWeave, the AI Hyperscaler™, acquired Weights \&amp; Biases to create the most powerful end\-to\-end platform to develop, deploy, and iterate AI faster. Since 2017, CoreWeave has operated a growing footprint of data centers covering every region of the US and across Europe, and was ranked as one of the TIME100 most influential companies of 2024\. By bringing together CoreWeave’s industry\-leading cloud infrastructure with the best\-in\-class tools AI practitioners know and love from Weights \&amp; Biases, we’re setting a new standard for how AI is built, trained, and scaled.
  The integration of our teams and technologies is accelerating our shared mission: to empower developers with the tools and infrastructure they need to push the boundaries of what AI can do. From experiment tracking and model optimization to high\-performance training clusters, agent building, and inference at scale, we’re combining forces to serve the full AI lifecycle — all in one seamless platform.
@@ -11022,39 +11839,36 @@
         </is>
       </c>
     </row>
-    <row r="108">
-      <c r="A108" t="inlineStr">
+    <row r="107">
+      <c r="A107" t="inlineStr">
         <is>
           <t>li-4349872344</t>
         </is>
       </c>
-      <c r="B108" t="inlineStr">
+      <c r="B107" t="inlineStr">
         <is>
           <t>Senior Data Platform Engineer- Weights &amp; Biases</t>
         </is>
       </c>
-      <c r="C108" t="inlineStr">
+      <c r="C107" t="inlineStr">
         <is>
           <t>Weights &amp; Biases</t>
         </is>
       </c>
-      <c r="D108" t="inlineStr">
+      <c r="D107" t="inlineStr">
         <is>
           <t>linkedin</t>
         </is>
       </c>
-      <c r="E108">
-        <f>HYPERLINK("https://www.linkedin.com/jobs/view/4349872344", "https://www.linkedin.com/jobs/view/4349872344")</f>
-        <v/>
-      </c>
-      <c r="F108" t="inlineStr"/>
-      <c r="G108" t="inlineStr">
+      <c r="E107" t="inlineStr"/>
+      <c r="F107" t="inlineStr"/>
+      <c r="G107" t="inlineStr">
         <is>
           <t>Sunnyvale, CA</t>
         </is>
       </c>
-      <c r="H108" t="inlineStr"/>
-      <c r="I108" t="inlineStr">
+      <c r="H107" t="inlineStr"/>
+      <c r="I107" t="inlineStr">
         <is>
           <t>CoreWeave, the AI Hyperscaler™, acquired Weights \&amp; Biases to create the most powerful end\-to\-end platform to develop, deploy, and iterate AI faster. Since 2017, CoreWeave has operated a growing footprint of data centers covering every region of the US and across Europe, and was ranked as one of the TIME100 most influential companies of 2024\. By bringing together CoreWeave’s industry\-leading cloud infrastructure with the best\-in\-class tools AI practitioners know and love from Weights \&amp; Biases, we’re setting a new standard for how AI is built, trained, and scaled.
  The integration of our teams and technologies is accelerating our shared mission: to empower developers with the tools and infrastructure they need to push the boundaries of what AI can do. From experiment tracking and model optimization to high\-performance training clusters, agent building, and inference at scale, we’re combining forces to serve the full AI lifecycle — all in one seamless platform.
@@ -11135,39 +11949,36 @@
         </is>
       </c>
     </row>
-    <row r="109">
-      <c r="A109" t="inlineStr">
+    <row r="108">
+      <c r="A108" t="inlineStr">
         <is>
           <t>li-4371332506</t>
         </is>
       </c>
-      <c r="B109" t="inlineStr">
+      <c r="B108" t="inlineStr">
         <is>
           <t>Data Engineer I</t>
         </is>
       </c>
-      <c r="C109" t="inlineStr">
+      <c r="C108" t="inlineStr">
         <is>
           <t>Jobs via Dice</t>
         </is>
       </c>
-      <c r="D109" t="inlineStr">
+      <c r="D108" t="inlineStr">
         <is>
           <t>linkedin</t>
         </is>
       </c>
-      <c r="E109">
-        <f>HYPERLINK("https://www.linkedin.com/jobs/view/4371332506", "https://www.linkedin.com/jobs/view/4371332506")</f>
-        <v/>
-      </c>
-      <c r="F109" t="inlineStr"/>
-      <c r="G109" t="inlineStr">
+      <c r="E108" t="inlineStr"/>
+      <c r="F108" t="inlineStr"/>
+      <c r="G108" t="inlineStr">
         <is>
           <t>Cincinnati, OH</t>
         </is>
       </c>
-      <c r="H109" t="inlineStr"/>
-      <c r="I109" t="inlineStr">
+      <c r="H108" t="inlineStr"/>
+      <c r="I108" t="inlineStr">
         <is>
           <t>**Description:**
 *Onsite in Cincinnati, OH*
@@ -11212,39 +12023,36 @@
         </is>
       </c>
     </row>
-    <row r="110">
-      <c r="A110" t="inlineStr">
+    <row r="109">
+      <c r="A109" t="inlineStr">
         <is>
           <t>li-4321384025</t>
         </is>
       </c>
-      <c r="B110" t="inlineStr">
+      <c r="B109" t="inlineStr">
         <is>
           <t>Lead, IT Data Engineer</t>
         </is>
       </c>
-      <c r="C110" t="inlineStr">
+      <c r="C109" t="inlineStr">
         <is>
           <t>Shure Incorporated</t>
         </is>
       </c>
-      <c r="D110" t="inlineStr">
+      <c r="D109" t="inlineStr">
         <is>
           <t>linkedin</t>
         </is>
       </c>
-      <c r="E110">
-        <f>HYPERLINK("https://www.linkedin.com/jobs/view/4321384025", "https://www.linkedin.com/jobs/view/4321384025")</f>
-        <v/>
-      </c>
-      <c r="F110" t="inlineStr"/>
-      <c r="G110" t="inlineStr">
+      <c r="E109" t="inlineStr"/>
+      <c r="F109" t="inlineStr"/>
+      <c r="G109" t="inlineStr">
         <is>
           <t>Niles, IL</t>
         </is>
       </c>
-      <c r="H110" t="inlineStr"/>
-      <c r="I110" t="inlineStr">
+      <c r="H109" t="inlineStr"/>
+      <c r="I109" t="inlineStr">
         <is>
           <t>**Come join the global IT team at Shure!**
  In your role as
@@ -11297,39 +12105,36 @@
         </is>
       </c>
     </row>
-    <row r="111">
-      <c r="A111" t="inlineStr">
+    <row r="110">
+      <c r="A110" t="inlineStr">
         <is>
           <t>li-4371196181</t>
         </is>
       </c>
-      <c r="B111" t="inlineStr">
+      <c r="B110" t="inlineStr">
         <is>
           <t>Data Engineer</t>
         </is>
       </c>
-      <c r="C111" t="inlineStr">
+      <c r="C110" t="inlineStr">
         <is>
           <t>Jobs via Dice</t>
         </is>
       </c>
-      <c r="D111" t="inlineStr">
+      <c r="D110" t="inlineStr">
         <is>
           <t>linkedin</t>
         </is>
       </c>
-      <c r="E111">
-        <f>HYPERLINK("https://www.linkedin.com/jobs/view/4371196181", "https://www.linkedin.com/jobs/view/4371196181")</f>
-        <v/>
-      </c>
-      <c r="F111" t="inlineStr"/>
-      <c r="G111" t="inlineStr">
+      <c r="E110" t="inlineStr"/>
+      <c r="F110" t="inlineStr"/>
+      <c r="G110" t="inlineStr">
         <is>
           <t>Dallas, TX</t>
         </is>
       </c>
-      <c r="H111" t="inlineStr"/>
-      <c r="I111" t="inlineStr">
+      <c r="H110" t="inlineStr"/>
+      <c r="I110" t="inlineStr">
         <is>
           <t>RESPONSIBILITIES:
  Kforce has a client in Dallas, TX that is looking for a Data Engineer to join their team building a new application that supports mainframe application rationalization and modernization. This application will ingest, model, and persist data used to analyze legacy systems and inform future decisions around which applications should be migrated off the mainframe. This role is heavily focused on data modeling, data architecture, and data stewardship\-not just pipelines. The Data Engineer will help define how critical application data is structured, stored, and later leveraged for analysis and graph\-based relationships.
@@ -11363,39 +12168,36 @@
         </is>
       </c>
     </row>
-    <row r="112">
-      <c r="A112" t="inlineStr">
+    <row r="111">
+      <c r="A111" t="inlineStr">
         <is>
           <t>li-4373226764</t>
         </is>
       </c>
-      <c r="B112" t="inlineStr">
+      <c r="B111" t="inlineStr">
         <is>
           <t>Remote Lead Data Engineer</t>
         </is>
       </c>
-      <c r="C112" t="inlineStr">
+      <c r="C111" t="inlineStr">
         <is>
           <t>Jobgether</t>
         </is>
       </c>
-      <c r="D112" t="inlineStr">
+      <c r="D111" t="inlineStr">
         <is>
           <t>linkedin</t>
         </is>
       </c>
-      <c r="E112">
-        <f>HYPERLINK("https://www.linkedin.com/jobs/view/4373226764", "https://www.linkedin.com/jobs/view/4373226764")</f>
-        <v/>
-      </c>
-      <c r="F112" t="inlineStr"/>
-      <c r="G112" t="inlineStr">
+      <c r="E111" t="inlineStr"/>
+      <c r="F111" t="inlineStr"/>
+      <c r="G111" t="inlineStr">
         <is>
           <t>Minnesota, United States</t>
         </is>
       </c>
-      <c r="H112" t="inlineStr"/>
-      <c r="I112" t="inlineStr">
+      <c r="H111" t="inlineStr"/>
+      <c r="I111" t="inlineStr">
         <is>
           <t>This position is posted by Jobgether on behalf of a partner company. We are currently looking for a Data Engineer. In this role, you will play a crucial part in constructing robust data pipelines that serve as the backbone for internal business analytics. Collaborating closely with senior engineers, you will ensure the seamless ingestion and preparation of data from various sources, elevating data quality for analysis. Your contributions will directly influence critical decision\-making processes, providing leaders with necessary insights efficiently. This role demands a commitment to excellence, allowing you to make a real impact in a fast\-paced, results\-oriented environment.
 **Accountabilities**
@@ -11427,39 +12229,36 @@
         </is>
       </c>
     </row>
-    <row r="113">
-      <c r="A113" t="inlineStr">
+    <row r="112">
+      <c r="A112" t="inlineStr">
         <is>
           <t>li-4290987963</t>
         </is>
       </c>
-      <c r="B113" t="inlineStr">
+      <c r="B112" t="inlineStr">
         <is>
           <t>Data Engineering Team Lead (Hybrid)</t>
         </is>
       </c>
-      <c r="C113" t="inlineStr">
+      <c r="C112" t="inlineStr">
         <is>
           <t>Selective Insurance</t>
         </is>
       </c>
-      <c r="D113" t="inlineStr">
+      <c r="D112" t="inlineStr">
         <is>
           <t>linkedin</t>
         </is>
       </c>
-      <c r="E113">
-        <f>HYPERLINK("https://www.linkedin.com/jobs/view/4290987963", "https://www.linkedin.com/jobs/view/4290987963")</f>
-        <v/>
-      </c>
-      <c r="F113" t="inlineStr"/>
-      <c r="G113" t="inlineStr">
+      <c r="E112" t="inlineStr"/>
+      <c r="F112" t="inlineStr"/>
+      <c r="G112" t="inlineStr">
         <is>
           <t>Short Hills, NJ</t>
         </is>
       </c>
-      <c r="H113" t="inlineStr"/>
-      <c r="I113" t="inlineStr">
+      <c r="H112" t="inlineStr"/>
+      <c r="I112" t="inlineStr">
         <is>
           <t>**About Us**
 *At Selective, we don't just insure uniquely, we employ uniqueness.*
@@ -11507,42 +12306,36 @@
         </is>
       </c>
     </row>
-    <row r="114">
-      <c r="A114" t="inlineStr">
+    <row r="113">
+      <c r="A113" t="inlineStr">
         <is>
           <t>li-4312310119</t>
         </is>
       </c>
-      <c r="B114" t="inlineStr">
+      <c r="B113" t="inlineStr">
         <is>
           <t>Data Engineering Team Lead (Hybrid)</t>
         </is>
       </c>
-      <c r="C114" t="inlineStr">
+      <c r="C113" t="inlineStr">
         <is>
           <t>Selective Insurance</t>
         </is>
       </c>
-      <c r="D114" t="inlineStr">
+      <c r="D113" t="inlineStr">
         <is>
           <t>linkedin</t>
         </is>
       </c>
-      <c r="E114">
-        <f>HYPERLINK("https://www.linkedin.com/jobs/view/4312310119", "https://www.linkedin.com/jobs/view/4312310119")</f>
-        <v/>
-      </c>
-      <c r="F114">
-        <f>HYPERLINK("https://jobs.selective.com/jobs/4915?lang=en-us&amp;iis=Job+Board&amp;iisn=LinkedIn&amp;urlHash=Rz8F", "https://jobs.selective.com/jobs/4915?lang=en-us&amp;iis=Job+Board&amp;iisn=LinkedIn&amp;urlHash=Rz8F")</f>
-        <v/>
-      </c>
-      <c r="G114" t="inlineStr">
+      <c r="E113" t="inlineStr"/>
+      <c r="F113" t="inlineStr"/>
+      <c r="G113" t="inlineStr">
         <is>
           <t>Charlotte, NC</t>
         </is>
       </c>
-      <c r="H114" t="inlineStr"/>
-      <c r="I114" t="inlineStr">
+      <c r="H113" t="inlineStr"/>
+      <c r="I113" t="inlineStr">
         <is>
           <t>**About Us**
 *At Selective, we don't just insure uniquely, we employ uniqueness.*
@@ -11591,42 +12384,36 @@
         </is>
       </c>
     </row>
-    <row r="115">
-      <c r="A115" t="inlineStr">
+    <row r="114">
+      <c r="A114" t="inlineStr">
         <is>
           <t>li-4365607046</t>
         </is>
       </c>
-      <c r="B115" t="inlineStr">
+      <c r="B114" t="inlineStr">
         <is>
           <t>Sr. Mgr, Data Engineering</t>
         </is>
       </c>
-      <c r="C115" t="inlineStr">
+      <c r="C114" t="inlineStr">
         <is>
           <t>Capital One</t>
         </is>
       </c>
-      <c r="D115" t="inlineStr">
+      <c r="D114" t="inlineStr">
         <is>
           <t>linkedin</t>
         </is>
       </c>
-      <c r="E115">
-        <f>HYPERLINK("https://www.linkedin.com/jobs/view/4365607046", "https://www.linkedin.com/jobs/view/4365607046")</f>
-        <v/>
-      </c>
-      <c r="F115">
-        <f>HYPERLINK("https://dsp.prng.co/Y5355_b&amp;urlHash=-QXU", "https://dsp.prng.co/Y5355_b&amp;urlHash=-QXU")</f>
-        <v/>
-      </c>
-      <c r="G115" t="inlineStr">
+      <c r="E114" t="inlineStr"/>
+      <c r="F114" t="inlineStr"/>
+      <c r="G114" t="inlineStr">
         <is>
           <t>Richmond, VA</t>
         </is>
       </c>
-      <c r="H115" t="inlineStr"/>
-      <c r="I115" t="inlineStr">
+      <c r="H114" t="inlineStr"/>
+      <c r="I114" t="inlineStr">
         <is>
           <t>Do you love building and pioneering in the technology space? Do you enjoy solving complex business problems in a fast\-paced, collaborative, inclusive, and iterative delivery environment? At Capital One, you'll be part of a big group of makers, breakers, doers and disruptors, who solve real problems and meet real customer needs. We are seeking Data Engineers who are passionate about marrying data with emerging technologies. As a Capital One Senior Manager Data Engineer, you’ll have the opportunity to be on the forefront of driving a major transformation within Capital One.
 ****What You’ll Do:****
@@ -11671,39 +12458,36 @@
         </is>
       </c>
     </row>
-    <row r="116">
-      <c r="A116" t="inlineStr">
+    <row r="115">
+      <c r="A115" t="inlineStr">
         <is>
           <t>li-4365607045</t>
         </is>
       </c>
-      <c r="B116" t="inlineStr">
+      <c r="B115" t="inlineStr">
         <is>
           <t>Sr. Mgr, Data Engineering</t>
         </is>
       </c>
-      <c r="C116" t="inlineStr">
+      <c r="C115" t="inlineStr">
         <is>
           <t>Capital One</t>
         </is>
       </c>
-      <c r="D116" t="inlineStr">
+      <c r="D115" t="inlineStr">
         <is>
           <t>linkedin</t>
         </is>
       </c>
-      <c r="E116">
-        <f>HYPERLINK("https://www.linkedin.com/jobs/view/4365607045", "https://www.linkedin.com/jobs/view/4365607045")</f>
-        <v/>
-      </c>
-      <c r="F116" t="inlineStr"/>
-      <c r="G116" t="inlineStr">
+      <c r="E115" t="inlineStr"/>
+      <c r="F115" t="inlineStr"/>
+      <c r="G115" t="inlineStr">
         <is>
           <t>McLean, VA</t>
         </is>
       </c>
-      <c r="H116" t="inlineStr"/>
-      <c r="I116" t="inlineStr">
+      <c r="H115" t="inlineStr"/>
+      <c r="I115" t="inlineStr">
         <is>
           <t>Do you love building and pioneering in the technology space? Do you enjoy solving complex business problems in a fast\-paced, collaborative, inclusive, and iterative delivery environment? At Capital One, you'll be part of a big group of makers, breakers, doers and disruptors, who solve real problems and meet real customer needs. We are seeking Data Engineers who are passionate about marrying data with emerging technologies. As a Capital One Senior Manager Data Engineer, you’ll have the opportunity to be on the forefront of driving a major transformation within Capital One.
 ****What You’ll Do:****
@@ -11748,42 +12532,36 @@
         </is>
       </c>
     </row>
-    <row r="117">
-      <c r="A117" t="inlineStr">
+    <row r="116">
+      <c r="A116" t="inlineStr">
         <is>
           <t>li-4343348942</t>
         </is>
       </c>
-      <c r="B117" t="inlineStr">
+      <c r="B116" t="inlineStr">
         <is>
           <t>Senior Data Engineer</t>
         </is>
       </c>
-      <c r="C117" t="inlineStr">
+      <c r="C116" t="inlineStr">
         <is>
           <t>SAIC</t>
         </is>
       </c>
-      <c r="D117" t="inlineStr">
+      <c r="D116" t="inlineStr">
         <is>
           <t>linkedin</t>
         </is>
       </c>
-      <c r="E117">
-        <f>HYPERLINK("https://www.linkedin.com/jobs/view/4343348942", "https://www.linkedin.com/jobs/view/4343348942")</f>
-        <v/>
-      </c>
-      <c r="F117">
-        <f>HYPERLINK("https://jsv3.recruitics.com/redirect?rx_cid=3284&amp;rx_jobId=2512347&amp;rx_url=https%3A%2F%2Fjobs.saic.com%2Fjobs%2F17136584-senior-data-engineer%3Fbid%3D370%26rx_campaign%3DLinkedin1%26rx_ch%3Djobpost%26rx_group%3D128565%26rx_id%3D5f3bca6a-d7bd-11f0-8d33-d73f12634dca%26rx_job%3D2512347%26rx_medium%3Dpost%26rx_paid%3D1%26rx_r%3Dnone%26rx_source%3Dlinkedin%26rx_ts%3D20260214T181208Z%26rx_vp%3Djobslots%26tm_company%3D2520%26tm_event%3Dview%26tm_job%3D2512347&amp;urlHash=tSNH", "https://jsv3.recruitics.com/redirect?rx_cid=3284&amp;rx_jobId=2512347&amp;rx_url=https%3A%2F%2Fjobs.saic.com%2Fjobs%2F17136584-senior-data-engineer%3Fbid%3D370%26rx_campaign%3DLinkedin1%26rx_ch%3Djobpost%26rx_group%3D128565%26rx_id%3D5f3bca6a-d7bd-11f0-8d33-d73f12634dca%26rx_job%3D2512347%26rx_medium%3Dpost%26rx_paid%3D1%26rx_r%3Dnone%26rx_source%3Dlinkedin%26rx_ts%3D20260214T181208Z%26rx_vp%3Djobslots%26tm_company%3D2520%26tm_event%3Dview%26tm_job%3D2512347&amp;urlHash=tSNH")</f>
-        <v/>
-      </c>
-      <c r="G117" t="inlineStr">
+      <c r="E116" t="inlineStr"/>
+      <c r="F116" t="inlineStr"/>
+      <c r="G116" t="inlineStr">
         <is>
           <t>San Diego, CA</t>
         </is>
       </c>
-      <c r="H117" t="inlineStr"/>
-      <c r="I117" t="inlineStr">
+      <c r="H116" t="inlineStr"/>
+      <c r="I116" t="inlineStr">
         <is>
           <t>Job ID 2512347
 **Location** 
@@ -11851,35 +12629,32 @@
         </is>
       </c>
     </row>
-    <row r="118">
-      <c r="A118" t="inlineStr">
+    <row r="117">
+      <c r="A117" t="inlineStr">
         <is>
           <t>li-4332801612</t>
         </is>
       </c>
-      <c r="B118" t="inlineStr">
+      <c r="B117" t="inlineStr">
         <is>
           <t>Senior Associate, Data Analytics Engineering</t>
         </is>
       </c>
-      <c r="C118" t="inlineStr">
+      <c r="C117" t="inlineStr">
         <is>
           <t>The Options Clearing Corporation (OCC)</t>
         </is>
       </c>
-      <c r="D118" t="inlineStr">
+      <c r="D117" t="inlineStr">
         <is>
           <t>linkedin</t>
         </is>
       </c>
-      <c r="E118">
-        <f>HYPERLINK("https://www.linkedin.com/jobs/view/4332801612", "https://www.linkedin.com/jobs/view/4332801612")</f>
-        <v/>
-      </c>
-      <c r="F118" t="inlineStr"/>
-      <c r="G118" t="inlineStr"/>
-      <c r="H118" t="inlineStr"/>
-      <c r="I118" t="inlineStr">
+      <c r="E117" t="inlineStr"/>
+      <c r="F117" t="inlineStr"/>
+      <c r="G117" t="inlineStr"/>
+      <c r="H117" t="inlineStr"/>
+      <c r="I117" t="inlineStr">
         <is>
           <t>* THIS POSITION IS NOT ELIGIBLE FOR VISA SPONSORSHIP\*\*\*\*\*
 **What You'll Do:**
@@ -11960,6 +12735,1157 @@
         </is>
       </c>
     </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>li-4373241699</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>Remote Junior Data Engineer</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>Lensa</t>
+        </is>
+      </c>
+      <c r="D118" t="inlineStr">
+        <is>
+          <t>linkedin</t>
+        </is>
+      </c>
+      <c r="E118">
+        <f>HYPERLINK("https://www.linkedin.com/jobs/view/4373241699", "https://www.linkedin.com/jobs/view/4373241699")</f>
+        <v/>
+      </c>
+      <c r="F118" t="inlineStr"/>
+      <c r="G118" t="inlineStr">
+        <is>
+          <t>Woonsocket, RI</t>
+        </is>
+      </c>
+      <c r="H118" t="inlineStr"/>
+      <c r="I118" t="inlineStr">
+        <is>
+          <t>Lensa is a career site that helps job seekers find great jobs in the US. We are not a staffing firm or agency. Lensa does not hire directly for these jobs, but promotes jobs on LinkedIn on behalf of its direct clients, recruitment ad agencies, and marketing partners. Lensa partners with DirectEmployers to promote this job for Insight Global. Clicking "Apply Now" or "Read more" on Lensa redirects you to the job board/employer site. Any information collected there is subject to their terms and privacy notice.
+**Job Description**
+ Insight Global is hiring a Data Engineer to contribute to ongoing operational data workflows for a major healthcare partner. The position focuses on day‑to‑day processing and transformation of client data, with most tasks being consistent and routine. Occasional data issues may arise that require analytical troubleshooting. Candidates should bring 2\+ years of data engineering experience and strong SQL expertise (SSIS, SQL Server), along with exceptional attention to detail and the ability to follow structured processes.
+ We are a company committed to creating diverse and inclusive environments where people can bring their full, authentic selves to work every day. We are an equal opportunity/affirmative action employer that believes everyone matters. Qualified candidates will receive consideration for employment regardless of their race, color, ethnicity, religion, sex (including pregnancy), sexual orientation, gender identity and expression, marital status, national origin, ancestry, genetic factors, age, disability, protected veteran status, military or uniformed service member status, or any other status or characteristic protected by applicable laws, regulations, and ordinances. If you need assistance and/or a reasonable accommodation due to a disability during the application or recruiting process, please send a request to HR@insightglobal.com.To learn more about how we collect, keep, and process your private information, please review Insight Global's Workforce Privacy Policy: https://insightglobal.com/workforce\-privacy\-policy/.
+**Skills And Requirements**
+* 2\+ years of data engineering experience
+* Hands\-on experience with SQL technologies, including SSIS and SQL Server
+* Strong understanding of SQL concepts and best practices
+* Demonstrates strong diligence and attention to detail
+* Follows instructions accurately and consistently
+* Experience working with client data ingestion processes and handling healthcare PHI
+ If you have questions about this posting, please contact support@lensa.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>li-4321134405</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>Founding Data Engineer (ML Pipelines)</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>Greylock Partners</t>
+        </is>
+      </c>
+      <c r="D119" t="inlineStr">
+        <is>
+          <t>linkedin</t>
+        </is>
+      </c>
+      <c r="E119">
+        <f>HYPERLINK("https://www.linkedin.com/jobs/view/4321134405", "https://www.linkedin.com/jobs/view/4321134405")</f>
+        <v/>
+      </c>
+      <c r="F119" t="inlineStr"/>
+      <c r="G119" t="inlineStr">
+        <is>
+          <t>Redwood City, CA</t>
+        </is>
+      </c>
+      <c r="H119" t="inlineStr"/>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>Early\-stage, cybersecurity investment (valued over $100M at Seed), founded by a successful serial entrepreneur, is looking to hire a Founding Data Engineer with a strong background supporting full ML pipelines. Bonus points for prior industry exp in cybersecurity.
+**Summary:** 
+ Supporting machine learning efforts by focusing on building and maintaining the real\-time data pipelines that feed models with reliable, high\-quality information. Your work will center on ingesting, transforming, and organizing massive data streams so that training and inference systems have consistent, accurate inputs. In this role, you will handle the backbone of ML workflows — ensuring scalability, low latency, and data governance. Your success will be measured by how efficiently and reliably data flows through the ecosystem, from raw sources to feature stores and production endpoints.
+**Key Qualifications:** 
+* Degree in CS (or a related field) with 4\+ years related industry experience in data engineering
+* Prior experience with a zero\-to\-one a strong plus
+* Proven ability to collaborate across different teams and adapt to new fields
+**Responsibilities:** 
+* Design and maintain real\-time data pipelines to support large\-scale machine learning workflows, ensuring low\-latency ingestion and high reliability.
+* Build and optimize data infrastructure for feature extraction, model training, and online inference using modern streaming and orchestration frameworks.
+* Collaborate with ML researchers and platform engineers to integrate models into production systems and enable continuous data feedback loops.
+* Implement robust data quality, observability, and governance practices to ensure scalability, compliance, and reproducibility across enterprise environments.
+ Please note:
+ There are no fees associated with any of the support we provide our investments. Greylock Talent provides free candidate referrals/introductions to all of our active investments (one of the many services we provide).
+ Due to the volume of applicants we typically receive, a follow\-up email will not be sent unless a match is identified.</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>li-4373239742</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>Data Engineer</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>Lensa</t>
+        </is>
+      </c>
+      <c r="D120" t="inlineStr">
+        <is>
+          <t>linkedin</t>
+        </is>
+      </c>
+      <c r="E120">
+        <f>HYPERLINK("https://www.linkedin.com/jobs/view/4373239742", "https://www.linkedin.com/jobs/view/4373239742")</f>
+        <v/>
+      </c>
+      <c r="F120" t="inlineStr"/>
+      <c r="G120" t="inlineStr">
+        <is>
+          <t>New York, NY</t>
+        </is>
+      </c>
+      <c r="H120" t="inlineStr"/>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>Lensa is a career site that helps job seekers find great jobs in the US. We are not a staffing firm or agency. Lensa does not hire directly for these jobs, but promotes jobs on LinkedIn on behalf of its direct clients, recruitment ad agencies, and marketing partners. Lensa partners with DirectEmployers to promote this job for Insight Global. Clicking "Apply Now" or "Read more" on Lensa redirects you to the job board/employer site. Any information collected there is subject to their terms and privacy notice.
+**Job Description**
+ Churchill is seeking an Associate to join the Investment Infrastructure and Technology team. The role is focused on designing, building, and optimizing core technology infrastructure that powers applications and tools used by front\-office professionals, executives, and other internal business units. Key areas include data warehouse, database management, application development, reporting systems, and ad\-hoc initiatives that support business operations. The position offers significant opportunities to apply modern technologies and innovative solutions to drive operational efficiency. The candidate will contribute to system integration efforts and data pipeline development, enabling seamless connectivity between enterprise systems and the data warehouse. The candidate will develop and maintain reports and dashboards related to the firm’s investment portfolio, and act as a technical liaison across all departments and affiliated business partners. The ideal candidate has an entrepreneurial personality with a strong ownership mentality, technical background, and the ability to handle multiple, ongoing projects
+ We are a company committed to creating diverse and inclusive environments where people can bring their full, authentic selves to work every day. We are an equal opportunity/affirmative action employer that believes everyone matters. Qualified candidates will receive consideration for employment regardless of their race, color, ethnicity, religion, sex (including pregnancy), sexual orientation, gender identity and expression, marital status, national origin, ancestry, genetic factors, age, disability, protected veteran status, military or uniformed service member status, or any other status or characteristic protected by applicable laws, regulations, and ordinances. If you need assistance and/or a reasonable accommodation due to a disability during the application or recruiting process, please send a request to HR@insightglobal.com.To learn more about how we collect, keep, and process your private information, please review Insight Global's Workforce Privacy Policy: https://insightglobal.com/workforce\-privacy\-policy/.
+**Skills And Requirements**
+* 2\-4 years of relevant professional experience in investment management, financial operations, or related industries
+* Strong familiarity with Snowflake, SQL Server, PowerBI or Tableau.
+* Bachelor’s degree in Computer Science with a data engineering background.
+* Proficient in SQL and Python, with experience using libraries such as pandas for data wrangling and practical experience integrating and consuming APIs.
+* Background in financial services.
+* Strong interpersonal and communication skills.
+* Experience working at firms specializing in private credit, private equity, and junior capital investments.
+* Masters Degree in Computer Science.
+* Direct experience developing applications or tools with AI
+ If you have questions about this posting, please contact support@lensa.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>li-4325260801</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>Founding Data Engineer</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>Greylock Partners</t>
+        </is>
+      </c>
+      <c r="D121" t="inlineStr">
+        <is>
+          <t>linkedin</t>
+        </is>
+      </c>
+      <c r="E121">
+        <f>HYPERLINK("https://www.linkedin.com/jobs/view/4325260801", "https://www.linkedin.com/jobs/view/4325260801")</f>
+        <v/>
+      </c>
+      <c r="F121" t="inlineStr"/>
+      <c r="G121" t="inlineStr">
+        <is>
+          <t>San Jose, CA</t>
+        </is>
+      </c>
+      <c r="H121" t="inlineStr"/>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>Early\-stage, cybersecurity investment (valued over $100M at Seed), founded by a successful serial entrepreneur, is looking to hire a Founding Data Engineer. Bonus points for prior industry exp in cybersecurity.
+ Our ideal candidate will be a seasoned data engineering specialist (with 5\+ years relevant industry exp) who can help this company create its next generation of analytics infrastructure. Working closely with a highly\-experienced founding team, you will play a central role in shaping data architecture from the ground up and will have significant room for professional growth as the organization scales.
+**What the Role Involves** 
+ The position centers on designing and operating a modern, open\-source data lakehouse environment built to handle extremely large datasets. The engineer will be responsible for constructing robust, end\-to\-end pipelines—from data intake to processing to end\-user access—while ensuring the platform is performant, dependable, and accurate at massive scale.
+**Qualifications:** 
+* Demonstrated expertise in building and managing very large data platforms (multi\-petabyte range)
+* Background in both streaming and batch data processing
+* Hands\-on familiarity with open\-source technologies commonly used in lakehouse setups (e.g., Iceberg, PostgreSQL, Parquet, graph databases such as Neo4j)
+* Strong experience with streaming and analytics frameworks like Kafka, Spark, or Flink
+* Solid understanding of data transformation practices
+* Advanced proficiency in Python
+* Clear communication skills and the ability to produce strong technical documentation
+* Bonus: experience with cloud service provider data ecosystems
+* Bonus: knowledge of tools related to governance, data quality, and lineage
+ Please note:
+ There are no fees associated with any of the support we provide our investments. Greylock Talent provides free candidate referrals/introductions to all of our active investments (one of the many services we provide).
+ Due to the volume of applicants we typically receive, a follow\-up email will not be sent unless a match is identified.</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>li-4373251391</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>REMOTE- Junior Data Engineer</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>Lensa</t>
+        </is>
+      </c>
+      <c r="D122" t="inlineStr">
+        <is>
+          <t>linkedin</t>
+        </is>
+      </c>
+      <c r="E122">
+        <f>HYPERLINK("https://www.linkedin.com/jobs/view/4373251391", "https://www.linkedin.com/jobs/view/4373251391")</f>
+        <v/>
+      </c>
+      <c r="F122">
+        <f>HYPERLINK("https://lensa.com/cgw/72918a38f3b7405397bd4c6ec4c0f582tjo1?jpsi=directemployers&amp;publisher_preference=easier_apply&amp;utm_campaign=Computer%20Occupations&amp;utm_medium=slot&amp;utm_source=linkedin&amp;utm_term=jse&amp;urlHash=9DIY", "https://lensa.com/cgw/72918a38f3b7405397bd4c6ec4c0f582tjo1?jpsi=directemployers&amp;publisher_preference=easier_apply&amp;utm_campaign=Computer%20Occupations&amp;utm_medium=slot&amp;utm_source=linkedin&amp;utm_term=jse&amp;urlHash=9DIY")</f>
+        <v/>
+      </c>
+      <c r="G122" t="inlineStr">
+        <is>
+          <t>Fort Worth, TX</t>
+        </is>
+      </c>
+      <c r="H122" t="inlineStr"/>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>Lensa is a career site that helps job seekers find great jobs in the US. We are not a staffing firm or agency. Lensa does not hire directly for these jobs, but promotes jobs on LinkedIn on behalf of its direct clients, recruitment ad agencies, and marketing partners. Lensa partners with DirectEmployers to promote this job for Insight Global. Clicking "Apply Now" or "Read more" on Lensa redirects you to the job board/employer site. Any information collected there is subject to their terms and privacy notice.
+**Job Description**
+ One of the largest logistics and transportation employers in the US is seeking a Jr. Data Engineer to join their expanding team. The Jr. Data Engineer will play a crucial role in understanding business problems and assisting in designing solutions that transform complex ideas into sustainable processes. This individual will focus on supporting the onboarding of new lines of business into the data analytics team. Their responsibilities will include assisting in the full life cycle of data engineering, from gathering requirements from internal customers to building data pipelines, testing, reporting, and maintaining solutions. Additionally, the Jr. Data Engineer will support escalation tasks, contribute to system development, help automate processes, maintain internal systems, and assist in data modeling. They will use their growing expertise in data structures specific to the company's operating systems to help turn data into valuable business insights.
+ We are a company committed to creating inclusive environments where people can bring their full, authentic selves to work every day. We are an equal opportunity employer that believes everyone matters. Qualified candidates will receive consideration for employment opportunities without regard to race, religion, sex, age, marital status, national origin, sexual orientation, citizenship status, disability, or any other status or characteristic protected by applicable laws, regulations, and ordinances. If you need assistance and/or a reasonable accommodation due to a disability during the application or recruiting process, please send a request to Human Resources Request Form (https://airtable.com/app21VjYyxLDIX0ez/shrOg4IQS1J6dRiMo) . The EEOC "Know Your Rights" Poster is available here (https://www.eeoc.gov/sites/default/files/2023\-06/22\-088\_EEOC\_KnowYourRights6\.12ScreenRdr.pdf) .
+ To learn more about how we collect, keep, and process your private information, please review Insight Global's Workforce Privacy Policy: https://insightglobal.com/workforce\-privacy\-policy/ .
+**Skills And Requirements**
+ 2\-5\+ years' experience of data engineer experience
+  Strong ADF experience (creating pipelines from scratch/ knowledge of connectors and activities following architect plan)
+  Strong knowledge of SQL (Mostly working with SQL scripting implementing into ADF)
+  Understanding of full life cycle data engineering
+  Extremely detail oriented and ability to provide effective updates
+  Strong communication for working with internal/ external customers
+  Strong critical thinking skills Python or Spark experience (Small environment is in Python\- basic level scripting and reviews)
+  DevOps Experience
+  Data Bricks Experience
+  Background in Logistics
+  Agile Methodologies
+  Experience with cloud (Azure specifically)
+ If you have questions about this posting, please contact support@lensa.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>li-4373234939</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>Data Engineer</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>Lensa</t>
+        </is>
+      </c>
+      <c r="D123" t="inlineStr">
+        <is>
+          <t>linkedin</t>
+        </is>
+      </c>
+      <c r="E123">
+        <f>HYPERLINK("https://www.linkedin.com/jobs/view/4373234939", "https://www.linkedin.com/jobs/view/4373234939")</f>
+        <v/>
+      </c>
+      <c r="F123" t="inlineStr"/>
+      <c r="G123" t="inlineStr">
+        <is>
+          <t>San Diego, CA</t>
+        </is>
+      </c>
+      <c r="H123" t="inlineStr"/>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>Lensa is a career site that helps job seekers find great jobs in the US. We are not a staffing firm or agency. Lensa does not hire directly for these jobs, but promotes jobs on LinkedIn on behalf of its direct clients, recruitment ad agencies, and marketing partners. Lensa partners with DirectEmployers to promote this job for SAIC. Clicking "Apply Now" or "Read more" on Lensa redirects you to the job board/employer site. Any information collected there is subject to their terms and privacy notice.
+**Description**
+ SAIC is seeking a
+ **TS/SCI cleared Data Engineer** 
+ in support of NAVWAR's Naval Operational Architecture (NOA) program in San Diego, CA. The Data Engineer will to support a transformational, Navy\-led network\-centric initiative that converges existing systems, automating the correlation of multiple ISR data streams, dramatically reducing the "sensor\-to\-shooter" timeline. This is a recently awarded contract, funded for five years.
+**Work is performed on site in San Diego, CA.**
+ Please view our program page for more information and to view all open positions available: https://jobs.saic.com/pages/NOA
+**Job Duties**
+* Build and optimize robust data pipelines: ingestion, transformation, storage, and governance.
+* Convert between tactical data formats, e.g., XML, JSON, GEOJSON, Cursor\-on\-Target (CoT), JREAP\-C, Link\-16\.
+* Implement automation using CHRON/CRON jobs and data orchestration frameworks (Apache Airflow, Kafka, AWS Step Functions).
+* Architect and maintain scalable data stores (e.g., Apache Iceberg, Elasticsearch) with schema evolution and deduplication.
+* Enable real\-time data indexing and fast query performance.
+* Implement MIL\-STD\-6016 (Link\-16\) and MIL\-STD\-3011 (JREAP) message handling.
+* Support integration or development of Cross\-Domain Solutions (CDS) for secure, policy\-based data transfers.
+* Present complex data flows and technical insights effectively to leadership and stakeholders using clear data models and visual aids.
+**Qualifications**
+**Citizenship and Clearance Requirement:**
+* U.S. Citizenship required.
+* Active TS/SCI security clearance required.
+**Education And Certification Requirements**
+* Bachelor's degree in Data Science, Computer Science, Engineering, or related STEM field.
+**Required Skills And Experience**
+* 5 \- 10 years' experience working as a business analyst, data analyst, data scientist, data engineer, database administrator, geospatial analyst, geospatial engineer, machine learning engineer, or software engineer.
+* Hands on Keyboard\- Developer Skillsets.
+* Fluency in Python, can code without Modern libraries.
+* Experience in format conversions with some of the following: XML, JREAP\-C, COT (cursor\-on\-target), JSON, GEO JSON, UMF/UHR, text link\-16, Tapil\-J, and other Tactical Data Links.
+* Experience in natural language parsing (NLP) and using regular expressions, RegEx.
+* Experience implementing CHRON/CRON jobs.
+* Experience in data pipeline orchestration, ETL, orchestration tools (e.g., Kafka, Apache Airflow, AWS Step Functions).
+* Focused experience implementing and monitoring data stores i.e. (Apache Iceberg, elastic search, data lake management).
+* Experience with schema evolution, dataflow and governance.
+* Experience with real\-time search and analytics engines for indexing and querying semi\-structured data.
+* Focused experience optimizing data store queries for speed and deduplication.
+* Direct experience implementing MIL\-STD\-6016 and MIL\-STD\-3011\.
+* Can translate data between source and destination schemas.
+* Data modeling and PowerPoint presentations for leadership and stakeholder presentations.
+* Experience working with or developing Cross Domain Solutions (CDS) systems.
+**Preferred Skills And Experience**
+* Familiarity with DoD data architecture principles (e.g. DoDAF, CADM).
+* Experience with DataOps or similar mission\-critical pipeline automation (e.g., deduplication, schema normalization).
+* Any experience leveraging universal data distribution architectures within DOD operations.
+ Target salary range: $120,001 \- $160,000\. The estimate displayed represents the typical salary range for this position based on experience and other factors.
+ REQNUMBER: 2600839
+ SAIC is a premier technology integrator, solving our nation's most complex modernization and systems engineering challenges across the defense, space, federal civilian, and intelligence markets. Our robust portfolio of offerings includes high\-end solutions in systems engineering and integration; enterprise IT, including cloud services; cyber; software; advanced analytics and simulation; and training. We are a team of 23,000 strong driven by mission, united purpose, and inspired by opportunity. Headquartered in Reston, Virginia, SAIC has annual revenues of approximately $6\.5 billion. For more information, visit saic.com. For information on the benefits SAIC offers, see Working at SAIC. EOE AA M/F/Vet/Disability
+ If you have questions about this posting, please contact support@lensa.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>li-4373239705</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>Jr Data Engineer</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>Lensa</t>
+        </is>
+      </c>
+      <c r="D124" t="inlineStr">
+        <is>
+          <t>linkedin</t>
+        </is>
+      </c>
+      <c r="E124">
+        <f>HYPERLINK("https://www.linkedin.com/jobs/view/4373239705", "https://www.linkedin.com/jobs/view/4373239705")</f>
+        <v/>
+      </c>
+      <c r="F124">
+        <f>HYPERLINK("https://lensa.com/cgw/a589e7e764d54b6dbd6a3754f87943b7tjo1?jpsi=directemployers&amp;publisher_preference=easier_apply&amp;utm_campaign=Computer%20Occupations&amp;utm_medium=slot&amp;utm_source=linkedin&amp;utm_term=jse&amp;urlHash=qpQS", "https://lensa.com/cgw/a589e7e764d54b6dbd6a3754f87943b7tjo1?jpsi=directemployers&amp;publisher_preference=easier_apply&amp;utm_campaign=Computer%20Occupations&amp;utm_medium=slot&amp;utm_source=linkedin&amp;utm_term=jse&amp;urlHash=qpQS")</f>
+        <v/>
+      </c>
+      <c r="G124" t="inlineStr">
+        <is>
+          <t>Chantilly, VA</t>
+        </is>
+      </c>
+      <c r="H124" t="inlineStr"/>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>Lensa is a career site that helps job seekers find great jobs in the US. We are not a staffing firm or agency. Lensa does not hire directly for these jobs, but promotes jobs on LinkedIn on behalf of its direct clients, recruitment ad agencies, and marketing partners. Lensa partners with DirectEmployers to promote this job for Accenture. Clicking "Apply Now" or "Read more" on Lensa redirects you to the job board/employer site. Any information collected there is subject to their terms and privacy notice.
+ At Accenture Federal Services, nothing matters more than helping the US federal government make the nation stronger and safer and life better for people. Our 13,000\+ people are united in a shared purpose to pursue the limitless potential of technology and ingenuity for clients across defense, national security, public safety, civilian, and military health organizations.
+ Join Accenture Federal Services, a technology company and part of global Accenture, to do work that matters in a collaborative and caring community, where you feel like you belong and are empowered to grow, learn and thrive through hands\-on experience, certifications, industry training and more.
+ Join us to drive positive, lasting change that moves missions and the government forward!
+**You Are**
+ A team player with an entrepreneurial mind. You have a strong record of leadership in an academic, professional, and/or extracurricular settings. You step up and volunteer to take on challenges to solve technical and strategic problems. Unafraid to experiment and drawn to problem solving. You are willing to share your ideas and work collaboratively in a team environment. You look closely at the way things work and often see a better approach to how it could be done You have excellent analytical and quantitative problem\-solving skills and thrive in the unknown and naturally a problem\-solver. You can see all around that the world is changing. You are ready to stretch boundaries –– and yourself.
+**The Work**
+* Learn first\-hand how we help the federal government develop and implement their tech strategy, as well as how we manage our business to help maximize business outcomes for both our clients and Accenture
+* Work with a diverse group of people across many different technologies
+* Connect with your teammates to design and develop new technology product features
+* Bridge the gap between technology and business by using your analytical expertise
+* Develop front end solutions to design, develop, test and implement software
+* Identifying and implementing process improvements to help deliver value
+* Manage deadlines diligently, working with your team to achieve project milestones
+* Support project management by reporting issues, risks, and status, and by assisting with financial activities as needed
+**Here’s What You Need**
+* Bachelor’s degree or Master’s degree
+**Bonus Points If You Are One Or More**
+* Experience in application design using prototyping tools such as Adobe XD,Axure, Balsamiq, Sketch, etc
+* Good working knowledge of Microsoft Suite (including Outlook, PowerPoint, Access, SharePoint, Project, Word)
+* Experience with software configuration(Microsoft PowerApps, SharePoint, etc.) or eCommerce platform configuration (Shopify, Squarespace, Wix, etc.)
+* Exposure to systems withAppian, Salesforce, SAP, ServiceNow, Oracle, Pega, or PeopleSoft components
+* Exposure to Agile methods and tools, such as Jira
+* Are known for being analytical, looking at things from all angles
+* Are resourceful and intellectually curious
+* Able to communicate complex ideas effectively – both verbally and in writing
+**Security Clearance**
+* Active TS/SCI with polygraph clearance
+ As required by local law, Accenture Federal Services provides reasonable ranges of compensation for hired roles based on labor costs in the states of
+ **California, Colorado, Hawaii, Illinois, Maryland,** 
+**Massachusetts,** 
+**Minnesota, New Jersey, New York, Washington, Vermont, the District of Columbia, and the city of Cleveland** 
+ . The base pay range for this position in these locations is shown below. Compensation for roles at Accenture Federal Services varies depending on a wide array of factors, including but not limited to office location, role, skill set, and level of experience. Accenture Federal Services offers a wide variety of benefits. You can find more information on benefits here. (https://www.accenture.com/us\-en/careers/your\-future\-rewards\-benefits) We accept applications on an on\-going basis and there is no fixed deadline to apply.
+ The Pay Range For The States Of California, Colorado, Hawaii, Illinois, Maryland, Massachusetts, Minnesota, New Jersey, New York, Washington, Vermont, The District Of Columbia, And The City Of Cleveland Is
+ $75,500—$131,200 USD
+**What We Believe**
+*As a company wholly dedicated to serving the US federal government, we bring together the best talent to help reinvent how federal agencies operate and deliver greater value for their mission and the American people. We have an unwavering commitment to creating a culture in which all our people are respected, feel a sense of belonging, and have equal opportunity. As a business imperative, every person at Accenture Federal Services has the responsibility to create and sustain a culture where everyone feels welcomed and included. This is grounded in our core values and our experience that hiring and developing great people who reflect different perspectives, experiences, and backgrounds is key to driving innovation and delivering the results that our clients and the country count on.*
+***Equal Employment Opportunity Statement***
+*We believe that no one should be discriminated against because of their differences. All employment decisions shall be made without regard to age, race, creed, color, religion, sex, national origin, ancestry, disability status, veteran status, sexual orientation, gender identity or expression, genetic information, marital status, citizenship status or any other basis as protected by federal, state, or local law. Our rich diversity makes us more innovative, more competitive, and more creative, which helps us better serve our clients and our communities. For details, view a copy of the Accenture Federal Services Equal Opportunity Policy Statement. (https://afscommunities.force.com/careers/s/equal\-opportunity\-annual\-policy)*
+*Accenture Federal Services is an Equal Employment Opportunity employer. Additionally, as an Affirmative Action Employer for Veterans and Individuals with Disabilities, Accenture Federal Services is committed to providing veteran employment opportunities to our service men and women.*
+***Requesting An Accommodation***
+*Accenture Federal Services is committed to providing equal employment opportunities for persons with disabilities or religious observances, including reasonable accommodation when needed. If you are hired by Accenture Federal Services and require accommodation to perform the essential functions of your role, you will be asked to participate in our reasonable accommodation process. Accommodations made to facilitate the recruiting process are not a guarantee of future or continued accommodations once hired.*
+*If you* 
+**\_ \_** 
+*are being considered for employment opportunities with Accenture Federal Services and need an accommodation for a disability or religious observance during the interview process or for the job you are interviewing for, please speak with your recruiter.*
+**Other Employment Statements**
+*Applicants for employment in the US must have work authorization that does not now or in the future require sponsorship of a visa for employment authorization in the United States.*
+*Candidates who are currently employed by a client of Accenture Federal Services or an affiliated Accenture business may not be eligible for consideration.*
+*Job candidates will not be obligated to disclose sealed or expunged records of conviction or arrest as part of the hiring process.*
+*The Company will not discharge or in any other manner discriminate against employees or applicants because they have inquired about, discussed, or disclosed their own pay or the pay of another employee or applicant. Additionally, employees who have access to the compensation information of other employees or applicants as a part of their essential job functions cannot disclose the pay of other employees or applicants to individuals who do not otherwise have access to compensation information, unless the disclosure is (a) in response to a formal complaint or charge, (b) in furtherance of an investigation, proceeding, hearing, or action, including an investigation conducted by the employer, or (c) consistent with the Company's legal duty to furnish information.*
+*California requires additional notifications for applicants and employees. If you are a California resident, live in or plan to work from Los Angeles County upon being hired for this position, please click here (https://www.accenture.com/us\-en/careers/life\-at\-accenture/e\-verify\-legal\-notices) for additional important information.*
+ If you have questions about this posting, please contact support@lensa.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>li-4373230126</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>Data Engineer I/II</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>Wiraa</t>
+        </is>
+      </c>
+      <c r="D125" t="inlineStr">
+        <is>
+          <t>linkedin</t>
+        </is>
+      </c>
+      <c r="E125">
+        <f>HYPERLINK("https://www.linkedin.com/jobs/view/4373230126", "https://www.linkedin.com/jobs/view/4373230126")</f>
+        <v/>
+      </c>
+      <c r="F125" t="inlineStr"/>
+      <c r="G125" t="inlineStr"/>
+      <c r="H125" t="inlineStr"/>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>**About The Company**
+ BNSF Railway is one of the largest freight railroads in the United States, operating across 28 western states and extending into three Canadian provinces. The company is committed to safety, inclusion, and excellence, playing a vital role in transporting essential products and materials that support communities nationwide and globally. As a member of our team, you will contribute to the movement of goods that feed, clothe, supply, and power communities, ensuring the seamless flow of commerce and daily life. BNSF is dedicated to fostering a culture of diversity, innovation, and continuous improvement, making it an ideal environment for professionals seeking impactful careers in the transportation sector.
+**About The Role**
+ We are seeking a highly skilled Data \&amp; AI Engineer to join our innovative BNSF \| Tech division, which is focused on transforming data assets into real\-time enterprise solutions. This remote position offers an exciting opportunity to lead the design, development, and implementation of data streaming solutions, data pipelines, and large\-scale data warehouses. The role involves collaborating with data scientists, analysts, and stakeholders to understand data requirements and deliver effective, scalable data solutions that support business intelligence and analytics. The ideal candidate will be responsible for ensuring data security, compliance, and performance optimization, while staying current with industry trends in data engineering, machine learning, and data science. This position provides a unique chance to influence the future of freight rail through data\-driven innovation, working from anywhere within the contiguous United States.
+**Qualifications**
+* Authorized to work in the United States
+* Minimum of 2 years of experience in software engineering, data engineering, or related fields
+* Proficiency in programming languages such as Python, SQL, Java
+* Strong understanding of data warehousing concepts, including dimensional modeling and star schema
+* Experience with ETL processes and cloud\-based solutions
+* Familiarity with database management systems (SQL, NoSQL) and lakehouse technologies (Apache Iceberg, Delta Lake, Apache Trino)
+* Experience with data streaming technologies such as Apache Kafka, AWS Kinesis, Apache Flink, and Apache Spark
+* Knowledge of data pipelines, data orchestration tools, and certified datasets
+* Excellent problem\-solving skills and attention to detail
+* Strong communication and collaboration skills
+* Ability to learn new technologies quickly and adapt to a dynamic environment
+**Responsibilities**
+* Design and implement real\-time data streaming solutions for efficient data processing
+* Develop and maintain robust data pipelines for both real\-time and batch processing, including ETL workflows
+* Create and manage large\-scale data warehouses to support analytics and business intelligence
+* Integrate data from diverse sources to develop certified datasets ensuring accuracy and reliability
+* Collaborate with data scientists, analysts, and stakeholders to understand data requirements and deliver tailored solutions
+* Optimize data workflows, monitor pipelines, and troubleshoot issues to ensure high performance and scalability
+* Ensure data security and compliance with industry standards and regulations
+* Stay updated on industry trends and advancements in data engineering, data science, and machine learning
+* Write efficient, well\-documented code with comprehensive testing and documentation
+* Lead the integration of data engineering solutions into production systems, overseeing design, development, testing, and monitoring
+**Benefits**
+* Industry\-leading 401(k) plan and Railroad Retirement program
+* Comprehensive health care options including medical, dental, vision, telemedicine, and mental health services
+* Health savings accounts (HSA) with employer contributions, life and disability insurance
+* Family benefits such as parental leave, pediatric and family building support, adoption and surrogacy reimbursement, and dependent care accounts
+* Discounts on travel, gym memberships, counseling, and wellness programs
+* Annual incentive bonus program
+* Generous paid time off and leave policies
+* Resources and support for professional development and career growth
+ Equal Opportunity
+ BNSF Railway is an Equal Opportunity Employer. We are committed to creating an inclusive environment where all qualified applicants receive consideration for employment without regard to race, color, religion, sex, sexual orientation, gender identity, national origin, disability, veteran status, or any other protected characteristic. We encourage individuals from diverse backgrounds to apply and contribute to our culture of safety, inclusion, and excellence.</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>li-4373211737</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>Data Engineer</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>Wiraa</t>
+        </is>
+      </c>
+      <c r="D126" t="inlineStr">
+        <is>
+          <t>linkedin</t>
+        </is>
+      </c>
+      <c r="E126">
+        <f>HYPERLINK("https://www.linkedin.com/jobs/view/4373211737", "https://www.linkedin.com/jobs/view/4373211737")</f>
+        <v/>
+      </c>
+      <c r="F126" t="inlineStr"/>
+      <c r="G126" t="inlineStr"/>
+      <c r="H126" t="inlineStr"/>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>**About The Company**
+ Join the Future of Commerce with Whatnot! Whatnot is the largest live shopping platform operating across North America and Europe, revolutionizing the way people buy, sell, and discover their passions. By seamlessly blending community engagement, entertainment, and e\-commerce, Whatnot offers a unique marketplace experience that caters to a diverse range of interests, including fashion, beauty, electronics, collectibles such as trading cards and comic books, and even live plants. The platform is designed to foster a vibrant community where users can participate in live auctions and connect over shared interests. With a strong emphasis on innovation and a values\-driven culture, Whatnot operates as a remote co\-located team with hubs in the US, UK, Germany, Ireland, and Poland, dedicated to building the future of online marketplaces. As one of the fastest\-growing marketplaces, Whatnot is committed to enabling individuals to turn their passions into thriving businesses and bringing people together through commerce.
+**About The Role**
+ As a Data Engineer at Whatnot, you will play a critical role in shaping the company's data infrastructure to support data\-driven decision\-making and business growth. You will be responsible for designing, building, and maintaining scalable, reliable, and efficient data systems that serve various internal teams such as product, sales, marketing, finance, and trust. Your work will involve creating robust data architectures, developing resilient data pipelines, and building foundational data products that power analytics, machine learning, and real\-time applications. You will own the entire data lifecycle—from capturing and modeling data to ensuring high data quality and operational efficiency. Collaborating closely with cross\-functional teams, you will help establish standards and best practices for data management, ensuring that data is accessible, accurate, and actionable across the organization. Your contributions will directly influence the company's ability to innovate, optimize operations, and enhance user experience.
+**Qualifications**
+* 3\+ years of experience as a data or software engineer, specializing in building data warehouses, distributed data systems, or event\-driven architectures.
+* Proficiency in designing and implementing data models using techniques such as dimensional modeling, Data Vault, or ledger\-style approaches.
+* Hands\-on experience with modern data tooling including Kafka, Debezium, dbt, Spark, Flink, Dagster, Airflow, Monte Carlo, and Great Expectations.
+* Experience operating cloud data warehouses such as Snowflake, BigQuery, or Redshift, including schema design, cost management, and workload tuning.
+* Strong coding skills in Python and SQL, with experience integrating with CI/CD pipelines and infrastructure\-as\-code workflows.
+* Ability to translate complex business requirements into scalable and efficient data systems through collaboration across disciplines such as engineering, product, and analytics.
+* Self\-motivated with the ability to manage multiple priorities in a fast\-paced environment, owning both technical and operational outcomes.
+**Responsibilities**
+* Design and implement end\-to\-end data architecture, including data capture, modeling, and serving strategies to support business needs.
+* Develop and operate streaming and batch data pipelines that process high\-volume events with guarantees for latency, completeness, and accuracy.
+* Create domain\-oriented data models that act as authoritative sources for analytics, machine learning, and real\-time applications.
+* Build and maintain data quality systems, including tests, lineage tracking, monitoring, and anomaly detection to ensure dataset reliability.
+* Automate operational workflows by partnering with business systems and platform teams to reduce manual data handoffs and reconcile data across systems.
+* Support analytics, ML, and product teams by providing high\-quality, low\-latency data access through semantic layers, APIs, and real\-time query systems.
+* Establish and enforce data modeling standards, ownership boundaries, and data contracts across teams to ensure consistency and compliance.
+* Continuously evaluate and optimize data storage formats, compute patterns, and SLAs balancing cost, scalability, and data integrity.
+**Benefits**
+* Generous holiday and time\-off policies to support work\-life balance.
+* Comprehensive health insurance options including Medical, Dental, and Vision coverage.
+* Support for remote work with home office setup allowances and monthly stipends for cell phone and internet expenses.
+* Care benefits including wellness allowances, annual childcare allowances, and lifetime family planning benefits.
+* Retirement plans such as 401(k) with employer matching in the US, and pension plans internationally.
+* Additional perks like monthly allowances for app testing (dogfooding), parental leave (16 weeks paid parental leave plus a gradual return), and a culture of continuous development and engagement.
+ Equal Opportunity
+ Whatnot is proud to be an Equal Opportunity Employer. We value diversity and are committed to creating an inclusive environment for all employees. We do not discriminate based on race, religion, color, national origin, gender, sexual orientation, age, marital status, veteran status, parental status, disability status, or any other protected characteristic under applicable law. We believe that embracing diversity enhances our work culture and drives innovation, and we actively encourage candidates from all backgrounds to apply.</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>li-4372088744</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>Data Engineer</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>CDC Foundation</t>
+        </is>
+      </c>
+      <c r="D127" t="inlineStr">
+        <is>
+          <t>linkedin</t>
+        </is>
+      </c>
+      <c r="E127">
+        <f>HYPERLINK("https://www.linkedin.com/jobs/view/4372088744", "https://www.linkedin.com/jobs/view/4372088744")</f>
+        <v/>
+      </c>
+      <c r="F127" t="inlineStr"/>
+      <c r="G127" t="inlineStr"/>
+      <c r="H127" t="inlineStr"/>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>**Data Engineer\-Synapse Analytics** 
+**Job Description** 
+**Overview** 
+ The Senior Data Engineer will play a crucial role in advancing the CDC Foundation's mission by designing, building, and maintaining data infrastructure for a public health organization. This role is aligned to the Workforce Acceleration Initiative (WAI). WAI is a federally funded CDC Foundation program with the goal of helping the nation’s public health agencies by providing them with the technology and data experts they need to accelerate their information system improvements.
+ Working within Prince George’s County Health Department, the Senior Data Engineer will support the development and operation of the enterprise data platform by building and maintaining data pipelines, supporting data ingestion and transformation, and enabling analytics and reporting use cases. This role collaborates closely with IT, data analysts, and program stakeholders to ensure data is reliable, accessible, and aligned with public health business needs.
+ The Senior Data Engineer serves as a senior technical contributor supporting the modernization of PGCHD’s enterprise data platform. The role focuses on designing and implementing data engineering solutions, supporting data ingestion and transformation, and enabling analytics and reporting capabilities across public health programs.
+ The Senior Data Engineer will be hired by the CDC Foundation and assigned to the Prince George’s County Health Department. This position is eligible for a fully remote work arrangement for U.S. based candidates.
+**Responsibilities** 
+ Azure Synapse \&amp; Medallion Architecture
+* Design and implement Azure Synapse Analytics solutions using Spark pools, dedicated and serverless SQL pools
+* Implement and operationalize Medallion Architecture (Bronze, Silver, Gold) layers within Azure Data Lake Storage Gen2 (ADLS).
+* Develop reusable, parameter\-driven data pipelines leveraging Synapse pipelines and Azure Data Factory–style orchestration.
+ Data Ingestion, Transformation \&amp; Modeling
+* Ingest and integrate data from diverse internal and external public health sources (clinical, operational, surveillance, census, and partner data).
+* Build Spark\-based transformations and SQL\-based data models to cleanse, standardize, and enrich data.
+* Design and maintain dimensional and analytical data models optimized for reporting, dashboards, and advanced analytics.
+ Performance, Reliability \&amp; Cost Optimization
+* Monitor, troubleshoot, and tune Synapse workloads for performance, scalability, and cost efficiency.
+* Identify and resolve data pipeline failures, data quality issues, and processing bottlenecks.
+* Implement logging, monitoring, and alerting for production\-grade data pipelines.
+ Data Governance, Security \&amp; Compliance
+* Implement data governance, metadata management, and lineage using Microsoft Purview.
+* Support compliance with public health data security, privacy, and regulatory requirements (HIPAA, CDC guidance, and county policies).
+* Apply role\-based access control (RBAC) and data protection best practices across Azure resources.
+ Collaboration \&amp; Stakeholder Engagement
+* Partner with public health program leaders, analysts, epidemiologists, and informatics teams to translate defined business needs into technical solutions
+* Ensure data products are analytics\-ready and aligned with reporting, performance management, and decision\-support needs.
+* Communicate technical concepts, progress, and recommendations clearly to both technical and non\-technical stakeholders.
+ Engineering Standards \&amp; Knowledge Transfer
+* Apply data engineering best practices including source control, CI/CD, automated testing, documentation, and code reviews.
+* Provide technical guidance related to data engineering implementations and best practices
+* Support documentation and knowledge sharing to promote sustainability of data solutions
+* Stay current on Azure data platform capabilities and data engineering trends relevant to public health use cases
+**Required Qualifications** 
+* Bachelor’s degree in Computer Science, Information Technology, Data Science, or a related field.
+* Minimum 5 years of professional experience in data engineering, analytics engineering, or data warehousing roles.
+* Hands\-on experience with Microsoft Azure data services, particularly Azure Synapse Analytics and ADLS Gen2\.
+* Strong proficiency in SQL and at least one programming language such as Python, Scala, or Java.
+* Experience developing Spark\-based data transformations and scalable ETL/ELT pipelines.
+* Solid understanding of data warehousing concepts, dimensional modeling, and analytics\-oriented data design.
+* Experience implementing engineering best practices such as source control, CI/CD pipelines, automated testing, and peer review.
+* Familiarity with agile development methodologies and modern software design patterns.
+* Strong analytical, troubleshooting, and problem\-solving skills.
+* Excellent written and verbal communication skills, with the ability to explain technical concepts to non\-technical audiences.
+* Experience collaborating with distributed and remote teams.
+* Up to 10% domestic travel may be required.
+**Preferred Qualifications** 
+* Experience working with public health, healthcare, or government data environments.
+* Familiarity with Microsoft Purview for data governance and lineage.
+* Experience supporting Power BI or other analytics and visualization tools.
+* Knowledge of HIPAA, public health data standards, and regulatory compliance.
+* Prior experience designing enterprise\-scale Azure data platforms using Medallion or Lakehouse architectures.
+**Job Highlights** 
+* Location: Remote, must be based in the United States, Up to 10% domestic travel may be required.
+* Salary Range: $103,500\-$143,500 per year, plus benefits. Individual salary offers will be based on experience and qualifications unique to each candidate.
+* Position Type: Grant funded, limited\-term opportunity
+* Position End Date: June 30, 2027</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>li-4373246176</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>Lead Data Engineer - Clinical AI</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>Qualified Health</t>
+        </is>
+      </c>
+      <c r="D128" t="inlineStr">
+        <is>
+          <t>linkedin</t>
+        </is>
+      </c>
+      <c r="E128">
+        <f>HYPERLINK("https://www.linkedin.com/jobs/view/4373246176", "https://www.linkedin.com/jobs/view/4373246176")</f>
+        <v/>
+      </c>
+      <c r="F128" t="inlineStr"/>
+      <c r="G128" t="inlineStr"/>
+      <c r="H128" t="inlineStr"/>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>**Transform healthcare with us.**
+ At Qualified Health, we’re redefining what’s possible with Generative AI in healthcare. Our infrastructure provides the guardrails for safe AI governance, healthcare\-specific agent creation, and real\-time algorithm monitoring—working alongside leading health systems to drive real change.
+ This is more than just a job. It’s an opportunity to build the future of AI in healthcare, solve complex challenges, and make a lasting impact on patient care. If you’re ambitious, innovative, and ready to move fast, we’d love to have you on board.
+**Join us in shaping the future of healthcare.**
+**Job Summary:**
+ Qualified Health is seeking a Principal (Lead) Data Engineer to lead the development of our clinical intelligence layer. In this senior technical role, you'll design and build the data transformation pipelines that convert raw clinical data into AI\-ready features, enabling our platform to deliver faster, more accurate clinical insights. You'll work closely with clinical SMEs to translate medical knowledge into scalable data systems, and partner with our AI team to define the data contracts that power LLM\-based workflows.
+ This is a technical leadership role for someone who thrives on solving complex data challenges and takes pride in building reliable, production\-grade systems.
+**Key Responsibilities:**
+**Clinical Data Transformation (60%)**
+* **Design and build clinical annotation pipelines** 
+ that extract conditions, medications, and procedures from unstructured clinical notes
+* **Implement negation and temporal detection** 
+ to distinguish current conditions from historical findings (critical for clinical decision\-making)
+* **Build business rules engines** 
+ that classify medications, calculate risk scores, and apply clinical logic at scale
+* **Integrate clinical reference data** 
+ (drug databases, terminology mappings) into transformation pipelines
+* **Optimize data structures** 
+ to reduce LLM processing time and improve downstream AI performance
+**Platform Engineering (30%)**
+* **Build production\-grade pipelines** 
+ using PySpark and Databricks for large\-scale clinical data processing
+* **Implement data quality frameworks** 
+ to validate clinical transformations and catch issues before they reach AI workflows
+* **Design feature stores** 
+ that serve pre\-computed clinical features to ML models and LLM applications
+* **Maintain pipeline observability** 
+ with monitoring, alerting, and performance tracking
+**Collaboration (10%)**
+* **Partner with clinical SMEs** 
+ to translate medical knowledge into data transformation logic
+* **Define data contracts** 
+ with AI team to ensure feature outputs meet LLM workflow requirements
+* **Contribute to technical standards and best practices for clinical data engineering**
+**Required Qualifications:**
+* **8\+ years of data engineering experience** 
+ , with demonstrated expertise building production data pipelines
+* **5\+ years on Databricks** 
+ , including PySpark, Delta Lake, and Unity Catalog
+* **Healthcare data experience** 
+ : Prior work with FHIR APIs, EHR databases, or claims data
+* **Clinical text processing experience** 
+ : Built pipelines that extract entities from unstructured clinical notes using tools like spaCy, medspaCy, or cloud NLP services
+* **Feature engineering for ML/AI** 
+ : Experience preparing data for machine learning models or LLM consumption
+* **Data quality mindset** 
+ : Track record implementing validation frameworks and monitoring for data pipelines
+* **Healthcare terminology** 
+ : Familiarity with ICD\-10, RxNorm, SNOMED CT, LOINC
+* **Epic Clarity experience** 
+ : Direct work with Epic's relational database structure
+**Desirable Skills:**
+* **Azure cloud platform** 
+ : Hands\-on with Azure Databricks, Data Lake Storage, Service Bus
+* **Clinical NLP tools** 
+ : Experience with Azure Text Analytics for Health, Amazon Comprehend Medical, or similar
+* **RAG architecture patterns** 
+ : Understanding of vector databases and retrieval\-augmented generation
+**Why Join Qualified Health?**
+ This is an opportunity to join a fast\-growing company and a world\-class team, that is poised to change the healthcare industry. We are a passionate, mission\-driven team that is building a category\-defining product. We are backed by premier investors and are looking for founding team members who are excited to do the best work of their careers.
+ Our employees are integral to achieving our goals so we are proud to offer competitive salaries with equity packages, robust medical/dental/vision insurance, flexible working hours, hybrid work options and an inclusive environment that fosters creativity and innovation.
+**Our Commitment to Diversity**
+ Qualified Health is an equal opportunity employer. We believe that a diverse and inclusive workplace is essential to our success, and we are committed to building a team that reflects the world we live in. We encourage applications from all qualified individuals, regardless of race, color, religion, gender, sexual orientation, gender identity or expression, age, national origin, marital status, disability, or veteran status.
+**Pay \&amp; Benefits:** 
+ The pay range for this role is between $160,000 and $210,000, and will depend on your skills, qualifications, experience, and location. This role is also eligible for equity and benefits.
+***Join our mission to revolutionize healthcare with AI.***
+ To apply, please send your resume through the application below.</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>li-4373254316</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>Senior Data Engineer</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>undisclosed</t>
+        </is>
+      </c>
+      <c r="D129" t="inlineStr">
+        <is>
+          <t>linkedin</t>
+        </is>
+      </c>
+      <c r="E129">
+        <f>HYPERLINK("https://www.linkedin.com/jobs/view/4373254316", "https://www.linkedin.com/jobs/view/4373254316")</f>
+        <v/>
+      </c>
+      <c r="F129" t="inlineStr"/>
+      <c r="G129" t="inlineStr"/>
+      <c r="H129" t="inlineStr"/>
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>**Overview** 
+ Our client is seeking a
+ **Senior Data Engineer** 
+ to design, build, and maintain scalable data platforms and pipelines that power analytics, reporting, and data\-driven decision\-making across the organization. This role plays a critical part in transforming raw data into reliable, high\-quality datasets used by Product, Analytics, Data Science, and business teams.
+ The ideal candidate is a hands\-on data expert with strong experience in modern data architectures, cloud platforms, and large\-scale data processing, who thrives in a collaborative, fast\-paced environment.
+**Key Responsibilities** 
+* Design, develop, and maintain scalable, reliable, and efficient data pipelines and ETL/ELT processes.
+* Build and optimize data models, data warehouses, and data lakes to support analytics and business intelligence use cases.
+* Collaborate closely with Analytics, Data Science, Product, and Engineering teams to understand data requirements and deliver trusted datasets.
+* Ensure data quality, accuracy, availability, and consistency through validation, monitoring, and testing.
+* Optimize data performance, cost, and scalability across storage and processing systems.
+* Implement and enforce data engineering best practices, including documentation, version control, and code reviews.
+* Support real\-time and batch data processing use cases.
+* Identify and resolve data pipeline failures, performance bottlenecks, and reliability issues.
+* Work with DevOps and Platform teams to improve CI/CD workflows, automation, and infrastructure\-as\-code for data systems.
+* Contribute to the evolution of the organization’s data architecture and long\-term data strategy.
+**Operating Context** 
+* Operates within a modern, cloud\-based data ecosystem.
+* Works closely with cross\-functional teams including Engineering, Analytics, Data Science, Product, and Business stakeholders.
+* Balances hands\-on development with architectural planning and technical leadership.
+* Typically works in a remote or hybrid environment using modern collaboration tools.
+* Reports to Data Engineering leadership, Engineering Management, or Platform leadership.
+**Required Skills** 
+* Strong experience building and maintaining production\-grade data pipelines.
+* Proficiency in SQL and at least one programming language such as Python, Java, or Scala.
+* Experience with data warehousing and analytics platforms (e.g., Snowflake, BigQuery, Redshift).
+* Solid understanding of data modeling, schema design, and performance optimization.
+* Experience with batch and streaming data processing frameworks.
+* Familiarity with REST APIs, data integrations, and third\-party data sources.
+* Strong problem\-solving skills and attention to data quality and reliability.
+* Excellent communication and collaboration skills.
+**Preferred Qualifications** 
+* 5–8\+ years of professional experience in data engineering or related roles.
+* Experience in
+ **SaaS, cloud\-native, or data\-driven product organizations** 
+ .
+* Hands\-on experience with cloud platforms such as
+ **AWS, Azure, or GCP** 
+ .
+* Experience with tools such as Airflow, dbt, Spark, Kafka, or similar technologies.
+* Exposure to DevOps practices, CI/CD pipelines, and infrastructure\-as\-code.
+* Bachelor’s degree in Computer Science, Engineering, or a related field, or equivalent practical experience.
+**Success Metrics** 
+* Reliable, scalable, and well\-documented data pipelines running in production.
+* High data quality and trust in analytics and reporting outputs.
+* Improved performance, cost efficiency, and scalability of data systems.
+* Strong collaboration with Analytics, Data Science, and Product teams.
+* Measurable impact on business insights, reporting accuracy, and decision\-making.
+**Job Function** 
+ Data Engineering / Software Engineering / Analytics Engineering
+**Industry** 
+ Information Technology \&amp; Services, SaaS, Cloud Computing, Data \&amp; Analytics
+**Please Read Before Applying** 
+ This posting is part of the
+ **MobiusEngine.ai Talent Network** 
+ and is not a single, guaranteed position at one specific company.
+ By applying, you:
+* Join our candidate network for current and future opportunities with our hiring partners
+* May receive feedback on your resume and job search approach
+* Will be contacted directly when a live opportunity matches your background and preferences
+-</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>li-4373246627</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>Software Developer/Data Engineer - Entry Level</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>Lensa</t>
+        </is>
+      </c>
+      <c r="D130" t="inlineStr">
+        <is>
+          <t>linkedin</t>
+        </is>
+      </c>
+      <c r="E130">
+        <f>HYPERLINK("https://www.linkedin.com/jobs/view/4373246627", "https://www.linkedin.com/jobs/view/4373246627")</f>
+        <v/>
+      </c>
+      <c r="F130" t="inlineStr"/>
+      <c r="G130" t="inlineStr">
+        <is>
+          <t>Atlanta, GA</t>
+        </is>
+      </c>
+      <c r="H130" t="inlineStr"/>
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>Lensa is a career site that helps job seekers find great jobs in the US. We are not a staffing firm or agency. Lensa does not hire directly for these jobs, but promotes jobs on LinkedIn on behalf of its direct clients, recruitment ad agencies, and marketing partners. Lensa partners with DirectEmployers to promote this job for CGI Technologies and Solutions, Inc.. Clicking "Apply Now" or "Read more" on Lensa redirects you to the job board/employer site. Any information collected there is subject to their terms and privacy notice.
+**Software Developer/Data Engineer \-\- Entry Level**
+**Category:** 
+ Software Development/ Engineering
+**Main location:** 
+ United States, Georgia, Atlanta
+**Position ID:** 
+ J0825\-1339
+**Employment Type:** 
+ Graduate
+**Position Description**
+ Launch a world\-class career with us.
+ Are you driven by the power of technology and its role in transforming business and government? Do you thrive in collaborative environments and want to build a career that spans impactful solutions across enterprises and agencies? If so, CGI is the place for you.
+ As a Software Developer/Data Engineer, you'll be an integral part of a highly collaborative team, working alongside architects, engineers, and stakeholders to design, build, and deliver software solutions that elevate IT services. At CGI, you're encouraged to explore your full potential, free from predefined boundaries and guided by the unique value of your contributions.
+ This position is in Atlanta, GA in a hybrid working model.
+ Spring Application Period: Monday, January 18th, 2026 \- Friday, February 27th, 2026
+**Your Future Duties And Responsibilities**
+ How You'll Make an Impact
+* Design, prototype, and develop front\-end, back\-end, and full\-stack software using modern languages and frameworks (e.g., .NET, Java, open\-source stacks, React).
+* Apply software design patterns and best practices for scalable, maintainable code.
+* Collaborate with team members to continuously improve approaches and tools.
+* Build database\-integrated and data\-enabled solutions, including ETL pipelines, using contemporary database technologies.
+* Deliver analytics and reporting solutions by working with data models, queries, and visualizations.
+* Contribute to projects that leverage AI or machine learning capabilities within software and data solutions.
+* Conduct peer code reviews, participate in Agile rituals, and contribute to engineering discussions.
+* Support quality assurance by understanding its value, helping craft test plans, and executing test cases.
+* Create technical documentation, including requirement specs, design docs, and user manuals.
+ This role includes opportunities to focus on application development, data and analytics work, or a blend of both, depending on project needs.
+**Required Qualifications To Be Successful In This Role**
+ What You'll Bring
+* Bachelor's degree from an accredited college or university in Computer Science, Computer Engineering, Information Systems or a related technical field
+* Foundational experience in software development (SQL, Java, C\#, .NET, J2EE, C\+\+).
+* Strong ability to learn new frameworks and technologies quickly.
+* A growth\-oriented mindset and a passion for learning.
+* Excellent analytical thinking, and strong written and verbal communication skills.
+* Comfort with ambiguity, adaptability, and team\-oriented collaboration.
+* Ability to work in the U.S. permanently and without restriction.
+**Let's Talk About Benefits**
+* Competitive base salary
+* Comprehensive insurance options
+* 401(k) with company match
+* Share purchase plan with a company match
+* Paid vacation, holidays, and sick leave
+* Up to 14 weeks of Maternity Leave with full pay
+* 4\-week Parental Leave for all non\-birth parents
+* Attorney\-assisted will preparation
+* Health savings account
+* Disability, life, and accidental death insurance
+* Pet insurance
+* Work\-life balance and flexibility
+* Tuition assistance continuous learning opportunities
+* Training, mentoring, and career development
+* Partner assistance program
+* Wellness program
+ The best version of you starts here
+ We're a global company of owners. Over 90,000 partners strong, we bring our diverse backgrounds and perspectives together to solve some of IT and business consulting's toughest problems for some of the world's best companies. Looking for a place that empowers you to explore your full potential and shape your own career? The scale and reach of our impact offer you just that. Join a team of great people, collaborate on meaningful work, and serve the communities you call home while you do it.
+ CGI is required by law in some jurisdictions to include a reasonable estimate of the compensation range for this role. The determination of this range includes various factors not limited to skill set level, experience and training, and licensure and certifications. To support the ability to reward for merit\-based performance, CGI typically does not hire individuals at or near the top of the range for their role. A reasonable estimate of the current range is $57,100 \- $94,200\.
+ \#CGIEarlyCareers
+**What You Can Expect From Us**
+**Together, as owners, let's turn meaningful insights into action.**
+ Life at CGI is rooted in ownership, teamwork, respect and belonging. Here, you'll reach your full potential because...
+ You are invited to be an owner from day 1 as we work together to bring our Dream to life. That's why we call ourselves CGI Partners rather than employees. We benefit from our collective success and actively shape our company's strategy and direction.
+ Your work creates value. You'll develop innovative solutions and build relationships with teammates and clients while accessing global capabilities to scale your ideas, embrace new opportunities, and benefit from expansive industry and technology expertise.
+ You'll shape your career by joining a company built to grow and last. You'll be supported by leaders who care about your health and well\-being and provide you with opportunities to deepen your skills and broaden your horizons.
+ Come join our team\-one of the largest IT and business consulting services firms in the world.
+ Qualified applicants will receive consideration for employment without regard to their race, ethnicity, ancestry, color, sex, religion, creed, age, national origin, citizenship status, disability, pregnancy, medical condition, military and veteran status, marital status, sexual orientation or perceived sexual orientation, gender, gender identity, and gender expression, familial status or responsibilities, reproductive health decisions, political affiliation, genetic information, height, weight, or any other legally protected status or characteristics to the extent required by applicable federal, state, and/or local laws where we do business.
+ CGI provides reasonable accommodations to qualified individuals with disabilities. If you need an accommodation to apply for a job in the U.S., please email the CGI U.S. Employment Compliance mailbox at US\_Employment\_Compliance@cgi.com . You will need to reference the Position ID of the position in which you are interested. Your message will be routed to the appropriate recruiter who will assist you. Please note, this email address is only to be used for those individuals who need an accommodation to apply for a job. Emails for any other reason or those that do not include a Position ID will not be returned.
+ We make it easy to translate military experience and skills! Clickhere (https://cgi\-veterans.jobs/) to be directed to our site that is dedicated to veterans and transitioning service members.
+ All CGI offers of employment in the U.S. are contingent upon the ability to successfully complete a background investigation. Background investigation components can vary dependent upon specific assignment and/or level of US government security clearance held. Dependent upon role and/or federal government security clearance requirements, and in accordance with applicable laws, some background investigations may include a credit check. CGI will consider for employment qualified applicants with arrests and conviction records in accordance with all local regulations and ordinances.
+ CGI will not discharge or in any other manner discriminate against employees or applicants because they have inquired about, discussed, or disclosed their own pay or the pay of another employee or applicant. However, employees who have access to the compensation information of other employees or applicants as a part of their essential job functions cannot disclose the pay of other employees or applicants to individuals who do not otherwise have access to compensation information, unless the disclosure is (a) in response to a formal complaint or charge, (b) in furtherance of an investigation, proceeding, hearing, or action, including an investigation conducted by the employer, or (c) consistent with CGI's legal duty to furnish information.
+ If you have questions about this posting, please contact support@lensa.com</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>li-4372308036</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>Data Engineer - IAM Data Lake (Google Cloud Platform)</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>Jobs via Dice</t>
+        </is>
+      </c>
+      <c r="D131" t="inlineStr">
+        <is>
+          <t>linkedin</t>
+        </is>
+      </c>
+      <c r="E131">
+        <f>HYPERLINK("https://www.linkedin.com/jobs/view/4372308036", "https://www.linkedin.com/jobs/view/4372308036")</f>
+        <v/>
+      </c>
+      <c r="F131">
+        <f>HYPERLINK("https://click.appcast.io/t/luyV6V9S8t1v6vY9nJvFO3EiQ03x1eOo_K4Ku_kulGs=&amp;urlHash=wUpf", "https://click.appcast.io/t/luyV6V9S8t1v6vY9nJvFO3EiQ03x1eOo_K4Ku_kulGs=&amp;urlHash=wUpf")</f>
+        <v/>
+      </c>
+      <c r="G131" t="inlineStr">
+        <is>
+          <t>Irving, TX</t>
+        </is>
+      </c>
+      <c r="H131" t="inlineStr"/>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>Dice is the leading career destination for tech experts at every stage of their careers. Our client, Strategic Staffing Solutions, is seeking the following. Apply via Dice today!
+**Job Title: Data Engineer IAM Data Lake (Google Cloud Platform)**
+**Location:** 
+ Irving, TX (Preferred) \| Ohio (Alternate)
+**Work Type:** 
+ Onsite/Hybrid (as required)
+**Position Overview**
+ We are seeking an experienced
+ **Data Engineer** 
+ to support
+ **IAM Data Lake and Data Engineering initiatives** 
+ , focused on building and enhancing a modern enterprise data lake on the
+ **Google Cloud Platform (Google Cloud Platform)** 
+ . This role requires hands\-on expertise in designing scalable ingestion pipelines, managing big data architectures, and working with both batch and streaming processing frameworks.
+ The ideal candidate will have strong experience with
+ **Google Cloud Platform\-native services** 
+ , big data tooling, and modern data formats, with additional preference for candidates with exposure to
+ **Hadoop/HDFS ecosystems** 
+ .
+**Key Responsibilities**
+* Design, build, and maintain a scalable IAM\-focused Data Lake on Google Cloud Platform.
+* Develop and optimize data pipelines for both batch and real\-time ingestion.
+* Implement ingestion frameworks leveraging Airflow, PySpark, and Google Cloud Platform\-native tools.
+* Build streaming architectures using Pub/Sub, supporting event\-driven ingestion patterns.
+* Apply best practices for schema design, schema evolution, and versioning across data domains.
+* Work with columnar data formats such as Parquet, Avro, and ORC, including compression and performance tuning.
+* Support incremental ingestion and Change Data Capture (CDC) methodologies.
+* Ensure data is properly structured and exposed through curated datasets, APIs, and analytical views.
+* Collaborate with cross\-functional teams to ensure data governance, security, and access controls align with IAM requirements.
+* Contribute to enterprise development standards through CI/CD automation and documentation.
+**Required Skills \&amp; Experience**
+* 4 6\+ years of Data Engineering experience in large\-scale environments.
+* Strong hands\-on experience building Data Lakes on Google Cloud Platform (Google Cloud Platform).
+* Expertise in developing pipelines using:
++ Apache Airflow
++ PySpark
++ Big data processing frameworks
+* Solid knowledge of the Hadoop ecosystem, with HDFS experience highly desirable.
+* Experience with:
++ APIs and data exposure patterns
++ CI/CD pipelines in enterprise environments
++ Data modeling concepts
+* Strong understanding of Google Cloud Platform architecture, including:
++ Bucket structuring and naming standards
++ Lifecycle management policies
++ Access control and security mechanisms
+**Preferred Technical Expertise**
+* Streaming ingestion and event\-driven design using Google Pub/Sub
+* Schema registry and governance practices
+* Knowledge of CDC tools/patterns
+* Familiarity with curated analytical dataset development
+* Experience supporting Identity \&amp; Access Management (IAM) data domains is a plus
+**Tools \&amp; Technologies**
+* Google Cloud Platform (Google Cloud Platform)
+* Airflow
+* PySpark
+* Hadoop / HDFS
+* Pub/Sub
+* Parquet, Avro, ORC
+* CI/CD Automation
+* APIs and Data Services
+**Ideal Candidate Traits**
+* Strong problem\-solving and analytical mindset
+* Comfortable working in complex enterprise environments
+* Able to collaborate effectively across engineering, security, and governance teams
+* Detail\-oriented with a focus on data quality and scalability</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>li-4372301059</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>Lead Data Engineer</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>Jobs via Dice</t>
+        </is>
+      </c>
+      <c r="D132" t="inlineStr">
+        <is>
+          <t>linkedin</t>
+        </is>
+      </c>
+      <c r="E132">
+        <f>HYPERLINK("https://www.linkedin.com/jobs/view/4372301059", "https://www.linkedin.com/jobs/view/4372301059")</f>
+        <v/>
+      </c>
+      <c r="F132">
+        <f>HYPERLINK("https://click.appcast.io/t/Gs1htXrNWMx2OPTaflFhb6PjRFOo4auEYnnGDnPY5AA=&amp;urlHash=VJ4z", "https://click.appcast.io/t/Gs1htXrNWMx2OPTaflFhb6PjRFOo4auEYnnGDnPY5AA=&amp;urlHash=VJ4z")</f>
+        <v/>
+      </c>
+      <c r="G132" t="inlineStr">
+        <is>
+          <t>McLean, VA</t>
+        </is>
+      </c>
+      <c r="H132" t="inlineStr"/>
+      <c r="I132" t="inlineStr">
+        <is>
+          <t>Why choose between doing meaningful work and having a fulfilling life? At MITRE, you can have both. That's because MITRE people are committed to tackling our nation's toughest challenges\-and we're committed to the long\-term well\-being of our employees. MITRE is different from most technology companies. We are a not\-for\-profit corporation chartered to work for the public interest, with no commercial conflicts to influence what we do. The R\&amp;D centers we operate for the government create lasting impact in fields as diverse as cybersecurity, healthcare, aviation, defense, and enterprise transformation. We're making a difference every day\-working for a safer, healthier, and more secure nation and world. Our workplace reflects our values. We offer competitive benefits, exceptional professional development opportunities for career growth, and a culture of innovation that embraces adaptability, collaboration, technical excellence, and people in partnership. If this sounds like the choice you want to make, then choose MITRE \- and make a difference with us.
+**Department Summary:**
+ Join our Enterprise Data Warehouse team as we prepare for a major evolution in technology and process roll\-out across MITRE. This is an exciting time to join the Enterprise Data Warehouse team as the use and gold source for our data evolves and grows exponentially. Your opportunity to make an impact is great as you help our team evolve to cloud\-based hybrid data and real time data access. We are looking for a highly collaborative, team\-oriented person to join us! A "can\-do" and growth\-focused attitude as well as the ability to work across more than one simultaneous project are musts!
+**Roles \&amp; Responsibilities:**
+ Design, develop, and implement robust ETL solutions using Python and PySpark to extract, transform, and load data from various sources into AWS data services.
+ Optimize ETL processes for performance and scalability utilizing AWS Glue, EMR, Step Functions, and Lambda to ensure efficient data processing and timely delivery.
+ Ensure data integrity and quality throughout the ETL process by implementing thorough data validation checks and error handling mechanisms.
+ Manage AWS services such as Glue, EMR, Step Functions, and Lambda, including configuration, monitoring, and troubleshooting to maintain operational excellence.
+ Collaborate with cross\-functional teams including data engineers, data scientists, and business stakeholders to understand data requirements and deliver tailored ETL solutions.
+ Troubleshoot complex technical issues and provide advanced operational support to internal MITRE customers in AWS
+**Basic Qualifications:**
+ Bachelor's degree with eight years' related experience, or a master's degree with six years' related experience, preferably with a technical major such as engineering, computer science, etc.
+ Demonstrated experience in developing ETL pipelines using Python and PySpark, with a strong understanding of data processing techniques.
+ Expertise in SQL for data manipulation, querying, and optimization to work with various database platforms including Postgres, DynamoDB, Oracle, and Redshift.
+ Hands\-on experience with AWS Glue, EMR, Step Functions, and Lambda for building and orchestrating ETL workflows in a cloud environment.
+ Experience implementing Continuous Integration/Continuous Deployment (CI/CD) pipelines using AWS CDK or similar tools for automating deployment and testing of ETL solutions.
+ This position requires a minimum of 60% hybrid on\-site.
+**Preferred Qualifications:**
+ Previous experience leading or mentoring a team of developers/engineers in a collaborative environment.
+ AWS certifications such as AWS Certified Developer or AWS Certified Solutions Architect, demonstrating proficiency in AWS services and best practices.
+ Familiarity with big data technologies such as Apache Spark, Hadoop, or Kafka for processing large\-scale datasets.
+ Experience in data modeling and schema design for optimizing database performance and scalability.
+ Experience working in Agile development methodologies, such as Scrum or Kanban, for iterative and collaborative project delivery.
+ Self\-motivated, curious, and collaborative, with a passion to learn new technologies and develop new skills
+ Proven ability to collaborate effectively and actively participate in cross\-training and team knowledge transfer.
+**This requisition requires the candidate to have a minimum of the following clearance(s):**
+ None
+**This requisition requires the hired candidate to have or obtain, within one year from the date of hire, the following clearance(s):**
+ None
+**Salary compensation range and midpoint:**
+ $144,800 \- $181,000 \- $217,200 Annual
+**Work Location Type:**
+ Hybrid
+**Commitment to Non\-Discrimination**
+ All qualified applicants will receive consideration for employment without regard to disability, status as a protected veteran or any other status protected by applicable federal, state, local or international law.
+ MITRE intends to maintain a website that is fully accessible to all individuals. If you are unable to search or apply for jobs and would like to request a reasonable accommodation for any part of MITRE's employment process, please email for general support and for intern positions. This service is for individuals requiring reasonable accommodation requests. Please note that vendor solicitations will not receive a reply.
+ Benefits information may be found here.
+ Copyright 1997\-2026, The MITRE Corporation. All rights reserved. MITRE is a registered trademark of The MITRE Corporation. Material on this site may be copied and distributed with permission only.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>